<commit_message>
feat: add Sheet 11 Formula Reference with all formulas, explanations, and references
Agent-Logs-Url: https://github.com/pramod51/medplus/sessions/8606954d-23f1-4e16-bfd7-affa7f482156

Co-authored-by: ydvashwani <47135442+ydvashwani@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/semiconductor_benchmarking.xlsx
+++ b/semiconductor_benchmarking.xlsx
@@ -17,6 +17,7 @@
     <sheet name="8 Business Model" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="9 Key Insights" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="10 Sources &amp; Assumptions" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="11 Formula Reference" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -26,7 +27,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="10">
+  <fonts count="17">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -77,8 +78,46 @@
       <color rgb="00FFFFFF"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Courier New"/>
+      <color rgb="001F3864"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00595959"/>
+      <sz val="9"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="00404040"/>
+      <sz val="9"/>
+    </font>
   </fonts>
-  <fills count="11">
+  <fills count="19">
     <fill>
       <patternFill/>
     </fill>
@@ -130,8 +169,48 @@
         <fgColor rgb="00BDD7EE"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F3864"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00F2F2F2"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00833C00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="007030A0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00156082"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00404040"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="7">
     <border>
       <left/>
       <right/>
@@ -153,11 +232,61 @@
         <color rgb="009E9E9E"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="009E9E9E"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="009E9E9E"/>
+      </right>
+      <top style="thin">
+        <color rgb="009E9E9E"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="009E9E9E"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="009E9E9E"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="009E9E9E"/>
+      </right>
+      <top style="thin">
+        <color rgb="009E9E9E"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="009E9E9E"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="42">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -236,6 +365,47 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="14" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="15" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="16" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="12" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1083,7 +1253,6 @@
         </is>
       </c>
     </row>
-    <row r="14"/>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
@@ -1496,7 +1665,6 @@
       </c>
       <c r="I26" s="5" t="inlineStr"/>
     </row>
-    <row r="27"/>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
         <is>
@@ -2455,9 +2623,7 @@
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" t="inlineStr"/>
-    </row>
+    <row r="14"/>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
@@ -2820,6 +2986,1337 @@
   <mergeCells count="2">
     <mergeCell ref="A15:E15"/>
     <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="48" customWidth="1" min="3" max="3"/>
+    <col width="36" customWidth="1" min="4" max="4"/>
+    <col width="30" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="6" max="6"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22" customHeight="1">
+      <c r="A1" s="29" t="inlineStr">
+        <is>
+          <t>STEP 11 — FORMULA REFERENCE  |  All formulas, explanations, and data source references</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="30" customHeight="1">
+      <c r="A2" s="30" t="inlineStr">
+        <is>
+          <t>#</t>
+        </is>
+      </c>
+      <c r="B2" s="30" t="inlineStr">
+        <is>
+          <t>Metric / Variable</t>
+        </is>
+      </c>
+      <c r="C2" s="30" t="inlineStr">
+        <is>
+          <t>Formula</t>
+        </is>
+      </c>
+      <c r="D2" s="30" t="inlineStr">
+        <is>
+          <t>Short Explanation</t>
+        </is>
+      </c>
+      <c r="E2" s="30" t="inlineStr">
+        <is>
+          <t>Source Sheet / Cells</t>
+        </is>
+      </c>
+      <c r="F2" s="30" t="inlineStr">
+        <is>
+          <t>Data Origin</t>
+        </is>
+      </c>
+      <c r="G2" s="30" t="inlineStr">
+        <is>
+          <t>Notes / Flags</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="31" t="inlineStr">
+        <is>
+          <t>A — AVERAGE BALANCE CALCULATIONS  (Sheet: 2 Average Balances)</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="42" customHeight="1">
+      <c r="A4" s="32" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="B4" s="32" t="inlineStr">
+        <is>
+          <t>Average Accounts Receivable (Avg AR)</t>
+        </is>
+      </c>
+      <c r="C4" s="33" t="inlineStr">
+        <is>
+          <t>Avg AR = (AR_CY + AR_PY) / 2</t>
+        </is>
+      </c>
+      <c r="D4" s="32" t="inlineStr">
+        <is>
+          <t>Simple two-period average smooths seasonality and point-in-time reporting differences.</t>
+        </is>
+      </c>
+      <c r="E4" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "2 Average Balances" col B
+AR data: Sheet "1 Raw Data" rows 29–39 cols B–C</t>
+        </is>
+      </c>
+      <c r="F4" s="32" t="inlineStr">
+        <is>
+          <t>Company 10-K / 20-F — Balance Sheet (Trade Receivables, net)</t>
+        </is>
+      </c>
+      <c r="G4" s="32" t="inlineStr">
+        <is>
+          <t>Use net AR (after allowance). TSMC values converted from TWD at annual avg FX.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="42" customHeight="1">
+      <c r="A5" s="32" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="B5" s="32" t="inlineStr">
+        <is>
+          <t>Average Inventory (Avg Inventory)</t>
+        </is>
+      </c>
+      <c r="C5" s="33" t="inlineStr">
+        <is>
+          <t>Avg Inv = (Inventory_CY + Inventory_PY) / 2</t>
+        </is>
+      </c>
+      <c r="D5" s="32" t="inlineStr">
+        <is>
+          <t>Averages opening and closing inventory to reduce distortion from period-end builds.</t>
+        </is>
+      </c>
+      <c r="E5" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "2 Average Balances" col C
+Inv data: Sheet "1 Raw Data" rows 29–39 cols D–E</t>
+        </is>
+      </c>
+      <c r="F5" s="32" t="inlineStr">
+        <is>
+          <t>Company 10-K / 20-F — Balance Sheet (Inventories)</t>
+        </is>
+      </c>
+      <c r="G5" s="32" t="inlineStr">
+        <is>
+          <t>⚠ TXN: strategic build. ⚠ Micron FY23: memory trough inflates avg.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="42" customHeight="1">
+      <c r="A6" s="32" t="inlineStr">
+        <is>
+          <t>A3</t>
+        </is>
+      </c>
+      <c r="B6" s="32" t="inlineStr">
+        <is>
+          <t>Average Accounts Payable (Avg AP)</t>
+        </is>
+      </c>
+      <c r="C6" s="33" t="inlineStr">
+        <is>
+          <t>Avg AP = (AP_CY + AP_PY) / 2</t>
+        </is>
+      </c>
+      <c r="D6" s="32" t="inlineStr">
+        <is>
+          <t>Two-period average of trade payables to align with the COGS denominator used in DPO.</t>
+        </is>
+      </c>
+      <c r="E6" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "2 Average Balances" col D
+AP data: Sheet "1 Raw Data" rows 29–39 cols F–G</t>
+        </is>
+      </c>
+      <c r="F6" s="32" t="inlineStr">
+        <is>
+          <t>Company 10-K / 20-F — Balance Sheet (Trade Payables / Accounts Payable)</t>
+        </is>
+      </c>
+      <c r="G6" s="32" t="inlineStr">
+        <is>
+          <t>Trade AP only; excludes accrued expenses and financing payables.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="42" customHeight="1">
+      <c r="A7" s="32" t="inlineStr">
+        <is>
+          <t>A4</t>
+        </is>
+      </c>
+      <c r="B7" s="32" t="inlineStr">
+        <is>
+          <t>Average COGS (Avg COGS)</t>
+        </is>
+      </c>
+      <c r="C7" s="33" t="inlineStr">
+        <is>
+          <t>Avg COGS = (COGS_CY + COGS_PY) / 2</t>
+        </is>
+      </c>
+      <c r="D7" s="32" t="inlineStr">
+        <is>
+          <t>Used as the denominator for DIO and DPO to neutralise single-year COGS anomalies.</t>
+        </is>
+      </c>
+      <c r="E7" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "2 Average Balances" col E
+COGS data: Sheet "1 Raw Data" rows 16–26 cols D–E</t>
+        </is>
+      </c>
+      <c r="F7" s="32" t="inlineStr">
+        <is>
+          <t>Company 10-K / 20-F — Income Statement (Cost of Revenue / Cost of Goods Sold)</t>
+        </is>
+      </c>
+      <c r="G7" s="32" t="inlineStr">
+        <is>
+          <t>Intel: COGS includes ~$5.2B impairment (not adjusted). Micron FY23 COGS &gt; Revenue (gross loss).</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="42" customHeight="1">
+      <c r="A8" s="32" t="inlineStr">
+        <is>
+          <t>A5</t>
+        </is>
+      </c>
+      <c r="B8" s="32" t="inlineStr">
+        <is>
+          <t>Average Revenue (Avg Revenue)</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="inlineStr">
+        <is>
+          <t>Avg Revenue = (Revenue_CY + Revenue_PY) / 2</t>
+        </is>
+      </c>
+      <c r="D8" s="32" t="inlineStr">
+        <is>
+          <t>Used as DSO denominator; smooths hyper-growth companies (NVIDIA +114% YoY).</t>
+        </is>
+      </c>
+      <c r="E8" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "2 Average Balances" col F
+Revenue data: Sheet "1 Raw Data" rows 16–26 cols B–C</t>
+        </is>
+      </c>
+      <c r="F8" s="32" t="inlineStr">
+        <is>
+          <t>Company 10-K / 20-F — Income Statement (Net Revenue / Net Sales)</t>
+        </is>
+      </c>
+      <c r="G8" s="32" t="inlineStr">
+        <is>
+          <t>TSMC: NT$ revenues converted at annual avg rate. Infineon: EUR converted at 1.085 USD/EUR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="A9" s="35" t="inlineStr">
+        <is>
+          <t>B — WORKING CAPITAL METRICS  (Sheet: 3 Metrics, cols B–G)</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="42" customHeight="1">
+      <c r="A10" s="32" t="inlineStr">
+        <is>
+          <t>B1</t>
+        </is>
+      </c>
+      <c r="B10" s="32" t="inlineStr">
+        <is>
+          <t>Working Capital (WC)</t>
+        </is>
+      </c>
+      <c r="C10" s="33" t="inlineStr">
+        <is>
+          <t>WC = Total Current Assets − Total Current Liabilities</t>
+        </is>
+      </c>
+      <c r="D10" s="32" t="inlineStr">
+        <is>
+          <t>Broadest liquidity measure; shows net short-term resources after all near-term obligations.</t>
+        </is>
+      </c>
+      <c r="E10" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "3 Metrics" col B
+CA/CL: Sheet "1 Raw Data" rows 40–51 cols B, E</t>
+        </is>
+      </c>
+      <c r="F10" s="32" t="inlineStr">
+        <is>
+          <t>10-K / 20-F Balance Sheet — Current Assets &amp; Current Liabilities totals</t>
+        </is>
+      </c>
+      <c r="G10" s="32" t="inlineStr">
+        <is>
+          <t>[A] CA and CL totals are approximated where not explicitly broken out.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="42" customHeight="1">
+      <c r="A11" s="32" t="inlineStr">
+        <is>
+          <t>B2</t>
+        </is>
+      </c>
+      <c r="B11" s="32" t="inlineStr">
+        <is>
+          <t>Balance Sheet NWC (BS NWC)</t>
+        </is>
+      </c>
+      <c r="C11" s="33" t="inlineStr">
+        <is>
+          <t>BS NWC = (Total CA − Cash &amp; ST Investments)
+         − (Total CL − ST Debt)</t>
+        </is>
+      </c>
+      <c r="D11" s="32" t="inlineStr">
+        <is>
+          <t>Strips financing items (cash, short-term debt) from WC to reveal the operating funding gap.</t>
+        </is>
+      </c>
+      <c r="E11" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "3 Metrics" col C
+Cash, ST Debt: Sheet "1 Raw Data" rows 40–51 cols C, G</t>
+        </is>
+      </c>
+      <c r="F11" s="32" t="inlineStr">
+        <is>
+          <t>10-K / 20-F Balance Sheet</t>
+        </is>
+      </c>
+      <c r="G11" s="32" t="inlineStr">
+        <is>
+          <t>[A] Cash &amp; ST Inv and ST Debt values approximated for several companies.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="42" customHeight="1">
+      <c r="A12" s="32" t="inlineStr">
+        <is>
+          <t>B3</t>
+        </is>
+      </c>
+      <c r="B12" s="32" t="inlineStr">
+        <is>
+          <t>Operating NWC (Op. NWC)</t>
+        </is>
+      </c>
+      <c r="C12" s="33" t="inlineStr">
+        <is>
+          <t>Op. NWC = Trade AR + Inventory − Trade AP</t>
+        </is>
+      </c>
+      <c r="D12" s="32" t="inlineStr">
+        <is>
+          <t>Isolates the cash tied up purely in the trade cycle — the most actionable metric.</t>
+        </is>
+      </c>
+      <c r="E12" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "3 Metrics" col D
+AR/Inv/AP: Sheet "1 Raw Data" rows 28–39</t>
+        </is>
+      </c>
+      <c r="F12" s="32" t="inlineStr">
+        <is>
+          <t>10-K / 20-F — AR (net), Inventories, Accounts Payable (CY values only)</t>
+        </is>
+      </c>
+      <c r="G12" s="32" t="inlineStr">
+        <is>
+          <t>Uses current-year balances only. Avg Op. NWC used in gap analysis (Sheet 6).</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="42" customHeight="1">
+      <c r="A13" s="32" t="inlineStr">
+        <is>
+          <t>B4</t>
+        </is>
+      </c>
+      <c r="B13" s="32" t="inlineStr">
+        <is>
+          <t>NWC as % of Revenue (NWC%)</t>
+        </is>
+      </c>
+      <c r="C13" s="33" t="inlineStr">
+        <is>
+          <t>NWC% = Op. NWC / Avg Revenue × 100</t>
+        </is>
+      </c>
+      <c r="D13" s="32" t="inlineStr">
+        <is>
+          <t>Revenue-normalised view; allows fair size-adjusted comparison across companies.</t>
+        </is>
+      </c>
+      <c r="E13" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "3 Metrics" col E
+Op. NWC: col D; Avg Revenue: Sheet "2 Avg Bal" col F</t>
+        </is>
+      </c>
+      <c r="F13" s="32" t="inlineStr">
+        <is>
+          <t>Derived — no direct filing source</t>
+        </is>
+      </c>
+      <c r="G13" s="32" t="inlineStr">
+        <is>
+          <t>Lower % = more capital-efficient. Qualcomm best (11.5%), Infineon worst (46.7%).</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="42" customHeight="1">
+      <c r="A14" s="32" t="inlineStr">
+        <is>
+          <t>B5</t>
+        </is>
+      </c>
+      <c r="B14" s="32" t="inlineStr">
+        <is>
+          <t>WC Intensity</t>
+        </is>
+      </c>
+      <c r="C14" s="33" t="inlineStr">
+        <is>
+          <t>WC Intensity = Op. NWC / Avg Revenue
+(decimal, not %)</t>
+        </is>
+      </c>
+      <c r="D14" s="32" t="inlineStr">
+        <is>
+          <t>Same as NWC% but expressed as a ratio. A value of 0.20 = $0.20 of WC per $1 of revenue.</t>
+        </is>
+      </c>
+      <c r="E14" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "3 Metrics" col F</t>
+        </is>
+      </c>
+      <c r="F14" s="32" t="inlineStr">
+        <is>
+          <t>Derived — no direct filing source</t>
+        </is>
+      </c>
+      <c r="G14" s="32" t="inlineStr">
+        <is>
+          <t>Equivalent to NWC% ÷ 100. Used in scoring model.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="42" customHeight="1">
+      <c r="A15" s="32" t="inlineStr">
+        <is>
+          <t>B6</t>
+        </is>
+      </c>
+      <c r="B15" s="32" t="inlineStr">
+        <is>
+          <t>Current Ratio</t>
+        </is>
+      </c>
+      <c r="C15" s="33" t="inlineStr">
+        <is>
+          <t>Current Ratio = Total CA / Total CL</t>
+        </is>
+      </c>
+      <c r="D15" s="32" t="inlineStr">
+        <is>
+          <t>Standard short-term solvency test. &gt;1 means current assets cover current liabilities.</t>
+        </is>
+      </c>
+      <c r="E15" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "3 Metrics" col G
+CA/CL: Sheet "1 Raw Data" rows 40–51</t>
+        </is>
+      </c>
+      <c r="F15" s="32" t="inlineStr">
+        <is>
+          <t>10-K / 20-F Balance Sheet</t>
+        </is>
+      </c>
+      <c r="G15" s="32" t="inlineStr">
+        <is>
+          <t>[A] Based on approximated CA/CL. A ratio of 1.5–3.0 is generally considered healthy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="A16" s="36" t="inlineStr">
+        <is>
+          <t>C — ACTIVITY / EFFICIENCY RATIOS  (Sheet: 3 Metrics, cols H–M)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="42" customHeight="1">
+      <c r="A17" s="32" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="B17" s="32" t="inlineStr">
+        <is>
+          <t>Days Sales Outstanding (DSO)</t>
+        </is>
+      </c>
+      <c r="C17" s="33" t="inlineStr">
+        <is>
+          <t>DSO = Avg AR / Avg Revenue × 365</t>
+        </is>
+      </c>
+      <c r="D17" s="32" t="inlineStr">
+        <is>
+          <t>Average number of days to collect cash after a sale. Lower = faster cash collection.</t>
+        </is>
+      </c>
+      <c r="E17" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "3 Metrics" col H
+Avg AR: Sheet "2" col B; Avg Revenue: Sheet "2" col F</t>
+        </is>
+      </c>
+      <c r="F17" s="32" t="inlineStr">
+        <is>
+          <t>Derived from 10-K / 20-F AR and Revenue figures</t>
+        </is>
+      </c>
+      <c r="G17" s="32" t="inlineStr">
+        <is>
+          <t>Best: Intel 35.5d (fast enterprise pay). Worst: Infineon 71.0d (auto OEM credit terms).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="42" customHeight="1">
+      <c r="A18" s="32" t="inlineStr">
+        <is>
+          <t>C2</t>
+        </is>
+      </c>
+      <c r="B18" s="32" t="inlineStr">
+        <is>
+          <t>Accounts Receivable Turnover (AR Turns)</t>
+        </is>
+      </c>
+      <c r="C18" s="33" t="inlineStr">
+        <is>
+          <t>AR Turns = Avg Revenue / Avg AR  (times per year)</t>
+        </is>
+      </c>
+      <c r="D18" s="32" t="inlineStr">
+        <is>
+          <t>How many times per year a company collects its entire AR balance. Higher = better.</t>
+        </is>
+      </c>
+      <c r="E18" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "3 Metrics" col I</t>
+        </is>
+      </c>
+      <c r="F18" s="32" t="inlineStr">
+        <is>
+          <t>Derived — no direct filing source</t>
+        </is>
+      </c>
+      <c r="G18" s="32" t="inlineStr">
+        <is>
+          <t>Mathematically inverse of DSO × 365. Used in ranking and scoring as a cross-check.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="42" customHeight="1">
+      <c r="A19" s="32" t="inlineStr">
+        <is>
+          <t>C3</t>
+        </is>
+      </c>
+      <c r="B19" s="32" t="inlineStr">
+        <is>
+          <t>Days Inventory Outstanding (DIO)</t>
+        </is>
+      </c>
+      <c r="C19" s="33" t="inlineStr">
+        <is>
+          <t>DIO = Avg Inventory / Avg COGS × 365</t>
+        </is>
+      </c>
+      <c r="D19" s="32" t="inlineStr">
+        <is>
+          <t>Average days inventory is held before sale. Lower = leaner supply chain.</t>
+        </is>
+      </c>
+      <c r="E19" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "3 Metrics" col J
+Avg Inv: Sheet "2" col C; Avg COGS: Sheet "2" col E</t>
+        </is>
+      </c>
+      <c r="F19" s="32" t="inlineStr">
+        <is>
+          <t>Derived from 10-K / 20-F Inventory and COGS figures</t>
+        </is>
+      </c>
+      <c r="G19" s="32" t="inlineStr">
+        <is>
+          <t>⚠ TXN 218.7d = strategic. ⚠ Infineon 243.7d = auto demand collapse. ⚠ Micron 165.4d = cycle.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="42" customHeight="1">
+      <c r="A20" s="32" t="inlineStr">
+        <is>
+          <t>C4</t>
+        </is>
+      </c>
+      <c r="B20" s="32" t="inlineStr">
+        <is>
+          <t>Days Payable Outstanding (DPO)</t>
+        </is>
+      </c>
+      <c r="C20" s="33" t="inlineStr">
+        <is>
+          <t>DPO = Avg AP / Avg COGS × 365</t>
+        </is>
+      </c>
+      <c r="D20" s="32" t="inlineStr">
+        <is>
+          <t>Average days taken to pay suppliers. Higher = better for the buyer (free credit period).</t>
+        </is>
+      </c>
+      <c r="E20" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "3 Metrics" col K
+Avg AP: Sheet "2" col D; Avg COGS: Sheet "2" col E</t>
+        </is>
+      </c>
+      <c r="F20" s="32" t="inlineStr">
+        <is>
+          <t>Derived from 10-K / 20-F AP and COGS figures</t>
+        </is>
+      </c>
+      <c r="G20" s="32" t="inlineStr">
+        <is>
+          <t>Best: Qualcomm 88.4d. Worst: TXN 22.4d (IDM own-fab model generates fewer trade payables).</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="42" customHeight="1">
+      <c r="A21" s="32" t="inlineStr">
+        <is>
+          <t>C5</t>
+        </is>
+      </c>
+      <c r="B21" s="32" t="inlineStr">
+        <is>
+          <t>Cash Conversion Cycle (CCC)</t>
+        </is>
+      </c>
+      <c r="C21" s="33" t="inlineStr">
+        <is>
+          <t>CCC = DSO + DIO − DPO  (days)</t>
+        </is>
+      </c>
+      <c r="D21" s="32" t="inlineStr">
+        <is>
+          <t>Days from paying suppliers to collecting cash from customers. Lower (or negative) = better.</t>
+        </is>
+      </c>
+      <c r="E21" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "3 Metrics" col L
+DSO col H, DIO col J, DPO col K</t>
+        </is>
+      </c>
+      <c r="F21" s="32" t="inlineStr">
+        <is>
+          <t>Derived — no direct filing source</t>
+        </is>
+      </c>
+      <c r="G21" s="32" t="inlineStr">
+        <is>
+          <t>Best: Qualcomm 22.1d. Worst: Infineon 240.5d. Negative CCC rare in semiconductors (see Sheet 8).</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="42" customHeight="1">
+      <c r="A22" s="32" t="inlineStr">
+        <is>
+          <t>C6</t>
+        </is>
+      </c>
+      <c r="B22" s="32" t="inlineStr">
+        <is>
+          <t>Cash Return Ratio (CRR)</t>
+        </is>
+      </c>
+      <c r="C22" s="33" t="inlineStr">
+        <is>
+          <t>CRR = OCF / Revenue_CY × 100  (%)</t>
+        </is>
+      </c>
+      <c r="D22" s="32" t="inlineStr">
+        <is>
+          <t>Fraction of each revenue dollar converted to operating cash. Captures D&amp;A and WC movements.</t>
+        </is>
+      </c>
+      <c r="E22" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "3 Metrics" col M
+OCF: Sheet "1 Raw Data" rows 40–51 col I; Revenue: col B rows 16–26</t>
+        </is>
+      </c>
+      <c r="F22" s="32" t="inlineStr">
+        <is>
+          <t>10-K / 20-F — Cash Flow Statement (Net Cash from Operating Activities)</t>
+        </is>
+      </c>
+      <c r="G22" s="32" t="inlineStr">
+        <is>
+          <t>Best: TSMC 62.2% (massive D&amp;A add-back). Worst: AMD 10.5% (R&amp;D investment). [A] TSMC OCF estimated.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="18" customHeight="1">
+      <c r="A23" s="37" t="inlineStr">
+        <is>
+          <t>D — CASH POTENTIAL GAP ANALYSIS  (Sheet: 6 Cash Potential)</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="42" customHeight="1">
+      <c r="A24" s="32" t="inlineStr">
+        <is>
+          <t>D1</t>
+        </is>
+      </c>
+      <c r="B24" s="32" t="inlineStr">
+        <is>
+          <t>DSO Lever (USD M)</t>
+        </is>
+      </c>
+      <c r="C24" s="33" t="inlineStr">
+        <is>
+          <t>DSO Lever = (DSO_company − DSO_best) × Avg Revenue / 365
+DSO_best = Intel 35.50 days</t>
+        </is>
+      </c>
+      <c r="D24" s="32" t="inlineStr">
+        <is>
+          <t>Cash unlocked if the company reduced DSO to the best-in-class peer level.</t>
+        </is>
+      </c>
+      <c r="E24" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "6 Cash Potential" col C–D
+DSO values: Sheet "3 Metrics" col H; Avg Revenue: Sheet "2" col F</t>
+        </is>
+      </c>
+      <c r="F24" s="32" t="inlineStr">
+        <is>
+          <t>Derived — no direct filing source</t>
+        </is>
+      </c>
+      <c r="G24" s="32" t="inlineStr">
+        <is>
+          <t>Only calculated for Q3 &amp; Q4 companies. DSO gap = company DSO − 35.50.</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="42" customHeight="1">
+      <c r="A25" s="32" t="inlineStr">
+        <is>
+          <t>D2</t>
+        </is>
+      </c>
+      <c r="B25" s="32" t="inlineStr">
+        <is>
+          <t>DIO Lever (USD M)</t>
+        </is>
+      </c>
+      <c r="C25" s="33" t="inlineStr">
+        <is>
+          <t>DIO Lever = (DIO_company − DIO_best) × Avg COGS / 365
+DIO_best = Qualcomm 54.28 days</t>
+        </is>
+      </c>
+      <c r="D25" s="32" t="inlineStr">
+        <is>
+          <t>Cash unlocked if the company reduced its inventory days to the best-in-class peer level.</t>
+        </is>
+      </c>
+      <c r="E25" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "6 Cash Potential" col E–F
+DIO values: Sheet "3 Metrics" col J; Avg COGS: Sheet "2" col E</t>
+        </is>
+      </c>
+      <c r="F25" s="32" t="inlineStr">
+        <is>
+          <t>Derived — no direct filing source</t>
+        </is>
+      </c>
+      <c r="G25" s="32" t="inlineStr">
+        <is>
+          <t>⚠ DIO improvements are subject to business-model constraints (IDM vs. fabless). See Sheet 8.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="42" customHeight="1">
+      <c r="A26" s="32" t="inlineStr">
+        <is>
+          <t>D3</t>
+        </is>
+      </c>
+      <c r="B26" s="32" t="inlineStr">
+        <is>
+          <t>DPO Lever (USD M)</t>
+        </is>
+      </c>
+      <c r="C26" s="33" t="inlineStr">
+        <is>
+          <t>DPO Lever = (DPO_best − DPO_company) × Avg COGS / 365
+DPO_best = Qualcomm 88.44 days</t>
+        </is>
+      </c>
+      <c r="D26" s="32" t="inlineStr">
+        <is>
+          <t>Additional supplier credit (free cash) available if DPO was extended to best-in-class.</t>
+        </is>
+      </c>
+      <c r="E26" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "6 Cash Potential" col G–H
+DPO values: Sheet "3 Metrics" col K; Avg COGS: Sheet "2" col E</t>
+        </is>
+      </c>
+      <c r="F26" s="32" t="inlineStr">
+        <is>
+          <t>Derived — no direct filing source</t>
+        </is>
+      </c>
+      <c r="G26" s="32" t="inlineStr">
+        <is>
+          <t>DPO extension requires supplier negotiation; subject to pricing-power constraints.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="42" customHeight="1">
+      <c r="A27" s="32" t="inlineStr">
+        <is>
+          <t>D4</t>
+        </is>
+      </c>
+      <c r="B27" s="32" t="inlineStr">
+        <is>
+          <t>Total Cash Potential (USD M)</t>
+        </is>
+      </c>
+      <c r="C27" s="33" t="inlineStr">
+        <is>
+          <t>Total = DSO Lever + DIO Lever + DPO Lever</t>
+        </is>
+      </c>
+      <c r="D27" s="32" t="inlineStr">
+        <is>
+          <t>Combined maximum cash release achievable by closing all three gaps simultaneously.</t>
+        </is>
+      </c>
+      <c r="E27" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "6 Cash Potential" col I</t>
+        </is>
+      </c>
+      <c r="F27" s="32" t="inlineStr">
+        <is>
+          <t>Derived — no direct filing source</t>
+        </is>
+      </c>
+      <c r="G27" s="32" t="inlineStr">
+        <is>
+          <t>Realistic release: 12–24 months. Micron DIO improvement is partially market-dependent.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="A28" s="38" t="inlineStr">
+        <is>
+          <t>E — SCORING MODEL  (Sheet: 5 Scoring Model)</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="42" customHeight="1">
+      <c r="A29" s="32" t="inlineStr">
+        <is>
+          <t>E1</t>
+        </is>
+      </c>
+      <c r="B29" s="32" t="inlineStr">
+        <is>
+          <t>Version A Score (Equal Weights)</t>
+        </is>
+      </c>
+      <c r="C29" s="33" t="inlineStr">
+        <is>
+          <t>V-A Score = (DSO_rank + AR_Turns_rank + CCC_rank
+             + CRR_rank + NWC%_rank) / 5
+Weight per metric = 20%</t>
+        </is>
+      </c>
+      <c r="D29" s="32" t="inlineStr">
+        <is>
+          <t>Simple average of 5 dimension ranks. Rank 1 = best in group. Lower score = better.</t>
+        </is>
+      </c>
+      <c r="E29" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "5 Scoring Model" col G
+Ranks: Sheet "4 Rankings" cols B–I</t>
+        </is>
+      </c>
+      <c r="F29" s="32" t="inlineStr">
+        <is>
+          <t>Derived — no direct filing source</t>
+        </is>
+      </c>
+      <c r="G29" s="32" t="inlineStr">
+        <is>
+          <t>Five metrics: DSO, AR Turns, CCC, CRR, NWC%. Equal 20% weight each.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="42" customHeight="1">
+      <c r="A30" s="32" t="inlineStr">
+        <is>
+          <t>E2</t>
+        </is>
+      </c>
+      <c r="B30" s="32" t="inlineStr">
+        <is>
+          <t>Version B Score (Sensitivity Weights)</t>
+        </is>
+      </c>
+      <c r="C30" s="33" t="inlineStr">
+        <is>
+          <t>V-B Score = CCC_rank × 0.30
+           + NWC%_rank × 0.25
+           + DSO_rank × 0.15
+           + AR_Turns_rank × 0.15
+           + CRR_rank × 0.15</t>
+        </is>
+      </c>
+      <c r="D30" s="32" t="inlineStr">
+        <is>
+          <t>Weighted scoring emphasising the cash cycle (CCC) and NWC efficiency as primary levers.</t>
+        </is>
+      </c>
+      <c r="E30" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "5 Scoring Model" col I
+Ranks: Sheet "4 Rankings"</t>
+        </is>
+      </c>
+      <c r="F30" s="32" t="inlineStr">
+        <is>
+          <t>Derived — no direct filing source</t>
+        </is>
+      </c>
+      <c r="G30" s="32" t="inlineStr">
+        <is>
+          <t>CCC and NWC% together = 55% of total score, reflecting their importance as strategic levers.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="42" customHeight="1">
+      <c r="A31" s="32" t="inlineStr">
+        <is>
+          <t>E3</t>
+        </is>
+      </c>
+      <c r="B31" s="32" t="inlineStr">
+        <is>
+          <t>Quartile Assignment</t>
+        </is>
+      </c>
+      <c r="C31" s="33" t="inlineStr">
+        <is>
+          <t>Q1: score 1.0–3.5  (Top performers)
+Q2: score 3.6–5.5
+Q3: score 5.6–7.5
+Q4: score 7.6–10.0  (Underperformers)</t>
+        </is>
+      </c>
+      <c r="D31" s="32" t="inlineStr">
+        <is>
+          <t>Groups companies into performance tiers for strategy and cash-potential analysis.</t>
+        </is>
+      </c>
+      <c r="E31" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "5 Scoring Model" col K</t>
+        </is>
+      </c>
+      <c r="F31" s="32" t="inlineStr">
+        <is>
+          <t>Derived — no direct filing source</t>
+        </is>
+      </c>
+      <c r="G31" s="32" t="inlineStr">
+        <is>
+          <t>Q3 &amp; Q4 companies are analysed further in Sheets 6 and 7 for cash release potential.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="18" customHeight="1">
+      <c r="A32" s="39" t="inlineStr">
+        <is>
+          <t>F — CURRENCY CONVERSION  (Sheet: 1 Raw Data, col H)</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="42" customHeight="1">
+      <c r="A33" s="32" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B33" s="32" t="inlineStr">
+        <is>
+          <t>TSMC: TWD → USD (FY2024)</t>
+        </is>
+      </c>
+      <c r="C33" s="33" t="inlineStr">
+        <is>
+          <t>USD value = TWD value ÷ 32.0</t>
+        </is>
+      </c>
+      <c r="D33" s="32" t="inlineStr">
+        <is>
+          <t>Converts TSMC financials from New Taiwan Dollar to USD using annual average FX rate.</t>
+        </is>
+      </c>
+      <c r="E33" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "1 Raw Data" cell H10
+Assumption A2: Sheet "10 Sources &amp; Assumptions" row 18</t>
+        </is>
+      </c>
+      <c r="F33" s="32" t="inlineStr">
+        <is>
+          <t>Annual average TWD/USD exchange rate for calendar year 2024 [Approximated]</t>
+        </is>
+      </c>
+      <c r="G33" s="32" t="inlineStr">
+        <is>
+          <t>⚠ [A] Verify vs. TSMC Form 20-F stated average translation rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="42" customHeight="1">
+      <c r="A34" s="32" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="B34" s="32" t="inlineStr">
+        <is>
+          <t>TSMC: TWD → USD (FY2023)</t>
+        </is>
+      </c>
+      <c r="C34" s="33" t="inlineStr">
+        <is>
+          <t>USD value = TWD value ÷ 31.1</t>
+        </is>
+      </c>
+      <c r="D34" s="32" t="inlineStr">
+        <is>
+          <t>Prior-year TSMC conversion for two-period average balance calculations.</t>
+        </is>
+      </c>
+      <c r="E34" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "1 Raw Data" cell H10
+Assumption A2: Sheet "10 Sources &amp; Assumptions" row 18</t>
+        </is>
+      </c>
+      <c r="F34" s="32" t="inlineStr">
+        <is>
+          <t>Annual average TWD/USD exchange rate for calendar year 2023 [Approximated]</t>
+        </is>
+      </c>
+      <c r="G34" s="32" t="inlineStr">
+        <is>
+          <t>⚠ [A] Verify vs. TSMC Form 20-F.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="42" customHeight="1">
+      <c r="A35" s="32" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="B35" s="32" t="inlineStr">
+        <is>
+          <t>Infineon: EUR → USD (FY2024)</t>
+        </is>
+      </c>
+      <c r="C35" s="33" t="inlineStr">
+        <is>
+          <t>USD value = EUR value × 1.085</t>
+        </is>
+      </c>
+      <c r="D35" s="32" t="inlineStr">
+        <is>
+          <t>Converts Infineon financials from Euro to USD. Infineon FY runs Oct 2023 – Sep 2024.</t>
+        </is>
+      </c>
+      <c r="E35" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "1 Raw Data" cell H13
+Assumption A3: Sheet "10 Sources &amp; Assumptions" row 19</t>
+        </is>
+      </c>
+      <c r="F35" s="32" t="inlineStr">
+        <is>
+          <t>Annual average EUR/USD exchange rate for Oct 2023 – Sep 2024 period [Approximated]</t>
+        </is>
+      </c>
+      <c r="G35" s="32" t="inlineStr">
+        <is>
+          <t>⚠ [A] Verify vs. Infineon Annual Report 2024 stated average rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="42" customHeight="1">
+      <c r="A36" s="32" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="B36" s="32" t="inlineStr">
+        <is>
+          <t>Infineon: EUR → USD (FY2023)</t>
+        </is>
+      </c>
+      <c r="C36" s="33" t="inlineStr">
+        <is>
+          <t>USD value = EUR value × 1.082</t>
+        </is>
+      </c>
+      <c r="D36" s="32" t="inlineStr">
+        <is>
+          <t>Prior-year Infineon conversion for two-period averages.</t>
+        </is>
+      </c>
+      <c r="E36" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "1 Raw Data" cell H13
+Assumption A3: Sheet "10 Sources &amp; Assumptions" row 19</t>
+        </is>
+      </c>
+      <c r="F36" s="32" t="inlineStr">
+        <is>
+          <t>Annual average EUR/USD exchange rate for Oct 2022 – Sep 2023 period [Approximated]</t>
+        </is>
+      </c>
+      <c r="G36" s="32" t="inlineStr">
+        <is>
+          <t>⚠ [A] Verify vs. Infineon Annual Report 2023.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="18" customHeight="1">
+      <c r="A37" s="40" t="inlineStr">
+        <is>
+          <t>G — DERIVED / RECONSTRUCTED INPUTS  (Sheet: 1 Raw Data, col H)</t>
+        </is>
+      </c>
+    </row>
+    <row r="38" ht="42" customHeight="1">
+      <c r="A38" s="32" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="B38" s="32" t="inlineStr">
+        <is>
+          <t>COGS (where not directly stated)</t>
+        </is>
+      </c>
+      <c r="C38" s="33" t="inlineStr">
+        <is>
+          <t>COGS = Revenue − Gross Profit</t>
+        </is>
+      </c>
+      <c r="D38" s="32" t="inlineStr">
+        <is>
+          <t>Standard accounting identity. Used when COGS line is not separately disclosed on the P&amp;L.</t>
+        </is>
+      </c>
+      <c r="E38" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "1 Raw Data" col H (COGS Method)
+Assumption A4: Sheet "10" row 20</t>
+        </is>
+      </c>
+      <c r="F38" s="32" t="inlineStr">
+        <is>
+          <t>Company 10-K — Income Statement (Revenue and Gross Profit are always disclosed)</t>
+        </is>
+      </c>
+      <c r="G38" s="32" t="inlineStr">
+        <is>
+          <t>Applied to: Intel (FY2024) and Micron (FY2023/FY2024). Result cross-checked against disclosed COGS where available.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39" ht="42" customHeight="1">
+      <c r="A39" s="32" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="B39" s="32" t="inlineStr">
+        <is>
+          <t>Gross Margin (verification)</t>
+        </is>
+      </c>
+      <c r="C39" s="33" t="inlineStr">
+        <is>
+          <t>Gross Margin % = Gross Profit / Revenue × 100
+= (Revenue − COGS) / Revenue × 100</t>
+        </is>
+      </c>
+      <c r="D39" s="32" t="inlineStr">
+        <is>
+          <t>Used to verify COGS figures against disclosed gross margin percentages in filings.</t>
+        </is>
+      </c>
+      <c r="E39" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "1 Raw Data" cols F–G</t>
+        </is>
+      </c>
+      <c r="F39" s="32" t="inlineStr">
+        <is>
+          <t>10-K / 20-F Income Statement</t>
+        </is>
+      </c>
+      <c r="G39" s="32" t="inlineStr">
+        <is>
+          <t>⚠ Intel FY2024 gross margin of 32.7% reflects $5.2B impairment in COGS (Assumption A5). ⚠ Micron FY2023 gross margin = −12.3% (gross loss).</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="42" customHeight="1">
+      <c r="A40" s="32" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="B40" s="32" t="inlineStr">
+        <is>
+          <t>TSMC OCF Estimate</t>
+        </is>
+      </c>
+      <c r="C40" s="33" t="inlineStr">
+        <is>
+          <t>OCF (USD M) = OCF (NT$B) × 1,000 / FX rate
+OCF ≈ NT$1,800B × 1,000 / 32.0 = $56,250M</t>
+        </is>
+      </c>
+      <c r="D40" s="32" t="inlineStr">
+        <is>
+          <t>TSMC operating cash flow converted from NT$ to USD using annual average FX rate.</t>
+        </is>
+      </c>
+      <c r="E40" s="34" t="inlineStr">
+        <is>
+          <t>Sheet "1 Raw Data" row 48 col I
+Assumption A9: Sheet "10" row 25</t>
+        </is>
+      </c>
+      <c r="F40" s="32" t="inlineStr">
+        <is>
+          <t>TSMC Form 20-F — Cash Flow Statement (NT$ figures) [Approximated]</t>
+        </is>
+      </c>
+      <c r="G40" s="32" t="inlineStr">
+        <is>
+          <t>⚠ [A] Estimate based on NT$ filing. Verify exact USD figure vs. TSMC 20-F cash flow statement.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42" ht="30" customHeight="1">
+      <c r="A42" s="41" t="inlineStr">
+        <is>
+          <t>KEY DEFINITIONS  |  AR = Accounts Receivable (net)  |  AP = Accounts Payable (trade)  |  COGS = Cost of Goods Sold / Cost of Revenue  |  OCF = Net Cash from Operations  |  CY = Current Year  |  PY = Prior Year  |  [A] = Approximated value</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="30" customHeight="1">
+      <c r="A43" s="41" t="inlineStr">
+        <is>
+          <t>PRIMARY DATA SOURCES  |  All raw financial data sourced from official SEC filings: 10-K (US companies) and 20-F (non-US: TSMC, NXP, STM) via SEC EDGAR.  See Sheet "10 Sources &amp; Assumptions" for full filing details, CIK numbers, and assumption log.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="10">
+    <mergeCell ref="A32:G32"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="A3:G3"/>
+    <mergeCell ref="A37:G37"/>
+    <mergeCell ref="A16:G16"/>
+    <mergeCell ref="A42:G42"/>
+    <mergeCell ref="A43:G43"/>
+    <mergeCell ref="A28:G28"/>
+    <mergeCell ref="A23:G23"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5232,7 +6729,6 @@
         <v>3564</v>
       </c>
     </row>
-    <row r="9"/>
     <row r="10">
       <c r="A10" s="18" t="inlineStr">
         <is>
@@ -5543,6 +7039,9 @@
           <t>8.1 — Fabless vs. Foundry vs. IDM</t>
         </is>
       </c>
+      <c r="B2" s="27" t="n"/>
+      <c r="C2" s="27" t="n"/>
+      <c r="D2" s="28" t="n"/>
     </row>
     <row r="3" ht="18" customHeight="1">
       <c r="A3" s="24" t="inlineStr">
@@ -5550,6 +7049,9 @@
           <t>Fabless (NVIDIA, AMD, Qualcomm)</t>
         </is>
       </c>
+      <c r="B3" s="27" t="n"/>
+      <c r="C3" s="27" t="n"/>
+      <c r="D3" s="28" t="n"/>
     </row>
     <row r="4" ht="18" customHeight="1">
       <c r="A4" s="19" t="inlineStr">
@@ -5557,6 +7059,9 @@
           <t>• No manufacturing assets. Production outsourced to TSMC/Samsung/GlobalFoundries.</t>
         </is>
       </c>
+      <c r="B4" s="27" t="n"/>
+      <c r="C4" s="27" t="n"/>
+      <c r="D4" s="28" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="A5" s="19" t="inlineStr">
@@ -5564,6 +7069,9 @@
           <t>• Inventory = finished goods only (at 3PL). No raw materials or WIP at own facilities.</t>
         </is>
       </c>
+      <c r="B5" s="27" t="n"/>
+      <c r="C5" s="27" t="n"/>
+      <c r="D5" s="28" t="n"/>
     </row>
     <row r="6" ht="18" customHeight="1">
       <c r="A6" s="19" t="inlineStr">
@@ -5571,6 +7079,9 @@
           <t>• DIO range: 54–77 days — lowest in peer group.</t>
         </is>
       </c>
+      <c r="B6" s="27" t="n"/>
+      <c r="C6" s="27" t="n"/>
+      <c r="D6" s="28" t="n"/>
     </row>
     <row r="7" ht="18" customHeight="1">
       <c r="A7" s="19" t="inlineStr">
@@ -5578,6 +7089,9 @@
           <t>• DPO constrained by TSMC pricing power; Qualcomm (88d DPO) is best achievable at scale.</t>
         </is>
       </c>
+      <c r="B7" s="27" t="n"/>
+      <c r="C7" s="27" t="n"/>
+      <c r="D7" s="28" t="n"/>
     </row>
     <row r="8" ht="18" customHeight="1">
       <c r="A8" s="19" t="inlineStr">
@@ -5585,6 +7099,9 @@
           <t>• CCC structurally 80–160 days lower than IDMs due to absence of manufacturing WIP.</t>
         </is>
       </c>
+      <c r="B8" s="27" t="n"/>
+      <c r="C8" s="27" t="n"/>
+      <c r="D8" s="28" t="n"/>
     </row>
     <row r="9" ht="18" customHeight="1">
       <c r="A9" s="24" t="inlineStr">
@@ -5592,6 +7109,9 @@
           <t>Foundry (TSMC)</t>
         </is>
       </c>
+      <c r="B9" s="27" t="n"/>
+      <c r="C9" s="27" t="n"/>
+      <c r="D9" s="28" t="n"/>
     </row>
     <row r="10" ht="18" customHeight="1">
       <c r="A10" s="19" t="inlineStr">
@@ -5599,6 +7119,9 @@
           <t>• Pure contract manufacturer. Inventory = entirely WIP (8–12 week fab cycle on N3/N5/N7).</t>
         </is>
       </c>
+      <c r="B10" s="27" t="n"/>
+      <c r="C10" s="27" t="n"/>
+      <c r="D10" s="28" t="n"/>
     </row>
     <row r="11" ht="18" customHeight="1">
       <c r="A11" s="19" t="inlineStr">
@@ -5606,6 +7129,9 @@
           <t>• DIO 137 days reflects physical wafer processing time — structurally unavoidable.</t>
         </is>
       </c>
+      <c r="B11" s="27" t="n"/>
+      <c r="C11" s="27" t="n"/>
+      <c r="D11" s="28" t="n"/>
     </row>
     <row r="12" ht="18" customHeight="1">
       <c r="A12" s="19" t="inlineStr">
@@ -5613,6 +7139,9 @@
           <t>• OCF/Revenue = 62% (CRR best in group) driven by $20–25B annual D&amp;A add-back + pricing power.</t>
         </is>
       </c>
+      <c r="B12" s="27" t="n"/>
+      <c r="C12" s="27" t="n"/>
+      <c r="D12" s="28" t="n"/>
     </row>
     <row r="13" ht="18" customHeight="1">
       <c r="A13" s="24" t="inlineStr">
@@ -5620,6 +7149,9 @@
           <t>IDMs (Intel, Micron, Infineon, STM, TXN, NXP)</t>
         </is>
       </c>
+      <c r="B13" s="27" t="n"/>
+      <c r="C13" s="27" t="n"/>
+      <c r="D13" s="28" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1">
       <c r="A14" s="19" t="inlineStr">
@@ -5627,6 +7159,9 @@
           <t>• Full vertical integration: raw materials → WIP (weeks/months in fab) → finished goods.</t>
         </is>
       </c>
+      <c r="B14" s="27" t="n"/>
+      <c r="C14" s="27" t="n"/>
+      <c r="D14" s="28" t="n"/>
     </row>
     <row r="15" ht="18" customHeight="1">
       <c r="A15" s="19" t="inlineStr">
@@ -5634,6 +7169,9 @@
           <t>• DIO ranges 120–244 days — 2–4× higher than fabless peers. Structural, not operational.</t>
         </is>
       </c>
+      <c r="B15" s="27" t="n"/>
+      <c r="C15" s="27" t="n"/>
+      <c r="D15" s="28" t="n"/>
     </row>
     <row r="16" ht="18" customHeight="1">
       <c r="A16" s="19" t="inlineStr">
@@ -5641,6 +7179,9 @@
           <t>• Best IDM: NXP (DIO 120d, CCC 100d) — lean footprint, strong DPO, diversified customers.</t>
         </is>
       </c>
+      <c r="B16" s="27" t="n"/>
+      <c r="C16" s="27" t="n"/>
+      <c r="D16" s="28" t="n"/>
     </row>
     <row r="17" ht="25" customHeight="1">
       <c r="A17" s="23" t="inlineStr">
@@ -5648,6 +7189,9 @@
           <t>8.2 — Outsourced vs. In-House Manufacturing</t>
         </is>
       </c>
+      <c r="B17" s="27" t="n"/>
+      <c r="C17" s="27" t="n"/>
+      <c r="D17" s="28" t="n"/>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="24" t="inlineStr">
@@ -5655,6 +7199,9 @@
           <t>Fab Model</t>
         </is>
       </c>
+      <c r="B18" s="27" t="n"/>
+      <c r="C18" s="27" t="n"/>
+      <c r="D18" s="28" t="n"/>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="19" t="inlineStr">
@@ -5662,6 +7209,9 @@
           <t>Pure fabless</t>
         </is>
       </c>
+      <c r="B19" s="27" t="n"/>
+      <c r="C19" s="27" t="n"/>
+      <c r="D19" s="28" t="n"/>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="19" t="inlineStr">
@@ -5669,6 +7219,9 @@
           <t>Asset-light IDM (NXP)</t>
         </is>
       </c>
+      <c r="B20" s="27" t="n"/>
+      <c r="C20" s="27" t="n"/>
+      <c r="D20" s="28" t="n"/>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="19" t="inlineStr">
@@ -5676,6 +7229,9 @@
           <t>Full IDM – mature node</t>
         </is>
       </c>
+      <c r="B21" s="27" t="n"/>
+      <c r="C21" s="27" t="n"/>
+      <c r="D21" s="28" t="n"/>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="19" t="inlineStr">
@@ -5683,6 +7239,9 @@
           <t>Full IDM – advanced/memory</t>
         </is>
       </c>
+      <c r="B22" s="27" t="n"/>
+      <c r="C22" s="27" t="n"/>
+      <c r="D22" s="28" t="n"/>
     </row>
     <row r="23" ht="18" customHeight="1">
       <c r="A23" s="19" t="inlineStr">
@@ -5690,6 +7249,9 @@
           <t>Pure foundry</t>
         </is>
       </c>
+      <c r="B23" s="27" t="n"/>
+      <c r="C23" s="27" t="n"/>
+      <c r="D23" s="28" t="n"/>
     </row>
     <row r="24" ht="25" customHeight="1">
       <c r="A24" s="23" t="inlineStr">
@@ -5697,6 +7259,9 @@
           <t>8.3 — Memory Cyclicality (Micron)</t>
         </is>
       </c>
+      <c r="B24" s="27" t="n"/>
+      <c r="C24" s="27" t="n"/>
+      <c r="D24" s="28" t="n"/>
     </row>
     <row r="25" ht="18" customHeight="1">
       <c r="A25" s="19" t="inlineStr">
@@ -5704,6 +7269,9 @@
           <t>• DRAM/NAND prices fell 50–80% in 2022–2023 trough. Micron FY2023 gross profit = −$1,906M.</t>
         </is>
       </c>
+      <c r="B25" s="27" t="n"/>
+      <c r="C25" s="27" t="n"/>
+      <c r="D25" s="28" t="n"/>
     </row>
     <row r="26" ht="18" customHeight="1">
       <c r="A26" s="19" t="inlineStr">
@@ -5711,6 +7279,9 @@
           <t>• DIO inflated by underabsorption (fixed fab costs / fewer units) + price deflation.</t>
         </is>
       </c>
+      <c r="B26" s="27" t="n"/>
+      <c r="C26" s="27" t="n"/>
+      <c r="D26" s="28" t="n"/>
     </row>
     <row r="27" ht="18" customHeight="1">
       <c r="A27" s="19" t="inlineStr">
@@ -5718,6 +7289,9 @@
           <t>• Point-in-time DIO for Micron is unreliable; evaluate over a full 3–5 year DRAM price cycle.</t>
         </is>
       </c>
+      <c r="B27" s="27" t="n"/>
+      <c r="C27" s="27" t="n"/>
+      <c r="D27" s="28" t="n"/>
     </row>
     <row r="28" ht="18" customHeight="1">
       <c r="A28" s="19" t="inlineStr">
@@ -5725,6 +7299,9 @@
           <t>• Avg COGS = $18,443M (blending trough FY23 + recovery FY24) — partially normalises distortion.</t>
         </is>
       </c>
+      <c r="B28" s="27" t="n"/>
+      <c r="C28" s="27" t="n"/>
+      <c r="D28" s="28" t="n"/>
     </row>
     <row r="29" ht="25" customHeight="1">
       <c r="A29" s="23" t="inlineStr">
@@ -5732,6 +7309,9 @@
           <t>8.4 — Why Negative CCC is Rare in Semiconductors</t>
         </is>
       </c>
+      <c r="B29" s="27" t="n"/>
+      <c r="C29" s="27" t="n"/>
+      <c r="D29" s="28" t="n"/>
     </row>
     <row r="30" ht="18" customHeight="1">
       <c r="A30" s="19" t="inlineStr">
@@ -5739,6 +7319,9 @@
           <t>• Negative CCC requires DPO &gt; DSO + DIO. Classic example: Dell (1990s), Amazon retail.</t>
         </is>
       </c>
+      <c r="B30" s="27" t="n"/>
+      <c r="C30" s="27" t="n"/>
+      <c r="D30" s="28" t="n"/>
     </row>
     <row r="31" ht="18" customHeight="1">
       <c r="A31" s="19" t="inlineStr">
@@ -5746,6 +7329,9 @@
           <t>• Even Qualcomm (CCC = 22.11d — group best) cannot reach negative CCC because:</t>
         </is>
       </c>
+      <c r="B31" s="27" t="n"/>
+      <c r="C31" s="27" t="n"/>
+      <c r="D31" s="28" t="n"/>
     </row>
     <row r="32" ht="18" customHeight="1">
       <c r="A32" s="19" t="inlineStr">
@@ -5753,6 +7339,9 @@
           <t xml:space="preserve">  (a) Safety stock inventory required for service levels (automotive safety, HPC spikes).</t>
         </is>
       </c>
+      <c r="B32" s="27" t="n"/>
+      <c r="C32" s="27" t="n"/>
+      <c r="D32" s="28" t="n"/>
     </row>
     <row r="33" ht="18" customHeight="1">
       <c r="A33" s="19" t="inlineStr">
@@ -5760,6 +7349,9 @@
           <t xml:space="preserve">  (b) TSMC/OSAT suppliers have pricing power — DPO cannot be pushed above 90+ days.</t>
         </is>
       </c>
+      <c r="B33" s="27" t="n"/>
+      <c r="C33" s="27" t="n"/>
+      <c r="D33" s="28" t="n"/>
     </row>
     <row r="34" ht="18" customHeight="1">
       <c r="A34" s="19" t="inlineStr">
@@ -5767,6 +7359,9 @@
           <t xml:space="preserve">  (c) Enterprise/OEM customers pay in 30–60 days (not instantly like consumers).</t>
         </is>
       </c>
+      <c r="B34" s="27" t="n"/>
+      <c r="C34" s="27" t="n"/>
+      <c r="D34" s="28" t="n"/>
     </row>
     <row r="35" ht="18" customHeight="1">
       <c r="A35" s="19" t="inlineStr">
@@ -5774,6 +7369,9 @@
           <t>• A negative CCC signals dominant market power that lets a company finance itself from supply chain.</t>
         </is>
       </c>
+      <c r="B35" s="27" t="n"/>
+      <c r="C35" s="27" t="n"/>
+      <c r="D35" s="28" t="n"/>
     </row>
     <row r="36" ht="25" customHeight="1">
       <c r="A36" s="23" t="inlineStr">
@@ -5781,6 +7379,9 @@
           <t>8.5 — US GAAP vs. IFRS Comparability</t>
         </is>
       </c>
+      <c r="B36" s="27" t="n"/>
+      <c r="C36" s="27" t="n"/>
+      <c r="D36" s="28" t="n"/>
     </row>
     <row r="37" ht="18" customHeight="1">
       <c r="A37" s="19" t="inlineStr">
@@ -5788,6 +7389,9 @@
           <t>T</t>
         </is>
       </c>
+      <c r="B37" s="27" t="n"/>
+      <c r="C37" s="27" t="n"/>
+      <c r="D37" s="28" t="n"/>
     </row>
     <row r="38" ht="18" customHeight="1">
       <c r="A38" s="19" t="inlineStr">
@@ -5795,6 +7399,9 @@
           <t>I</t>
         </is>
       </c>
+      <c r="B38" s="27" t="n"/>
+      <c r="C38" s="27" t="n"/>
+      <c r="D38" s="28" t="n"/>
     </row>
     <row r="39" ht="18" customHeight="1">
       <c r="A39" s="19" t="inlineStr">
@@ -5802,6 +7409,9 @@
           <t>I</t>
         </is>
       </c>
+      <c r="B39" s="27" t="n"/>
+      <c r="C39" s="27" t="n"/>
+      <c r="D39" s="28" t="n"/>
     </row>
     <row r="40" ht="18" customHeight="1">
       <c r="A40" s="19" t="inlineStr">
@@ -5809,6 +7419,9 @@
           <t>R</t>
         </is>
       </c>
+      <c r="B40" s="27" t="n"/>
+      <c r="C40" s="27" t="n"/>
+      <c r="D40" s="28" t="n"/>
     </row>
     <row r="41" ht="18" customHeight="1">
       <c r="A41" s="19" t="inlineStr">
@@ -5816,6 +7429,9 @@
           <t>R</t>
         </is>
       </c>
+      <c r="B41" s="27" t="n"/>
+      <c r="C41" s="27" t="n"/>
+      <c r="D41" s="28" t="n"/>
     </row>
     <row r="42" ht="18" customHeight="1">
       <c r="A42" s="19" t="inlineStr">
@@ -5823,6 +7439,9 @@
           <t>Overall GAAP/IFRS verdict: Not material for this analysis. Trade working capital items treated similarly under both standards.</t>
         </is>
       </c>
+      <c r="B42" s="27" t="n"/>
+      <c r="C42" s="27" t="n"/>
+      <c r="D42" s="28" t="n"/>
     </row>
     <row r="43" ht="25" customHeight="1">
       <c r="A43" s="23" t="inlineStr">
@@ -5830,6 +7449,9 @@
           <t>8.6 — Fiscal Year-End Differences</t>
         </is>
       </c>
+      <c r="B43" s="27" t="n"/>
+      <c r="C43" s="27" t="n"/>
+      <c r="D43" s="28" t="n"/>
     </row>
     <row r="44" ht="18" customHeight="1">
       <c r="A44" s="19" t="inlineStr">
@@ -5837,6 +7459,9 @@
           <t>C</t>
         </is>
       </c>
+      <c r="B44" s="27" t="n"/>
+      <c r="C44" s="27" t="n"/>
+      <c r="D44" s="28" t="n"/>
     </row>
     <row r="45" ht="18" customHeight="1">
       <c r="A45" s="19" t="inlineStr">
@@ -5844,6 +7469,9 @@
           <t>N</t>
         </is>
       </c>
+      <c r="B45" s="27" t="n"/>
+      <c r="C45" s="27" t="n"/>
+      <c r="D45" s="28" t="n"/>
     </row>
     <row r="46" ht="18" customHeight="1">
       <c r="A46" s="19" t="inlineStr">
@@ -5851,6 +7479,9 @@
           <t>Q</t>
         </is>
       </c>
+      <c r="B46" s="27" t="n"/>
+      <c r="C46" s="27" t="n"/>
+      <c r="D46" s="28" t="n"/>
     </row>
     <row r="47" ht="18" customHeight="1">
       <c r="A47" s="19" t="inlineStr">
@@ -5858,6 +7489,9 @@
           <t>I</t>
         </is>
       </c>
+      <c r="B47" s="27" t="n"/>
+      <c r="C47" s="27" t="n"/>
+      <c r="D47" s="28" t="n"/>
     </row>
     <row r="48" ht="18" customHeight="1">
       <c r="A48" s="19" t="inlineStr">
@@ -5865,6 +7499,9 @@
           <t>M</t>
         </is>
       </c>
+      <c r="B48" s="27" t="n"/>
+      <c r="C48" s="27" t="n"/>
+      <c r="D48" s="28" t="n"/>
     </row>
     <row r="49" ht="25" customHeight="1">
       <c r="A49" s="23" t="inlineStr">
@@ -5872,6 +7509,9 @@
           <t>8.7 — Overall Verdict: Is This a Fair Peer Group?</t>
         </is>
       </c>
+      <c r="B49" s="27" t="n"/>
+      <c r="C49" s="27" t="n"/>
+      <c r="D49" s="28" t="n"/>
     </row>
     <row r="50" ht="18" customHeight="1">
       <c r="A50" s="19" t="inlineStr">
@@ -5879,6 +7519,9 @@
           <t>Partially fair. Key limitations:</t>
         </is>
       </c>
+      <c r="B50" s="27" t="n"/>
+      <c r="C50" s="27" t="n"/>
+      <c r="D50" s="28" t="n"/>
     </row>
     <row r="51" ht="18" customHeight="1">
       <c r="A51" s="19" t="inlineStr">
@@ -5886,6 +7529,9 @@
           <t>1. Business model heterogeneity: Fabless vs. IDM DIO gap is a model artefact, not management performance.</t>
         </is>
       </c>
+      <c r="B51" s="27" t="n"/>
+      <c r="C51" s="27" t="n"/>
+      <c r="D51" s="28" t="n"/>
     </row>
     <row r="52" ht="18" customHeight="1">
       <c r="A52" s="19" t="inlineStr">
@@ -5893,6 +7539,9 @@
           <t>2. Revenue scale differences: NVIDIA 114% YoY growth compresses DSO/AR Turns mechanically.</t>
         </is>
       </c>
+      <c r="B52" s="27" t="n"/>
+      <c r="C52" s="27" t="n"/>
+      <c r="D52" s="28" t="n"/>
     </row>
     <row r="53" ht="18" customHeight="1">
       <c r="A53" s="19" t="inlineStr">
@@ -5900,6 +7549,9 @@
           <t>3. Cycle position mismatch: NVIDIA/TSMC in AI upswing vs. Intel/STM/Infineon/TXN in downcycle.</t>
         </is>
       </c>
+      <c r="B53" s="27" t="n"/>
+      <c r="C53" s="27" t="n"/>
+      <c r="D53" s="28" t="n"/>
     </row>
     <row r="54" ht="18" customHeight="1">
       <c r="A54" s="19" t="inlineStr">
@@ -5907,6 +7559,9 @@
           <t>4. Currency translation noise: TSMC (TWD) and Infineon (EUR) add FX approximation error.</t>
         </is>
       </c>
+      <c r="B54" s="27" t="n"/>
+      <c r="C54" s="27" t="n"/>
+      <c r="D54" s="28" t="n"/>
     </row>
     <row r="55" ht="18" customHeight="1">
       <c r="A55" s="19" t="inlineStr">
@@ -5914,6 +7569,9 @@
           <t>5. Despite limitations, the group is academically valid: same end-markets, customers, input costs, full model spectrum.</t>
         </is>
       </c>
+      <c r="B55" s="27" t="n"/>
+      <c r="C55" s="27" t="n"/>
+      <c r="D55" s="28" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="55">

</xml_diff>

<commit_message>
feat: replace all hardcoded computed values with live Excel formulas across Sheets 2-6 and 9, add URL references in Sheet 12
Agent-Logs-Url: https://github.com/pramod51/medplus/sessions/642b021b-872b-4d41-99b8-b3b3c9c9ef58

Co-authored-by: ydvashwani <47135442+ydvashwani@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/semiconductor_benchmarking.xlsx
+++ b/semiconductor_benchmarking.xlsx
@@ -21,7 +21,7 @@
     <sheet name="12 URL References" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="124519" calcMode="auto" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -3098,7 +3098,8 @@
     <row r="1" ht="22" customHeight="1">
       <c r="A1" s="29" t="inlineStr">
         <is>
-          <t>STEP 11 — FORMULA REFERENCE  |  All formulas, explanations, and data source references</t>
+          <t>STEP 11 — FORMULA REFERENCE  |  All formulas, explanations, and data source references
+⚡ NOTE: As of this version all calculated cells in Sheets 2–6 and 9 use live Excel formulas linked to Sheet 1 raw data — no hardcoded computed values. Select any cell in those sheets to see and audit the formula in the formula bar.</t>
         </is>
       </c>
     </row>
@@ -3471,7 +3472,7 @@
       </c>
       <c r="C13" s="33" t="inlineStr">
         <is>
-          <t>NWC% = Op. NWC / Avg Revenue × 100</t>
+          <t>NWC% = Op. NWC / Revenue_CY × 100</t>
         </is>
       </c>
       <c r="D13" s="32" t="inlineStr">
@@ -3482,7 +3483,7 @@
       <c r="E13" s="34" t="inlineStr">
         <is>
           <t>Sheet "3 Metrics" col E
-Op. NWC: col D; Avg Revenue: Sheet "2 Avg Bal" col F</t>
+Op. NWC: col D same row; Revenue CY: Sheet "1 Raw Data" col B rows 17–26</t>
         </is>
       </c>
       <c r="F13" s="32" t="inlineStr">
@@ -3509,8 +3510,9 @@
       </c>
       <c r="C14" s="33" t="inlineStr">
         <is>
-          <t>WC Intensity = Op. NWC / Avg Revenue
-(decimal, not %)</t>
+          <t>WC Intensity = WC / Revenue_CY
+(decimal, not %)
+where WC = Total CA − Total CL</t>
         </is>
       </c>
       <c r="D14" s="32" t="inlineStr">
@@ -3520,7 +3522,8 @@
       </c>
       <c r="E14" s="34" t="inlineStr">
         <is>
-          <t>Sheet "3 Metrics" col F</t>
+          <t>Sheet "3 Metrics" col F
+WC: col B same row; Revenue CY: Sheet "1 Raw Data" col B rows 17–26</t>
         </is>
       </c>
       <c r="F14" s="32" t="inlineStr">
@@ -3592,7 +3595,7 @@
       </c>
       <c r="C17" s="33" t="inlineStr">
         <is>
-          <t>DSO = Avg AR / Avg Revenue × 365</t>
+          <t>DSO = Avg AR / (Revenue_CY / 365)</t>
         </is>
       </c>
       <c r="D17" s="32" t="inlineStr">
@@ -3603,7 +3606,7 @@
       <c r="E17" s="34" t="inlineStr">
         <is>
           <t>Sheet "3 Metrics" col H
-Avg AR: Sheet "2" col B; Avg Revenue: Sheet "2" col F</t>
+Avg AR: Sheet "2" col B; Revenue CY: Sheet "1 Raw Data" col B rows 17–26</t>
         </is>
       </c>
       <c r="F17" s="32" t="inlineStr">
@@ -3630,7 +3633,7 @@
       </c>
       <c r="C18" s="33" t="inlineStr">
         <is>
-          <t>AR Turns = Avg Revenue / Avg AR  (times per year)</t>
+          <t>AR Turns = Revenue_CY / Avg AR  (times per year)</t>
         </is>
       </c>
       <c r="D18" s="32" t="inlineStr">
@@ -3640,7 +3643,8 @@
       </c>
       <c r="E18" s="34" t="inlineStr">
         <is>
-          <t>Sheet "3 Metrics" col I</t>
+          <t>Sheet "3 Metrics" col I
+Revenue CY: Sheet "1 Raw Data" col B rows 17–26; Avg AR: Sheet "2" col B</t>
         </is>
       </c>
       <c r="F18" s="32" t="inlineStr">
@@ -4069,10 +4073,11 @@
       </c>
       <c r="C31" s="33" t="inlineStr">
         <is>
-          <t>Q1: score 1.0–3.5  (Top performers)
-Q2: score 3.6–5.5
-Q3: score 5.6–7.5
-Q4: score 7.6–10.0  (Underperformers)</t>
+          <t>Q1: V-A Rank 1–3  (Top performers)
+Q2: V-A Rank 4–5
+Q3: V-A Rank 6–8
+Q4: V-A Rank 9–10  (Underperformers)
+Formula: =IF(H&lt;=3,"Q1",IF(H&lt;=5,"Q2",IF(H&lt;=8,"Q3","Q4")))</t>
         </is>
       </c>
       <c r="D31" s="32" t="inlineStr">
@@ -5784,45 +5789,45 @@
           <t>NVIDIA</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
-        <v>13626.5</v>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>5623.5</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>2048</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>26809.5</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>95709.5</v>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>(17254+9999)/2</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>(5965+5282)/2</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>(2667+1429)/2</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>(36998+16621)/2</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>(130497+60922)/2</t>
-        </is>
+      <c r="B3" s="4">
+        <f>('1 Raw Data'!B30+'1 Raw Data'!C30)/2</f>
+        <v/>
+      </c>
+      <c r="C3" s="4">
+        <f>('1 Raw Data'!D30+'1 Raw Data'!E30)/2</f>
+        <v/>
+      </c>
+      <c r="D3" s="4">
+        <f>('1 Raw Data'!F30+'1 Raw Data'!G30)/2</f>
+        <v/>
+      </c>
+      <c r="E3" s="4">
+        <f>('1 Raw Data'!D17+'1 Raw Data'!E17)/2</f>
+        <v/>
+      </c>
+      <c r="F3" s="4">
+        <f>('1 Raw Data'!B17+'1 Raw Data'!C17)/2</f>
+        <v/>
+      </c>
+      <c r="G3" s="4">
+        <f>FORMULATEXT(B3)</f>
+        <v/>
+      </c>
+      <c r="H3" s="4">
+        <f>FORMULATEXT(C3)</f>
+        <v/>
+      </c>
+      <c r="I3" s="4">
+        <f>FORMULATEXT(D3)</f>
+        <v/>
+      </c>
+      <c r="J3" s="4">
+        <f>FORMULATEXT(E3)</f>
+        <v/>
+      </c>
+      <c r="K3" s="4">
+        <f>FORMULATEXT(F3)</f>
+        <v/>
       </c>
     </row>
     <row r="4">
@@ -5831,45 +5836,45 @@
           <t>AMD</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
-        <v>4280</v>
-      </c>
-      <c r="C4" s="5" t="n">
-        <v>1988.5</v>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>1453.5</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>11979</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>24232.5</v>
-      </c>
-      <c r="G4" s="5" t="inlineStr">
-        <is>
-          <t>(4427+4133)/2</t>
-        </is>
-      </c>
-      <c r="H4" s="5" t="inlineStr">
-        <is>
-          <t>(1969+2008)/2</t>
-        </is>
-      </c>
-      <c r="I4" s="5" t="inlineStr">
-        <is>
-          <t>(1518+1389)/2</t>
-        </is>
-      </c>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t>(12408+11550)/2</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr">
-        <is>
-          <t>(25785+22680)/2</t>
-        </is>
+      <c r="B4" s="5">
+        <f>('1 Raw Data'!B31+'1 Raw Data'!C31)/2</f>
+        <v/>
+      </c>
+      <c r="C4" s="5">
+        <f>('1 Raw Data'!D31+'1 Raw Data'!E31)/2</f>
+        <v/>
+      </c>
+      <c r="D4" s="5">
+        <f>('1 Raw Data'!F31+'1 Raw Data'!G31)/2</f>
+        <v/>
+      </c>
+      <c r="E4" s="5">
+        <f>('1 Raw Data'!D18+'1 Raw Data'!E18)/2</f>
+        <v/>
+      </c>
+      <c r="F4" s="5">
+        <f>('1 Raw Data'!B18+'1 Raw Data'!C18)/2</f>
+        <v/>
+      </c>
+      <c r="G4" s="5">
+        <f>FORMULATEXT(B4)</f>
+        <v/>
+      </c>
+      <c r="H4" s="5">
+        <f>FORMULATEXT(C4)</f>
+        <v/>
+      </c>
+      <c r="I4" s="5">
+        <f>FORMULATEXT(D4)</f>
+        <v/>
+      </c>
+      <c r="J4" s="5">
+        <f>FORMULATEXT(E4)</f>
+        <v/>
+      </c>
+      <c r="K4" s="5">
+        <f>FORMULATEXT(F4)</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -5878,45 +5883,45 @@
           <t>Intel</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
-        <v>5164.5</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>11535</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>4017.5</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>33379</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>53664.5</v>
-      </c>
-      <c r="G5" s="4" t="inlineStr">
-        <is>
-          <t>(5021+5308)/2</t>
-        </is>
-      </c>
-      <c r="H5" s="4" t="inlineStr">
-        <is>
-          <t>(11774+11296)/2</t>
-        </is>
-      </c>
-      <c r="I5" s="4" t="inlineStr">
-        <is>
-          <t>(3968+4067)/2</t>
-        </is>
-      </c>
-      <c r="J5" s="4" t="inlineStr">
-        <is>
-          <t>(35737+31021)/2</t>
-        </is>
-      </c>
-      <c r="K5" s="4" t="inlineStr">
-        <is>
-          <t>(53101+54228)/2</t>
-        </is>
+      <c r="B5" s="4">
+        <f>('1 Raw Data'!B32+'1 Raw Data'!C32)/2</f>
+        <v/>
+      </c>
+      <c r="C5" s="4">
+        <f>('1 Raw Data'!D32+'1 Raw Data'!E32)/2</f>
+        <v/>
+      </c>
+      <c r="D5" s="4">
+        <f>('1 Raw Data'!F32+'1 Raw Data'!G32)/2</f>
+        <v/>
+      </c>
+      <c r="E5" s="4">
+        <f>('1 Raw Data'!D19+'1 Raw Data'!E19)/2</f>
+        <v/>
+      </c>
+      <c r="F5" s="4">
+        <f>('1 Raw Data'!B19+'1 Raw Data'!C19)/2</f>
+        <v/>
+      </c>
+      <c r="G5" s="4">
+        <f>FORMULATEXT(B5)</f>
+        <v/>
+      </c>
+      <c r="H5" s="4">
+        <f>FORMULATEXT(C5)</f>
+        <v/>
+      </c>
+      <c r="I5" s="4">
+        <f>FORMULATEXT(D5)</f>
+        <v/>
+      </c>
+      <c r="J5" s="4">
+        <f>FORMULATEXT(E5)</f>
+        <v/>
+      </c>
+      <c r="K5" s="4">
+        <f>FORMULATEXT(F5)</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -5925,45 +5930,45 @@
           <t>TXN</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
-        <v>1831</v>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>3814</v>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>390</v>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>6365.5</v>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>16579.5</v>
-      </c>
-      <c r="G6" s="5" t="inlineStr">
-        <is>
-          <t>(1741+1921)/2</t>
-        </is>
-      </c>
-      <c r="H6" s="5" t="inlineStr">
-        <is>
-          <t>(4081+3547)/2</t>
-        </is>
-      </c>
-      <c r="I6" s="5" t="inlineStr">
-        <is>
-          <t>(376+404)/2</t>
-        </is>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>(6240+6491)/2</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="inlineStr">
-        <is>
-          <t>(15640+17519)/2</t>
-        </is>
+      <c r="B6" s="5">
+        <f>('1 Raw Data'!B33+'1 Raw Data'!C33)/2</f>
+        <v/>
+      </c>
+      <c r="C6" s="5">
+        <f>('1 Raw Data'!D33+'1 Raw Data'!E33)/2</f>
+        <v/>
+      </c>
+      <c r="D6" s="5">
+        <f>('1 Raw Data'!F33+'1 Raw Data'!G33)/2</f>
+        <v/>
+      </c>
+      <c r="E6" s="5">
+        <f>('1 Raw Data'!D20+'1 Raw Data'!E20)/2</f>
+        <v/>
+      </c>
+      <c r="F6" s="5">
+        <f>('1 Raw Data'!B20+'1 Raw Data'!C20)/2</f>
+        <v/>
+      </c>
+      <c r="G6" s="5">
+        <f>FORMULATEXT(B6)</f>
+        <v/>
+      </c>
+      <c r="H6" s="5">
+        <f>FORMULATEXT(C6)</f>
+        <v/>
+      </c>
+      <c r="I6" s="5">
+        <f>FORMULATEXT(D6)</f>
+        <v/>
+      </c>
+      <c r="J6" s="5">
+        <f>FORMULATEXT(E6)</f>
+        <v/>
+      </c>
+      <c r="K6" s="5">
+        <f>FORMULATEXT(F6)</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -5972,45 +5977,45 @@
           <t>Qualcomm</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
-        <v>6007</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>2441</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>3977.5</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>16416.5</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>37391</v>
-      </c>
-      <c r="G7" s="4" t="inlineStr">
-        <is>
-          <t>(6400+5614)/2</t>
-        </is>
-      </c>
-      <c r="H7" s="4" t="inlineStr">
-        <is>
-          <t>(2327+2555)/2</t>
-        </is>
-      </c>
-      <c r="I7" s="4" t="inlineStr">
-        <is>
-          <t>(4213+3742)/2</t>
-        </is>
-      </c>
-      <c r="J7" s="4" t="inlineStr">
-        <is>
-          <t>(17026+15807)/2</t>
-        </is>
-      </c>
-      <c r="K7" s="4" t="inlineStr">
-        <is>
-          <t>(38962+35820)/2</t>
-        </is>
+      <c r="B7" s="4">
+        <f>('1 Raw Data'!B34+'1 Raw Data'!C34)/2</f>
+        <v/>
+      </c>
+      <c r="C7" s="4">
+        <f>('1 Raw Data'!D34+'1 Raw Data'!E34)/2</f>
+        <v/>
+      </c>
+      <c r="D7" s="4">
+        <f>('1 Raw Data'!F34+'1 Raw Data'!G34)/2</f>
+        <v/>
+      </c>
+      <c r="E7" s="4">
+        <f>('1 Raw Data'!D21+'1 Raw Data'!E21)/2</f>
+        <v/>
+      </c>
+      <c r="F7" s="4">
+        <f>('1 Raw Data'!B21+'1 Raw Data'!C21)/2</f>
+        <v/>
+      </c>
+      <c r="G7" s="4">
+        <f>FORMULATEXT(B7)</f>
+        <v/>
+      </c>
+      <c r="H7" s="4">
+        <f>FORMULATEXT(C7)</f>
+        <v/>
+      </c>
+      <c r="I7" s="4">
+        <f>FORMULATEXT(D7)</f>
+        <v/>
+      </c>
+      <c r="J7" s="4">
+        <f>FORMULATEXT(E7)</f>
+        <v/>
+      </c>
+      <c r="K7" s="4">
+        <f>FORMULATEXT(F7)</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -6019,45 +6024,45 @@
           <t>NXP</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
-        <v>1669</v>
-      </c>
-      <c r="C8" s="5" t="n">
-        <v>1821</v>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>1040</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>5528</v>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>12943.5</v>
-      </c>
-      <c r="G8" s="5" t="inlineStr">
-        <is>
-          <t>(1597+1741)/2</t>
-        </is>
-      </c>
-      <c r="H8" s="5" t="inlineStr">
-        <is>
-          <t>(1736+1906)/2</t>
-        </is>
-      </c>
-      <c r="I8" s="5" t="inlineStr">
-        <is>
-          <t>(980+1100)/2</t>
-        </is>
-      </c>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>(5348+5708)/2</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr">
-        <is>
-          <t>(12613+13274)/2</t>
-        </is>
+      <c r="B8" s="5">
+        <f>('1 Raw Data'!B35+'1 Raw Data'!C35)/2</f>
+        <v/>
+      </c>
+      <c r="C8" s="5">
+        <f>('1 Raw Data'!D35+'1 Raw Data'!E35)/2</f>
+        <v/>
+      </c>
+      <c r="D8" s="5">
+        <f>('1 Raw Data'!F35+'1 Raw Data'!G35)/2</f>
+        <v/>
+      </c>
+      <c r="E8" s="5">
+        <f>('1 Raw Data'!D22+'1 Raw Data'!E22)/2</f>
+        <v/>
+      </c>
+      <c r="F8" s="5">
+        <f>('1 Raw Data'!B22+'1 Raw Data'!C22)/2</f>
+        <v/>
+      </c>
+      <c r="G8" s="5">
+        <f>FORMULATEXT(B8)</f>
+        <v/>
+      </c>
+      <c r="H8" s="5">
+        <f>FORMULATEXT(C8)</f>
+        <v/>
+      </c>
+      <c r="I8" s="5">
+        <f>FORMULATEXT(D8)</f>
+        <v/>
+      </c>
+      <c r="J8" s="5">
+        <f>FORMULATEXT(E8)</f>
+        <v/>
+      </c>
+      <c r="K8" s="5">
+        <f>FORMULATEXT(F8)</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -6066,45 +6071,45 @@
           <t>TSMC</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
-        <v>9814.5</v>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>13398.5</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>5360.5</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>35643.5</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>79977.5</v>
-      </c>
-      <c r="G9" s="4" t="inlineStr">
-        <is>
-          <t>(10938+8691)/2</t>
-        </is>
-      </c>
-      <c r="H9" s="4" t="inlineStr">
-        <is>
-          <t>(14063+12734)/2</t>
-        </is>
-      </c>
-      <c r="I9" s="4" t="inlineStr">
-        <is>
-          <t>(5625+5096)/2</t>
-        </is>
-      </c>
-      <c r="J9" s="4" t="inlineStr">
-        <is>
-          <t>(39686+31601)/2</t>
-        </is>
-      </c>
-      <c r="K9" s="4" t="inlineStr">
-        <is>
-          <t>(90447+69508)/2</t>
-        </is>
+      <c r="B9" s="4">
+        <f>('1 Raw Data'!B36+'1 Raw Data'!C36)/2</f>
+        <v/>
+      </c>
+      <c r="C9" s="4">
+        <f>('1 Raw Data'!D36+'1 Raw Data'!E36)/2</f>
+        <v/>
+      </c>
+      <c r="D9" s="4">
+        <f>('1 Raw Data'!F36+'1 Raw Data'!G36)/2</f>
+        <v/>
+      </c>
+      <c r="E9" s="4">
+        <f>('1 Raw Data'!D23+'1 Raw Data'!E23)/2</f>
+        <v/>
+      </c>
+      <c r="F9" s="4">
+        <f>('1 Raw Data'!B23+'1 Raw Data'!C23)/2</f>
+        <v/>
+      </c>
+      <c r="G9" s="4">
+        <f>FORMULATEXT(B9)</f>
+        <v/>
+      </c>
+      <c r="H9" s="4">
+        <f>FORMULATEXT(C9)</f>
+        <v/>
+      </c>
+      <c r="I9" s="4">
+        <f>FORMULATEXT(D9)</f>
+        <v/>
+      </c>
+      <c r="J9" s="4">
+        <f>FORMULATEXT(E9)</f>
+        <v/>
+      </c>
+      <c r="K9" s="4">
+        <f>FORMULATEXT(F9)</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -6113,45 +6118,45 @@
           <t>Micron</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
-        <v>3029.5</v>
-      </c>
-      <c r="C10" s="5" t="n">
-        <v>8358</v>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>1957</v>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>18443</v>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>20325.5</v>
-      </c>
-      <c r="G10" s="5" t="inlineStr">
-        <is>
-          <t>(3302+2757)/2</t>
-        </is>
-      </c>
-      <c r="H10" s="5" t="inlineStr">
-        <is>
-          <t>(8622+8094)/2</t>
-        </is>
-      </c>
-      <c r="I10" s="5" t="inlineStr">
-        <is>
-          <t>(2232+1682)/2</t>
-        </is>
-      </c>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>(19440+17446)/2</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr">
-        <is>
-          <t>(25111+15540)/2</t>
-        </is>
+      <c r="B10" s="5">
+        <f>('1 Raw Data'!B37+'1 Raw Data'!C37)/2</f>
+        <v/>
+      </c>
+      <c r="C10" s="5">
+        <f>('1 Raw Data'!D37+'1 Raw Data'!E37)/2</f>
+        <v/>
+      </c>
+      <c r="D10" s="5">
+        <f>('1 Raw Data'!F37+'1 Raw Data'!G37)/2</f>
+        <v/>
+      </c>
+      <c r="E10" s="5">
+        <f>('1 Raw Data'!D24+'1 Raw Data'!E24)/2</f>
+        <v/>
+      </c>
+      <c r="F10" s="5">
+        <f>('1 Raw Data'!B24+'1 Raw Data'!C24)/2</f>
+        <v/>
+      </c>
+      <c r="G10" s="5">
+        <f>FORMULATEXT(B10)</f>
+        <v/>
+      </c>
+      <c r="H10" s="5">
+        <f>FORMULATEXT(C10)</f>
+        <v/>
+      </c>
+      <c r="I10" s="5">
+        <f>FORMULATEXT(D10)</f>
+        <v/>
+      </c>
+      <c r="J10" s="5">
+        <f>FORMULATEXT(E10)</f>
+        <v/>
+      </c>
+      <c r="K10" s="5">
+        <f>FORMULATEXT(F10)</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -6160,45 +6165,45 @@
           <t>STM</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n">
-        <v>2307</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>2902.5</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>1411.5</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>8748.5</v>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>15283</v>
-      </c>
-      <c r="G11" s="4" t="inlineStr">
-        <is>
-          <t>(2014+2600)/2</t>
-        </is>
-      </c>
-      <c r="H11" s="4" t="inlineStr">
-        <is>
-          <t>(2737+3068)/2</t>
-        </is>
-      </c>
-      <c r="I11" s="4" t="inlineStr">
-        <is>
-          <t>(1300+1523)/2</t>
-        </is>
-      </c>
-      <c r="J11" s="4" t="inlineStr">
-        <is>
-          <t>(8351+9146)/2</t>
-        </is>
-      </c>
-      <c r="K11" s="4" t="inlineStr">
-        <is>
-          <t>(13276+17290)/2</t>
-        </is>
+      <c r="B11" s="4">
+        <f>('1 Raw Data'!B38+'1 Raw Data'!C38)/2</f>
+        <v/>
+      </c>
+      <c r="C11" s="4">
+        <f>('1 Raw Data'!D38+'1 Raw Data'!E38)/2</f>
+        <v/>
+      </c>
+      <c r="D11" s="4">
+        <f>('1 Raw Data'!F38+'1 Raw Data'!G38)/2</f>
+        <v/>
+      </c>
+      <c r="E11" s="4">
+        <f>('1 Raw Data'!D25+'1 Raw Data'!E25)/2</f>
+        <v/>
+      </c>
+      <c r="F11" s="4">
+        <f>('1 Raw Data'!B25+'1 Raw Data'!C25)/2</f>
+        <v/>
+      </c>
+      <c r="G11" s="4">
+        <f>FORMULATEXT(B11)</f>
+        <v/>
+      </c>
+      <c r="H11" s="4">
+        <f>FORMULATEXT(C11)</f>
+        <v/>
+      </c>
+      <c r="I11" s="4">
+        <f>FORMULATEXT(D11)</f>
+        <v/>
+      </c>
+      <c r="J11" s="4">
+        <f>FORMULATEXT(E11)</f>
+        <v/>
+      </c>
+      <c r="K11" s="4">
+        <f>FORMULATEXT(F11)</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -6207,45 +6212,45 @@
           <t>Infineon</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
-        <v>1631.5</v>
-      </c>
-      <c r="C12" s="5" t="n">
-        <v>3288</v>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>1001</v>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>4925.5</v>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>8539</v>
-      </c>
-      <c r="G12" s="5" t="inlineStr">
-        <is>
-          <t>(1554+1709)/2</t>
-        </is>
-      </c>
-      <c r="H12" s="5" t="inlineStr">
-        <is>
-          <t>(3279+3297)/2</t>
-        </is>
-      </c>
-      <c r="I12" s="5" t="inlineStr">
-        <is>
-          <t>(966+1036)/2</t>
-        </is>
-      </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>(5160+4691)/2</t>
-        </is>
-      </c>
-      <c r="K12" s="5" t="inlineStr">
-        <is>
-          <t>(8390+8688)/2</t>
-        </is>
+      <c r="B12" s="5">
+        <f>('1 Raw Data'!B39+'1 Raw Data'!C39)/2</f>
+        <v/>
+      </c>
+      <c r="C12" s="5">
+        <f>('1 Raw Data'!D39+'1 Raw Data'!E39)/2</f>
+        <v/>
+      </c>
+      <c r="D12" s="5">
+        <f>('1 Raw Data'!F39+'1 Raw Data'!G39)/2</f>
+        <v/>
+      </c>
+      <c r="E12" s="5">
+        <f>('1 Raw Data'!D26+'1 Raw Data'!E26)/2</f>
+        <v/>
+      </c>
+      <c r="F12" s="5">
+        <f>('1 Raw Data'!B26+'1 Raw Data'!C26)/2</f>
+        <v/>
+      </c>
+      <c r="G12" s="5">
+        <f>FORMULATEXT(B12)</f>
+        <v/>
+      </c>
+      <c r="H12" s="5">
+        <f>FORMULATEXT(C12)</f>
+        <v/>
+      </c>
+      <c r="I12" s="5">
+        <f>FORMULATEXT(D12)</f>
+        <v/>
+      </c>
+      <c r="J12" s="5">
+        <f>FORMULATEXT(E12)</f>
+        <v/>
+      </c>
+      <c r="K12" s="5">
+        <f>FORMULATEXT(F12)</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -6367,41 +6372,53 @@
           <t>NVIDIA</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
-        <v>33901</v>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>20088</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>17202</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>13.18</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>0.26</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>2.79</v>
-      </c>
-      <c r="H3" s="4" t="n">
-        <v>38.12</v>
-      </c>
-      <c r="I3" s="4" t="n">
-        <v>9.58</v>
-      </c>
-      <c r="J3" s="4" t="n">
-        <v>76.56999999999999</v>
-      </c>
-      <c r="K3" s="4" t="n">
-        <v>27.88</v>
-      </c>
-      <c r="L3" s="4" t="n">
-        <v>86.81</v>
-      </c>
-      <c r="M3" s="4" t="n">
-        <v>49.11</v>
+      <c r="B3" s="4">
+        <f>'1 Raw Data'!B42-'1 Raw Data'!E42</f>
+        <v/>
+      </c>
+      <c r="C3" s="4">
+        <f>'1 Raw Data'!B42-'1 Raw Data'!C42-'1 Raw Data'!E42+'1 Raw Data'!G42</f>
+        <v/>
+      </c>
+      <c r="D3" s="4">
+        <f>'2 Average Balances'!B3+'2 Average Balances'!C3-'2 Average Balances'!D3</f>
+        <v/>
+      </c>
+      <c r="E3" s="4">
+        <f>D3/('1 Raw Data'!B17)*100</f>
+        <v/>
+      </c>
+      <c r="F3" s="4">
+        <f>B3/('1 Raw Data'!B17)</f>
+        <v/>
+      </c>
+      <c r="G3" s="4">
+        <f>'1 Raw Data'!B42/'1 Raw Data'!E42</f>
+        <v/>
+      </c>
+      <c r="H3" s="4">
+        <f>'2 Average Balances'!B3/('1 Raw Data'!B17/365)</f>
+        <v/>
+      </c>
+      <c r="I3" s="4">
+        <f>'1 Raw Data'!B17/'2 Average Balances'!B3</f>
+        <v/>
+      </c>
+      <c r="J3" s="4">
+        <f>'2 Average Balances'!C3/('2 Average Balances'!E3/365)</f>
+        <v/>
+      </c>
+      <c r="K3" s="4">
+        <f>'2 Average Balances'!D3/('2 Average Balances'!E3/365)</f>
+        <v/>
+      </c>
+      <c r="L3" s="4">
+        <f>H3+J3-K3</f>
+        <v/>
+      </c>
+      <c r="M3" s="4">
+        <f>'1 Raw Data'!I42/('1 Raw Data'!B17)*100</f>
+        <v/>
       </c>
       <c r="N3" s="4" t="inlineStr"/>
     </row>
@@ -6411,41 +6428,53 @@
           <t>AMD</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
-        <v>8250</v>
-      </c>
-      <c r="C4" s="5" t="n">
-        <v>2850</v>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>4815</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>18.67</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>0.32</v>
-      </c>
-      <c r="G4" s="5" t="n">
-        <v>2.74</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>60.59</v>
-      </c>
-      <c r="I4" s="5" t="n">
-        <v>6.02</v>
-      </c>
-      <c r="J4" s="5" t="n">
-        <v>60.59</v>
-      </c>
-      <c r="K4" s="5" t="n">
-        <v>44.29</v>
-      </c>
-      <c r="L4" s="5" t="n">
-        <v>76.89</v>
-      </c>
-      <c r="M4" s="5" t="n">
-        <v>10.46</v>
+      <c r="B4" s="5">
+        <f>'1 Raw Data'!B43-'1 Raw Data'!E43</f>
+        <v/>
+      </c>
+      <c r="C4" s="5">
+        <f>'1 Raw Data'!B43-'1 Raw Data'!C43-'1 Raw Data'!E43+'1 Raw Data'!G43</f>
+        <v/>
+      </c>
+      <c r="D4" s="5">
+        <f>'2 Average Balances'!B4+'2 Average Balances'!C4-'2 Average Balances'!D4</f>
+        <v/>
+      </c>
+      <c r="E4" s="5">
+        <f>D4/('1 Raw Data'!B18)*100</f>
+        <v/>
+      </c>
+      <c r="F4" s="5">
+        <f>B4/('1 Raw Data'!B18)</f>
+        <v/>
+      </c>
+      <c r="G4" s="5">
+        <f>'1 Raw Data'!B43/'1 Raw Data'!E43</f>
+        <v/>
+      </c>
+      <c r="H4" s="5">
+        <f>'2 Average Balances'!B4/('1 Raw Data'!B18/365)</f>
+        <v/>
+      </c>
+      <c r="I4" s="5">
+        <f>'1 Raw Data'!B18/'2 Average Balances'!B4</f>
+        <v/>
+      </c>
+      <c r="J4" s="5">
+        <f>'2 Average Balances'!C4/('2 Average Balances'!E4/365)</f>
+        <v/>
+      </c>
+      <c r="K4" s="5">
+        <f>'2 Average Balances'!D4/('2 Average Balances'!E4/365)</f>
+        <v/>
+      </c>
+      <c r="L4" s="5">
+        <f>H4+J4-K4</f>
+        <v/>
+      </c>
+      <c r="M4" s="5">
+        <f>'1 Raw Data'!I43/('1 Raw Data'!B18)*100</f>
+        <v/>
       </c>
       <c r="N4" s="8" t="inlineStr"/>
     </row>
@@ -6455,41 +6484,53 @@
           <t>Intel</t>
         </is>
       </c>
-      <c r="B5" s="4" t="n">
-        <v>7107</v>
-      </c>
-      <c r="C5" s="4" t="n">
-        <v>1207</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>12682</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>23.88</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>0.13</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>1.33</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>35.5</v>
-      </c>
-      <c r="I5" s="9" t="n">
-        <v>10.28</v>
-      </c>
-      <c r="J5" s="4" t="n">
-        <v>126.13</v>
-      </c>
-      <c r="K5" s="4" t="n">
-        <v>43.93</v>
-      </c>
-      <c r="L5" s="4" t="n">
-        <v>117.7</v>
-      </c>
-      <c r="M5" s="4" t="n">
-        <v>15.62</v>
+      <c r="B5" s="4">
+        <f>'1 Raw Data'!B44-'1 Raw Data'!E44</f>
+        <v/>
+      </c>
+      <c r="C5" s="4">
+        <f>'1 Raw Data'!B44-'1 Raw Data'!C44-'1 Raw Data'!E44+'1 Raw Data'!G44</f>
+        <v/>
+      </c>
+      <c r="D5" s="4">
+        <f>'2 Average Balances'!B5+'2 Average Balances'!C5-'2 Average Balances'!D5</f>
+        <v/>
+      </c>
+      <c r="E5" s="4">
+        <f>D5/('1 Raw Data'!B19)*100</f>
+        <v/>
+      </c>
+      <c r="F5" s="4">
+        <f>B5/('1 Raw Data'!B19)</f>
+        <v/>
+      </c>
+      <c r="G5" s="4">
+        <f>'1 Raw Data'!B44/'1 Raw Data'!E44</f>
+        <v/>
+      </c>
+      <c r="H5" s="4">
+        <f>'2 Average Balances'!B5/('1 Raw Data'!B19/365)</f>
+        <v/>
+      </c>
+      <c r="I5" s="9">
+        <f>'1 Raw Data'!B19/'2 Average Balances'!B5</f>
+        <v/>
+      </c>
+      <c r="J5" s="4">
+        <f>'2 Average Balances'!C5/('2 Average Balances'!E5/365)</f>
+        <v/>
+      </c>
+      <c r="K5" s="4">
+        <f>'2 Average Balances'!D5/('2 Average Balances'!E5/365)</f>
+        <v/>
+      </c>
+      <c r="L5" s="4">
+        <f>H5+J5-K5</f>
+        <v/>
+      </c>
+      <c r="M5" s="4">
+        <f>'1 Raw Data'!I44/('1 Raw Data'!B19)*100</f>
+        <v/>
       </c>
       <c r="N5" s="10" t="inlineStr">
         <is>
@@ -6503,41 +6544,53 @@
           <t>TXN</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
-        <v>5483</v>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>2349</v>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>5255</v>
-      </c>
-      <c r="E6" s="5" t="n">
-        <v>33.6</v>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>0.35</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>2.55</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>42.74</v>
-      </c>
-      <c r="I6" s="5" t="n">
-        <v>8.539999999999999</v>
-      </c>
-      <c r="J6" s="8" t="n">
-        <v>218.7</v>
-      </c>
-      <c r="K6" s="5" t="n">
-        <v>22.37</v>
-      </c>
-      <c r="L6" s="5" t="n">
-        <v>239.07</v>
-      </c>
-      <c r="M6" s="5" t="n">
-        <v>40.17</v>
+      <c r="B6" s="5">
+        <f>'1 Raw Data'!B45-'1 Raw Data'!E45</f>
+        <v/>
+      </c>
+      <c r="C6" s="5">
+        <f>'1 Raw Data'!B45-'1 Raw Data'!C45-'1 Raw Data'!E45+'1 Raw Data'!G45</f>
+        <v/>
+      </c>
+      <c r="D6" s="5">
+        <f>'2 Average Balances'!B6+'2 Average Balances'!C6-'2 Average Balances'!D6</f>
+        <v/>
+      </c>
+      <c r="E6" s="5">
+        <f>D6/('1 Raw Data'!B20)*100</f>
+        <v/>
+      </c>
+      <c r="F6" s="5">
+        <f>B6/('1 Raw Data'!B20)</f>
+        <v/>
+      </c>
+      <c r="G6" s="5">
+        <f>'1 Raw Data'!B45/'1 Raw Data'!E45</f>
+        <v/>
+      </c>
+      <c r="H6" s="5">
+        <f>'2 Average Balances'!B6/('1 Raw Data'!B20/365)</f>
+        <v/>
+      </c>
+      <c r="I6" s="5">
+        <f>'1 Raw Data'!B20/'2 Average Balances'!B6</f>
+        <v/>
+      </c>
+      <c r="J6" s="8">
+        <f>'2 Average Balances'!C6/('2 Average Balances'!E6/365)</f>
+        <v/>
+      </c>
+      <c r="K6" s="5">
+        <f>'2 Average Balances'!D6/('2 Average Balances'!E6/365)</f>
+        <v/>
+      </c>
+      <c r="L6" s="5">
+        <f>H6+J6-K6</f>
+        <v/>
+      </c>
+      <c r="M6" s="5">
+        <f>'1 Raw Data'!I45/('1 Raw Data'!B20)*100</f>
+        <v/>
       </c>
       <c r="N6" s="11" t="inlineStr">
         <is>
@@ -6551,41 +6604,53 @@
           <t>Qualcomm</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
-        <v>9360</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>3120</v>
-      </c>
-      <c r="D7" s="4" t="n">
-        <v>4470.5</v>
-      </c>
-      <c r="E7" s="4" t="n">
-        <v>11.47</v>
-      </c>
-      <c r="F7" s="4" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>1.93</v>
-      </c>
-      <c r="H7" s="9" t="n">
-        <v>56.27</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>6.49</v>
-      </c>
-      <c r="J7" s="9" t="n">
-        <v>54.28</v>
-      </c>
-      <c r="K7" s="9" t="n">
-        <v>88.44</v>
-      </c>
-      <c r="L7" s="9" t="n">
-        <v>22.11</v>
-      </c>
-      <c r="M7" s="9" t="n">
-        <v>28.05</v>
+      <c r="B7" s="4">
+        <f>'1 Raw Data'!B46-'1 Raw Data'!E46</f>
+        <v/>
+      </c>
+      <c r="C7" s="4">
+        <f>'1 Raw Data'!B46-'1 Raw Data'!C46-'1 Raw Data'!E46+'1 Raw Data'!G46</f>
+        <v/>
+      </c>
+      <c r="D7" s="4">
+        <f>'2 Average Balances'!B7+'2 Average Balances'!C7-'2 Average Balances'!D7</f>
+        <v/>
+      </c>
+      <c r="E7" s="4">
+        <f>D7/('1 Raw Data'!B21)*100</f>
+        <v/>
+      </c>
+      <c r="F7" s="4">
+        <f>B7/('1 Raw Data'!B21)</f>
+        <v/>
+      </c>
+      <c r="G7" s="4">
+        <f>'1 Raw Data'!B46/'1 Raw Data'!E46</f>
+        <v/>
+      </c>
+      <c r="H7" s="9">
+        <f>'2 Average Balances'!B7/('1 Raw Data'!B21/365)</f>
+        <v/>
+      </c>
+      <c r="I7" s="4">
+        <f>'1 Raw Data'!B21/'2 Average Balances'!B7</f>
+        <v/>
+      </c>
+      <c r="J7" s="9">
+        <f>'2 Average Balances'!C7/('2 Average Balances'!E7/365)</f>
+        <v/>
+      </c>
+      <c r="K7" s="9">
+        <f>'2 Average Balances'!D7/('2 Average Balances'!E7/365)</f>
+        <v/>
+      </c>
+      <c r="L7" s="9">
+        <f>H7+J7-K7</f>
+        <v/>
+      </c>
+      <c r="M7" s="9">
+        <f>'1 Raw Data'!I46/('1 Raw Data'!B21)*100</f>
+        <v/>
       </c>
       <c r="N7" s="9" t="inlineStr"/>
     </row>
@@ -6595,41 +6660,53 @@
           <t>NXP</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
-        <v>2305</v>
-      </c>
-      <c r="C8" s="5" t="n">
-        <v>805</v>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>2450</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>19.43</v>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>1.55</v>
-      </c>
-      <c r="H8" s="5" t="n">
-        <v>48.29</v>
-      </c>
-      <c r="I8" s="5" t="n">
-        <v>7.56</v>
-      </c>
-      <c r="J8" s="5" t="n">
-        <v>120.21</v>
-      </c>
-      <c r="K8" s="5" t="n">
-        <v>68.65000000000001</v>
-      </c>
-      <c r="L8" s="5" t="n">
-        <v>99.84999999999999</v>
-      </c>
-      <c r="M8" s="5" t="n">
-        <v>22.3</v>
+      <c r="B8" s="5">
+        <f>'1 Raw Data'!B47-'1 Raw Data'!E47</f>
+        <v/>
+      </c>
+      <c r="C8" s="5">
+        <f>'1 Raw Data'!B47-'1 Raw Data'!C47-'1 Raw Data'!E47+'1 Raw Data'!G47</f>
+        <v/>
+      </c>
+      <c r="D8" s="5">
+        <f>'2 Average Balances'!B8+'2 Average Balances'!C8-'2 Average Balances'!D8</f>
+        <v/>
+      </c>
+      <c r="E8" s="5">
+        <f>D8/('1 Raw Data'!B22)*100</f>
+        <v/>
+      </c>
+      <c r="F8" s="5">
+        <f>B8/('1 Raw Data'!B22)</f>
+        <v/>
+      </c>
+      <c r="G8" s="5">
+        <f>'1 Raw Data'!B47/'1 Raw Data'!E47</f>
+        <v/>
+      </c>
+      <c r="H8" s="5">
+        <f>'2 Average Balances'!B8/('1 Raw Data'!B22/365)</f>
+        <v/>
+      </c>
+      <c r="I8" s="5">
+        <f>'1 Raw Data'!B22/'2 Average Balances'!B8</f>
+        <v/>
+      </c>
+      <c r="J8" s="5">
+        <f>'2 Average Balances'!C8/('2 Average Balances'!E8/365)</f>
+        <v/>
+      </c>
+      <c r="K8" s="5">
+        <f>'2 Average Balances'!D8/('2 Average Balances'!E8/365)</f>
+        <v/>
+      </c>
+      <c r="L8" s="5">
+        <f>H8+J8-K8</f>
+        <v/>
+      </c>
+      <c r="M8" s="5">
+        <f>'1 Raw Data'!I47/('1 Raw Data'!B22)*100</f>
+        <v/>
       </c>
       <c r="N8" s="5" t="inlineStr"/>
     </row>
@@ -6639,41 +6716,53 @@
           <t>TSMC</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
-        <v>44001</v>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>7001</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>17852.5</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>19.74</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>0.49</v>
-      </c>
-      <c r="G9" s="4" t="n">
-        <v>2.76</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>39.63</v>
-      </c>
-      <c r="I9" s="4" t="n">
-        <v>9.210000000000001</v>
-      </c>
-      <c r="J9" s="4" t="n">
-        <v>137.22</v>
-      </c>
-      <c r="K9" s="4" t="n">
-        <v>54.9</v>
-      </c>
-      <c r="L9" s="4" t="n">
-        <v>121.95</v>
-      </c>
-      <c r="M9" s="4" t="n">
-        <v>62.19</v>
+      <c r="B9" s="4">
+        <f>'1 Raw Data'!B48-'1 Raw Data'!E48</f>
+        <v/>
+      </c>
+      <c r="C9" s="4">
+        <f>'1 Raw Data'!B48-'1 Raw Data'!C48-'1 Raw Data'!E48+'1 Raw Data'!G48</f>
+        <v/>
+      </c>
+      <c r="D9" s="4">
+        <f>'2 Average Balances'!B9+'2 Average Balances'!C9-'2 Average Balances'!D9</f>
+        <v/>
+      </c>
+      <c r="E9" s="4">
+        <f>D9/('1 Raw Data'!B23)*100</f>
+        <v/>
+      </c>
+      <c r="F9" s="4">
+        <f>B9/('1 Raw Data'!B23)</f>
+        <v/>
+      </c>
+      <c r="G9" s="4">
+        <f>'1 Raw Data'!B48/'1 Raw Data'!E48</f>
+        <v/>
+      </c>
+      <c r="H9" s="4">
+        <f>'2 Average Balances'!B9/('1 Raw Data'!B23/365)</f>
+        <v/>
+      </c>
+      <c r="I9" s="4">
+        <f>'1 Raw Data'!B23/'2 Average Balances'!B9</f>
+        <v/>
+      </c>
+      <c r="J9" s="4">
+        <f>'2 Average Balances'!C9/('2 Average Balances'!E9/365)</f>
+        <v/>
+      </c>
+      <c r="K9" s="4">
+        <f>'2 Average Balances'!D9/('2 Average Balances'!E9/365)</f>
+        <v/>
+      </c>
+      <c r="L9" s="4">
+        <f>H9+J9-K9</f>
+        <v/>
+      </c>
+      <c r="M9" s="4">
+        <f>'1 Raw Data'!I48/('1 Raw Data'!B23)*100</f>
+        <v/>
       </c>
       <c r="N9" s="10" t="inlineStr">
         <is>
@@ -6687,41 +6776,53 @@
           <t>Micron</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
-        <v>10116</v>
-      </c>
-      <c r="C10" s="5" t="n">
-        <v>1831</v>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>9430.5</v>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>37.55</v>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="G10" s="5" t="n">
-        <v>2.52</v>
-      </c>
-      <c r="H10" s="5" t="n">
-        <v>44.04</v>
-      </c>
-      <c r="I10" s="8" t="n">
-        <v>8.289999999999999</v>
-      </c>
-      <c r="J10" s="5" t="n">
-        <v>165.43</v>
-      </c>
-      <c r="K10" s="5" t="n">
-        <v>38.73</v>
-      </c>
-      <c r="L10" s="5" t="n">
-        <v>170.74</v>
-      </c>
-      <c r="M10" s="5" t="n">
-        <v>33.88</v>
+      <c r="B10" s="5">
+        <f>'1 Raw Data'!B49-'1 Raw Data'!E49</f>
+        <v/>
+      </c>
+      <c r="C10" s="5">
+        <f>'1 Raw Data'!B49-'1 Raw Data'!C49-'1 Raw Data'!E49+'1 Raw Data'!G49</f>
+        <v/>
+      </c>
+      <c r="D10" s="5">
+        <f>'2 Average Balances'!B10+'2 Average Balances'!C10-'2 Average Balances'!D10</f>
+        <v/>
+      </c>
+      <c r="E10" s="5">
+        <f>D10/('1 Raw Data'!B24)*100</f>
+        <v/>
+      </c>
+      <c r="F10" s="5">
+        <f>B10/('1 Raw Data'!B24)</f>
+        <v/>
+      </c>
+      <c r="G10" s="5">
+        <f>'1 Raw Data'!B49/'1 Raw Data'!E49</f>
+        <v/>
+      </c>
+      <c r="H10" s="5">
+        <f>'2 Average Balances'!B10/('1 Raw Data'!B24/365)</f>
+        <v/>
+      </c>
+      <c r="I10" s="8">
+        <f>'1 Raw Data'!B24/'2 Average Balances'!B10</f>
+        <v/>
+      </c>
+      <c r="J10" s="5">
+        <f>'2 Average Balances'!C10/('2 Average Balances'!E10/365)</f>
+        <v/>
+      </c>
+      <c r="K10" s="5">
+        <f>'2 Average Balances'!D10/('2 Average Balances'!E10/365)</f>
+        <v/>
+      </c>
+      <c r="L10" s="5">
+        <f>H10+J10-K10</f>
+        <v/>
+      </c>
+      <c r="M10" s="5">
+        <f>'1 Raw Data'!I49/('1 Raw Data'!B24)*100</f>
+        <v/>
       </c>
       <c r="N10" s="11" t="inlineStr">
         <is>
@@ -6735,41 +6836,53 @@
           <t>STM</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n">
-        <v>4845</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>1861</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>3798</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>28.61</v>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>0.37</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>2.13</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>63.43</v>
-      </c>
-      <c r="I11" s="4" t="n">
-        <v>5.75</v>
-      </c>
-      <c r="J11" s="4" t="n">
-        <v>121.1</v>
-      </c>
-      <c r="K11" s="4" t="n">
-        <v>58.89</v>
-      </c>
-      <c r="L11" s="4" t="n">
-        <v>125.64</v>
-      </c>
-      <c r="M11" s="8" t="n">
-        <v>18</v>
+      <c r="B11" s="4">
+        <f>'1 Raw Data'!B50-'1 Raw Data'!E50</f>
+        <v/>
+      </c>
+      <c r="C11" s="4">
+        <f>'1 Raw Data'!B50-'1 Raw Data'!C50-'1 Raw Data'!E50+'1 Raw Data'!G50</f>
+        <v/>
+      </c>
+      <c r="D11" s="4">
+        <f>'2 Average Balances'!B11+'2 Average Balances'!C11-'2 Average Balances'!D11</f>
+        <v/>
+      </c>
+      <c r="E11" s="4">
+        <f>D11/('1 Raw Data'!B25)*100</f>
+        <v/>
+      </c>
+      <c r="F11" s="4">
+        <f>B11/('1 Raw Data'!B25)</f>
+        <v/>
+      </c>
+      <c r="G11" s="4">
+        <f>'1 Raw Data'!B50/'1 Raw Data'!E50</f>
+        <v/>
+      </c>
+      <c r="H11" s="4">
+        <f>'2 Average Balances'!B11/('1 Raw Data'!B25/365)</f>
+        <v/>
+      </c>
+      <c r="I11" s="4">
+        <f>'1 Raw Data'!B25/'2 Average Balances'!B11</f>
+        <v/>
+      </c>
+      <c r="J11" s="4">
+        <f>'2 Average Balances'!C11/('2 Average Balances'!E11/365)</f>
+        <v/>
+      </c>
+      <c r="K11" s="4">
+        <f>'2 Average Balances'!D11/('2 Average Balances'!E11/365)</f>
+        <v/>
+      </c>
+      <c r="L11" s="4">
+        <f>H11+J11-K11</f>
+        <v/>
+      </c>
+      <c r="M11" s="8">
+        <f>'1 Raw Data'!I50/('1 Raw Data'!B25)*100</f>
+        <v/>
       </c>
       <c r="N11" s="4" t="inlineStr"/>
     </row>
@@ -6779,41 +6892,53 @@
           <t>Infineon</t>
         </is>
       </c>
-      <c r="B12" s="5" t="n">
-        <v>3400</v>
-      </c>
-      <c r="C12" s="5" t="n">
-        <v>1338</v>
-      </c>
-      <c r="D12" s="5" t="n">
-        <v>3918.5</v>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>46.71</v>
-      </c>
-      <c r="F12" s="5" t="n">
-        <v>0.41</v>
-      </c>
-      <c r="G12" s="5" t="n">
-        <v>1.74</v>
-      </c>
-      <c r="H12" s="8" t="n">
-        <v>70.97</v>
-      </c>
-      <c r="I12" s="5" t="n">
-        <v>5.14</v>
-      </c>
-      <c r="J12" s="5" t="n">
-        <v>243.74</v>
-      </c>
-      <c r="K12" s="8" t="n">
-        <v>74.18000000000001</v>
-      </c>
-      <c r="L12" s="8" t="n">
-        <v>240.53</v>
-      </c>
-      <c r="M12" s="5" t="n">
-        <v>28.14</v>
+      <c r="B12" s="5">
+        <f>'1 Raw Data'!B51-'1 Raw Data'!E51</f>
+        <v/>
+      </c>
+      <c r="C12" s="5">
+        <f>'1 Raw Data'!B51-'1 Raw Data'!C51-'1 Raw Data'!E51+'1 Raw Data'!G51</f>
+        <v/>
+      </c>
+      <c r="D12" s="5">
+        <f>'2 Average Balances'!B12+'2 Average Balances'!C12-'2 Average Balances'!D12</f>
+        <v/>
+      </c>
+      <c r="E12" s="5">
+        <f>D12/('1 Raw Data'!B26)*100</f>
+        <v/>
+      </c>
+      <c r="F12" s="5">
+        <f>B12/('1 Raw Data'!B26)</f>
+        <v/>
+      </c>
+      <c r="G12" s="5">
+        <f>'1 Raw Data'!B51/'1 Raw Data'!E51</f>
+        <v/>
+      </c>
+      <c r="H12" s="8">
+        <f>'2 Average Balances'!B12/('1 Raw Data'!B26/365)</f>
+        <v/>
+      </c>
+      <c r="I12" s="5">
+        <f>'1 Raw Data'!B26/'2 Average Balances'!B12</f>
+        <v/>
+      </c>
+      <c r="J12" s="5">
+        <f>'2 Average Balances'!C12/('2 Average Balances'!E12/365)</f>
+        <v/>
+      </c>
+      <c r="K12" s="8">
+        <f>'2 Average Balances'!D12/('2 Average Balances'!E12/365)</f>
+        <v/>
+      </c>
+      <c r="L12" s="8">
+        <f>H12+J12-K12</f>
+        <v/>
+      </c>
+      <c r="M12" s="5">
+        <f>'1 Raw Data'!I51/('1 Raw Data'!B26)*100</f>
+        <v/>
       </c>
       <c r="N12" s="11" t="inlineStr">
         <is>
@@ -6915,29 +7040,37 @@
           <t>NVIDIA</t>
         </is>
       </c>
-      <c r="B3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D3" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E3" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="F3" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="G3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="H3" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I3" s="4" t="n">
-        <v>5</v>
+      <c r="B3" s="4">
+        <f>RANK('3 Metrics'!H3,'3 Metrics'!$H$3:$H$12,1)</f>
+        <v/>
+      </c>
+      <c r="C3" s="4">
+        <f>RANK('3 Metrics'!I3,'3 Metrics'!$I$3:$I$12,0)</f>
+        <v/>
+      </c>
+      <c r="D3" s="4">
+        <f>RANK('3 Metrics'!J3,'3 Metrics'!$J$3:$J$12,1)</f>
+        <v/>
+      </c>
+      <c r="E3" s="4">
+        <f>RANK('3 Metrics'!K3,'3 Metrics'!$K$3:$K$12,0)</f>
+        <v/>
+      </c>
+      <c r="F3" s="4">
+        <f>RANK('3 Metrics'!L3,'3 Metrics'!$L$3:$L$12,1)</f>
+        <v/>
+      </c>
+      <c r="G3" s="4">
+        <f>RANK('3 Metrics'!M3,'3 Metrics'!$M$3:$M$12,0)</f>
+        <v/>
+      </c>
+      <c r="H3" s="4">
+        <f>RANK('3 Metrics'!E3,'3 Metrics'!$E$3:$E$12,1)</f>
+        <v/>
+      </c>
+      <c r="I3" s="4">
+        <f>RANK('3 Metrics'!F3,'3 Metrics'!$F$3:$F$12,1)</f>
+        <v/>
       </c>
       <c r="J3" s="4" t="inlineStr">
         <is>
@@ -6951,29 +7084,37 @@
           <t>AMD</t>
         </is>
       </c>
-      <c r="B4" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="C4" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="D4" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E4" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="F4" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="G4" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="H4" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="I4" s="5" t="n">
-        <v>6</v>
+      <c r="B4" s="5">
+        <f>RANK('3 Metrics'!H4,'3 Metrics'!$H$3:$H$12,1)</f>
+        <v/>
+      </c>
+      <c r="C4" s="5">
+        <f>RANK('3 Metrics'!I4,'3 Metrics'!$I$3:$I$12,0)</f>
+        <v/>
+      </c>
+      <c r="D4" s="5">
+        <f>RANK('3 Metrics'!J4,'3 Metrics'!$J$3:$J$12,1)</f>
+        <v/>
+      </c>
+      <c r="E4" s="5">
+        <f>RANK('3 Metrics'!K4,'3 Metrics'!$K$3:$K$12,0)</f>
+        <v/>
+      </c>
+      <c r="F4" s="5">
+        <f>RANK('3 Metrics'!L4,'3 Metrics'!$L$3:$L$12,1)</f>
+        <v/>
+      </c>
+      <c r="G4" s="12">
+        <f>RANK('3 Metrics'!M4,'3 Metrics'!$M$3:$M$12,0)</f>
+        <v/>
+      </c>
+      <c r="H4" s="5">
+        <f>RANK('3 Metrics'!E4,'3 Metrics'!$E$3:$E$12,1)</f>
+        <v/>
+      </c>
+      <c r="I4" s="5">
+        <f>RANK('3 Metrics'!F4,'3 Metrics'!$F$3:$F$12,1)</f>
+        <v/>
       </c>
       <c r="J4" s="5" t="inlineStr">
         <is>
@@ -6987,29 +7128,37 @@
           <t>Intel</t>
         </is>
       </c>
-      <c r="B5" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="C5" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="D5" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="E5" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="F5" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G5" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="H5" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="I5" s="13" t="n">
-        <v>1</v>
+      <c r="B5" s="13">
+        <f>RANK('3 Metrics'!H5,'3 Metrics'!$H$3:$H$12,1)</f>
+        <v/>
+      </c>
+      <c r="C5" s="13">
+        <f>RANK('3 Metrics'!I5,'3 Metrics'!$I$3:$I$12,0)</f>
+        <v/>
+      </c>
+      <c r="D5" s="4">
+        <f>RANK('3 Metrics'!J5,'3 Metrics'!$J$3:$J$12,1)</f>
+        <v/>
+      </c>
+      <c r="E5" s="4">
+        <f>RANK('3 Metrics'!K5,'3 Metrics'!$K$3:$K$12,0)</f>
+        <v/>
+      </c>
+      <c r="F5" s="4">
+        <f>RANK('3 Metrics'!L5,'3 Metrics'!$L$3:$L$12,1)</f>
+        <v/>
+      </c>
+      <c r="G5" s="4">
+        <f>RANK('3 Metrics'!M5,'3 Metrics'!$M$3:$M$12,0)</f>
+        <v/>
+      </c>
+      <c r="H5" s="4">
+        <f>RANK('3 Metrics'!E5,'3 Metrics'!$E$3:$E$12,1)</f>
+        <v/>
+      </c>
+      <c r="I5" s="13">
+        <f>RANK('3 Metrics'!F5,'3 Metrics'!$F$3:$F$12,1)</f>
+        <v/>
       </c>
       <c r="J5" s="4" t="inlineStr">
         <is>
@@ -7023,29 +7172,37 @@
           <t>TXN</t>
         </is>
       </c>
-      <c r="B6" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C6" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="D6" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="E6" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="F6" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="G6" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="H6" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="I6" s="5" t="n">
-        <v>7</v>
+      <c r="B6" s="5">
+        <f>RANK('3 Metrics'!H6,'3 Metrics'!$H$3:$H$12,1)</f>
+        <v/>
+      </c>
+      <c r="C6" s="5">
+        <f>RANK('3 Metrics'!I6,'3 Metrics'!$I$3:$I$12,0)</f>
+        <v/>
+      </c>
+      <c r="D6" s="5">
+        <f>RANK('3 Metrics'!J6,'3 Metrics'!$J$3:$J$12,1)</f>
+        <v/>
+      </c>
+      <c r="E6" s="12">
+        <f>RANK('3 Metrics'!K6,'3 Metrics'!$K$3:$K$12,0)</f>
+        <v/>
+      </c>
+      <c r="F6" s="5">
+        <f>RANK('3 Metrics'!L6,'3 Metrics'!$L$3:$L$12,1)</f>
+        <v/>
+      </c>
+      <c r="G6" s="5">
+        <f>RANK('3 Metrics'!M6,'3 Metrics'!$M$3:$M$12,0)</f>
+        <v/>
+      </c>
+      <c r="H6" s="5">
+        <f>RANK('3 Metrics'!E6,'3 Metrics'!$E$3:$E$12,1)</f>
+        <v/>
+      </c>
+      <c r="I6" s="5">
+        <f>RANK('3 Metrics'!F6,'3 Metrics'!$F$3:$F$12,1)</f>
+        <v/>
       </c>
       <c r="J6" s="5" t="inlineStr">
         <is>
@@ -7059,29 +7216,37 @@
           <t>Qualcomm</t>
         </is>
       </c>
-      <c r="B7" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="C7" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="D7" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="F7" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="H7" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="I7" s="4" t="n">
-        <v>4</v>
+      <c r="B7" s="4">
+        <f>RANK('3 Metrics'!H7,'3 Metrics'!$H$3:$H$12,1)</f>
+        <v/>
+      </c>
+      <c r="C7" s="4">
+        <f>RANK('3 Metrics'!I7,'3 Metrics'!$I$3:$I$12,0)</f>
+        <v/>
+      </c>
+      <c r="D7" s="13">
+        <f>RANK('3 Metrics'!J7,'3 Metrics'!$J$3:$J$12,1)</f>
+        <v/>
+      </c>
+      <c r="E7" s="13">
+        <f>RANK('3 Metrics'!K7,'3 Metrics'!$K$3:$K$12,0)</f>
+        <v/>
+      </c>
+      <c r="F7" s="13">
+        <f>RANK('3 Metrics'!L7,'3 Metrics'!$L$3:$L$12,1)</f>
+        <v/>
+      </c>
+      <c r="G7" s="4">
+        <f>RANK('3 Metrics'!M7,'3 Metrics'!$M$3:$M$12,0)</f>
+        <v/>
+      </c>
+      <c r="H7" s="13">
+        <f>RANK('3 Metrics'!E7,'3 Metrics'!$E$3:$E$12,1)</f>
+        <v/>
+      </c>
+      <c r="I7" s="4">
+        <f>RANK('3 Metrics'!F7,'3 Metrics'!$F$3:$F$12,1)</f>
+        <v/>
       </c>
       <c r="J7" s="4" t="inlineStr">
         <is>
@@ -7095,29 +7260,37 @@
           <t>NXP</t>
         </is>
       </c>
-      <c r="B8" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="C8" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="D8" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E8" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F8" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="G8" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="H8" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="I8" s="5" t="n">
-        <v>2</v>
+      <c r="B8" s="5">
+        <f>RANK('3 Metrics'!H8,'3 Metrics'!$H$3:$H$12,1)</f>
+        <v/>
+      </c>
+      <c r="C8" s="5">
+        <f>RANK('3 Metrics'!I8,'3 Metrics'!$I$3:$I$12,0)</f>
+        <v/>
+      </c>
+      <c r="D8" s="5">
+        <f>RANK('3 Metrics'!J8,'3 Metrics'!$J$3:$J$12,1)</f>
+        <v/>
+      </c>
+      <c r="E8" s="5">
+        <f>RANK('3 Metrics'!K8,'3 Metrics'!$K$3:$K$12,0)</f>
+        <v/>
+      </c>
+      <c r="F8" s="5">
+        <f>RANK('3 Metrics'!L8,'3 Metrics'!$L$3:$L$12,1)</f>
+        <v/>
+      </c>
+      <c r="G8" s="5">
+        <f>RANK('3 Metrics'!M8,'3 Metrics'!$M$3:$M$12,0)</f>
+        <v/>
+      </c>
+      <c r="H8" s="5">
+        <f>RANK('3 Metrics'!E8,'3 Metrics'!$E$3:$E$12,1)</f>
+        <v/>
+      </c>
+      <c r="I8" s="5">
+        <f>RANK('3 Metrics'!F8,'3 Metrics'!$F$3:$F$12,1)</f>
+        <v/>
       </c>
       <c r="J8" s="5" t="inlineStr">
         <is>
@@ -7131,29 +7304,37 @@
           <t>TSMC</t>
         </is>
       </c>
-      <c r="B9" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C9" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="E9" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="F9" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="G9" s="13" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="I9" s="12" t="n">
-        <v>10</v>
+      <c r="B9" s="4">
+        <f>RANK('3 Metrics'!H9,'3 Metrics'!$H$3:$H$12,1)</f>
+        <v/>
+      </c>
+      <c r="C9" s="4">
+        <f>RANK('3 Metrics'!I9,'3 Metrics'!$I$3:$I$12,0)</f>
+        <v/>
+      </c>
+      <c r="D9" s="4">
+        <f>RANK('3 Metrics'!J9,'3 Metrics'!$J$3:$J$12,1)</f>
+        <v/>
+      </c>
+      <c r="E9" s="4">
+        <f>RANK('3 Metrics'!K9,'3 Metrics'!$K$3:$K$12,0)</f>
+        <v/>
+      </c>
+      <c r="F9" s="4">
+        <f>RANK('3 Metrics'!L9,'3 Metrics'!$L$3:$L$12,1)</f>
+        <v/>
+      </c>
+      <c r="G9" s="13">
+        <f>RANK('3 Metrics'!M9,'3 Metrics'!$M$3:$M$12,0)</f>
+        <v/>
+      </c>
+      <c r="H9" s="4">
+        <f>RANK('3 Metrics'!E9,'3 Metrics'!$E$3:$E$12,1)</f>
+        <v/>
+      </c>
+      <c r="I9" s="12">
+        <f>RANK('3 Metrics'!F9,'3 Metrics'!$F$3:$F$12,1)</f>
+        <v/>
       </c>
       <c r="J9" s="4" t="inlineStr">
         <is>
@@ -7167,29 +7348,37 @@
           <t>Micron</t>
         </is>
       </c>
-      <c r="B10" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="C10" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="D10" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="E10" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="F10" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="G10" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="H10" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="I10" s="5" t="n">
-        <v>9</v>
+      <c r="B10" s="5">
+        <f>RANK('3 Metrics'!H10,'3 Metrics'!$H$3:$H$12,1)</f>
+        <v/>
+      </c>
+      <c r="C10" s="5">
+        <f>RANK('3 Metrics'!I10,'3 Metrics'!$I$3:$I$12,0)</f>
+        <v/>
+      </c>
+      <c r="D10" s="5">
+        <f>RANK('3 Metrics'!J10,'3 Metrics'!$J$3:$J$12,1)</f>
+        <v/>
+      </c>
+      <c r="E10" s="5">
+        <f>RANK('3 Metrics'!K10,'3 Metrics'!$K$3:$K$12,0)</f>
+        <v/>
+      </c>
+      <c r="F10" s="5">
+        <f>RANK('3 Metrics'!L10,'3 Metrics'!$L$3:$L$12,1)</f>
+        <v/>
+      </c>
+      <c r="G10" s="5">
+        <f>RANK('3 Metrics'!M10,'3 Metrics'!$M$3:$M$12,0)</f>
+        <v/>
+      </c>
+      <c r="H10" s="5">
+        <f>RANK('3 Metrics'!E10,'3 Metrics'!$E$3:$E$12,1)</f>
+        <v/>
+      </c>
+      <c r="I10" s="5">
+        <f>RANK('3 Metrics'!F10,'3 Metrics'!$F$3:$F$12,1)</f>
+        <v/>
       </c>
       <c r="J10" s="5" t="inlineStr">
         <is>
@@ -7203,29 +7392,37 @@
           <t>STM</t>
         </is>
       </c>
-      <c r="B11" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="D11" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E11" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="F11" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="G11" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="H11" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="I11" s="4" t="n">
-        <v>8</v>
+      <c r="B11" s="4">
+        <f>RANK('3 Metrics'!H11,'3 Metrics'!$H$3:$H$12,1)</f>
+        <v/>
+      </c>
+      <c r="C11" s="4">
+        <f>RANK('3 Metrics'!I11,'3 Metrics'!$I$3:$I$12,0)</f>
+        <v/>
+      </c>
+      <c r="D11" s="4">
+        <f>RANK('3 Metrics'!J11,'3 Metrics'!$J$3:$J$12,1)</f>
+        <v/>
+      </c>
+      <c r="E11" s="4">
+        <f>RANK('3 Metrics'!K11,'3 Metrics'!$K$3:$K$12,0)</f>
+        <v/>
+      </c>
+      <c r="F11" s="4">
+        <f>RANK('3 Metrics'!L11,'3 Metrics'!$L$3:$L$12,1)</f>
+        <v/>
+      </c>
+      <c r="G11" s="4">
+        <f>RANK('3 Metrics'!M11,'3 Metrics'!$M$3:$M$12,0)</f>
+        <v/>
+      </c>
+      <c r="H11" s="4">
+        <f>RANK('3 Metrics'!E11,'3 Metrics'!$E$3:$E$12,1)</f>
+        <v/>
+      </c>
+      <c r="I11" s="4">
+        <f>RANK('3 Metrics'!F11,'3 Metrics'!$F$3:$F$12,1)</f>
+        <v/>
       </c>
       <c r="J11" s="4" t="inlineStr">
         <is>
@@ -7239,29 +7436,37 @@
           <t>Infineon</t>
         </is>
       </c>
-      <c r="B12" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="C12" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="D12" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="E12" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="F12" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="G12" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="H12" s="12" t="n">
-        <v>10</v>
-      </c>
-      <c r="I12" s="5" t="n">
-        <v>9</v>
+      <c r="B12" s="12">
+        <f>RANK('3 Metrics'!H12,'3 Metrics'!$H$3:$H$12,1)</f>
+        <v/>
+      </c>
+      <c r="C12" s="12">
+        <f>RANK('3 Metrics'!I12,'3 Metrics'!$I$3:$I$12,0)</f>
+        <v/>
+      </c>
+      <c r="D12" s="12">
+        <f>RANK('3 Metrics'!J12,'3 Metrics'!$J$3:$J$12,1)</f>
+        <v/>
+      </c>
+      <c r="E12" s="5">
+        <f>RANK('3 Metrics'!K12,'3 Metrics'!$K$3:$K$12,0)</f>
+        <v/>
+      </c>
+      <c r="F12" s="12">
+        <f>RANK('3 Metrics'!L12,'3 Metrics'!$L$3:$L$12,1)</f>
+        <v/>
+      </c>
+      <c r="G12" s="5">
+        <f>RANK('3 Metrics'!M12,'3 Metrics'!$M$3:$M$12,0)</f>
+        <v/>
+      </c>
+      <c r="H12" s="12">
+        <f>RANK('3 Metrics'!E12,'3 Metrics'!$E$3:$E$12,1)</f>
+        <v/>
+      </c>
+      <c r="I12" s="5">
+        <f>RANK('3 Metrics'!F12,'3 Metrics'!$F$3:$F$12,1)</f>
+        <v/>
       </c>
       <c r="J12" s="5" t="inlineStr">
         <is>
@@ -7388,47 +7593,54 @@
           <t>NVIDIA</t>
         </is>
       </c>
-      <c r="B4" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" s="4" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="J4" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" s="14" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
+      <c r="B4" s="4">
+        <f>'4 Rankings'!B3</f>
+        <v/>
+      </c>
+      <c r="C4" s="4">
+        <f>'4 Rankings'!C3</f>
+        <v/>
+      </c>
+      <c r="D4" s="4">
+        <f>'4 Rankings'!F3</f>
+        <v/>
+      </c>
+      <c r="E4" s="4">
+        <f>'4 Rankings'!G3</f>
+        <v/>
+      </c>
+      <c r="F4" s="4">
+        <f>'4 Rankings'!H3</f>
+        <v/>
+      </c>
+      <c r="G4" s="4">
+        <f>(B4+C4+D4+E4+F4)/5</f>
+        <v/>
+      </c>
+      <c r="H4" s="4">
+        <f>RANK(G4,$G$4:$G$13,1)</f>
+        <v/>
+      </c>
+      <c r="I4" s="4">
+        <f>D4*0.30+F4*0.25+B4*0.15+C4*0.15+E4*0.15</f>
+        <v/>
+      </c>
+      <c r="J4" s="4">
+        <f>RANK(I4,$I$4:$I$13,1)</f>
+        <v/>
+      </c>
+      <c r="K4" s="14">
+        <f>IF(H4&lt;=3,"Q1",IF(H4&lt;=5,"Q2",IF(H4&lt;=8,"Q3","Q4")))</f>
+        <v/>
       </c>
       <c r="L4" s="13" t="inlineStr">
         <is>
           <t>🏆 Overall Best</t>
         </is>
       </c>
-      <c r="M4" s="4" t="inlineStr">
-        <is>
-          <t>Stable</t>
-        </is>
+      <c r="M4" s="4">
+        <f>IF(H4-J4=0,"Stable",IF(H4-J4&gt;0,"+"&amp;(H4-J4)&amp;" (V-B)",(H4-J4)&amp;" (V-B)"))</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -7437,43 +7649,50 @@
           <t>AMD</t>
         </is>
       </c>
-      <c r="B5" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>2</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="H5" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="I5" s="5" t="n">
-        <v>5.25</v>
-      </c>
-      <c r="J5" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="K5" s="15" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
+      <c r="B5" s="5">
+        <f>'4 Rankings'!B4</f>
+        <v/>
+      </c>
+      <c r="C5" s="5">
+        <f>'4 Rankings'!C4</f>
+        <v/>
+      </c>
+      <c r="D5" s="5">
+        <f>'4 Rankings'!F4</f>
+        <v/>
+      </c>
+      <c r="E5" s="5">
+        <f>'4 Rankings'!G4</f>
+        <v/>
+      </c>
+      <c r="F5" s="5">
+        <f>'4 Rankings'!H4</f>
+        <v/>
+      </c>
+      <c r="G5" s="5">
+        <f>(B5+C5+D5+E5+F5)/5</f>
+        <v/>
+      </c>
+      <c r="H5" s="5">
+        <f>RANK(G5,$G$4:$G$13,1)</f>
+        <v/>
+      </c>
+      <c r="I5" s="5">
+        <f>D5*0.30+F5*0.25+B5*0.15+C5*0.15+E5*0.15</f>
+        <v/>
+      </c>
+      <c r="J5" s="5">
+        <f>RANK(I5,$I$4:$I$13,1)</f>
+        <v/>
+      </c>
+      <c r="K5" s="15">
+        <f>IF(H5&lt;=3,"Q1",IF(H5&lt;=5,"Q2",IF(H5&lt;=8,"Q3","Q4")))</f>
+        <v/>
       </c>
       <c r="L5" s="5" t="inlineStr"/>
-      <c r="M5" s="5" t="inlineStr">
-        <is>
-          <t>+1 (V-B)</t>
-        </is>
+      <c r="M5" s="5">
+        <f>IF(H5-J5=0,"Stable",IF(H5-J5&gt;0,"+"&amp;(H5-J5)&amp;" (V-B)",(H5-J5)&amp;" (V-B)"))</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -7482,43 +7701,50 @@
           <t>Intel</t>
         </is>
       </c>
-      <c r="B6" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="I6" s="4" t="n">
-        <v>4.65</v>
-      </c>
-      <c r="J6" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="K6" s="14" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
+      <c r="B6" s="4">
+        <f>'4 Rankings'!B5</f>
+        <v/>
+      </c>
+      <c r="C6" s="4">
+        <f>'4 Rankings'!C5</f>
+        <v/>
+      </c>
+      <c r="D6" s="4">
+        <f>'4 Rankings'!F5</f>
+        <v/>
+      </c>
+      <c r="E6" s="4">
+        <f>'4 Rankings'!G5</f>
+        <v/>
+      </c>
+      <c r="F6" s="4">
+        <f>'4 Rankings'!H5</f>
+        <v/>
+      </c>
+      <c r="G6" s="4">
+        <f>(B6+C6+D6+E6+F6)/5</f>
+        <v/>
+      </c>
+      <c r="H6" s="4">
+        <f>RANK(G6,$G$4:$G$13,1)</f>
+        <v/>
+      </c>
+      <c r="I6" s="4">
+        <f>D6*0.30+F6*0.25+B6*0.15+C6*0.15+E6*0.15</f>
+        <v/>
+      </c>
+      <c r="J6" s="4">
+        <f>RANK(I6,$I$4:$I$13,1)</f>
+        <v/>
+      </c>
+      <c r="K6" s="14">
+        <f>IF(H6&lt;=3,"Q1",IF(H6&lt;=5,"Q2",IF(H6&lt;=8,"Q3","Q4")))</f>
+        <v/>
       </c>
       <c r="L6" s="4" t="inlineStr"/>
-      <c r="M6" s="4" t="inlineStr">
-        <is>
-          <t>Stable</t>
-        </is>
+      <c r="M6" s="4">
+        <f>IF(H6-J6=0,"Stable",IF(H6-J6&gt;0,"+"&amp;(H6-J6)&amp;" (V-B)",(H6-J6)&amp;" (V-B)"))</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -7527,43 +7753,50 @@
           <t>TXN</t>
         </is>
       </c>
-      <c r="B7" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>3</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="I7" s="5" t="n">
-        <v>6.35</v>
-      </c>
-      <c r="J7" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="K7" s="15" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
+      <c r="B7" s="5">
+        <f>'4 Rankings'!B6</f>
+        <v/>
+      </c>
+      <c r="C7" s="5">
+        <f>'4 Rankings'!C6</f>
+        <v/>
+      </c>
+      <c r="D7" s="5">
+        <f>'4 Rankings'!F6</f>
+        <v/>
+      </c>
+      <c r="E7" s="5">
+        <f>'4 Rankings'!G6</f>
+        <v/>
+      </c>
+      <c r="F7" s="5">
+        <f>'4 Rankings'!H6</f>
+        <v/>
+      </c>
+      <c r="G7" s="5">
+        <f>(B7+C7+D7+E7+F7)/5</f>
+        <v/>
+      </c>
+      <c r="H7" s="5">
+        <f>RANK(G7,$G$4:$G$13,1)</f>
+        <v/>
+      </c>
+      <c r="I7" s="5">
+        <f>D7*0.30+F7*0.25+B7*0.15+C7*0.15+E7*0.15</f>
+        <v/>
+      </c>
+      <c r="J7" s="5">
+        <f>RANK(I7,$I$4:$I$13,1)</f>
+        <v/>
+      </c>
+      <c r="K7" s="15">
+        <f>IF(H7&lt;=3,"Q1",IF(H7&lt;=5,"Q2",IF(H7&lt;=8,"Q3","Q4")))</f>
+        <v/>
       </c>
       <c r="L7" s="5" t="inlineStr"/>
-      <c r="M7" s="5" t="inlineStr">
-        <is>
-          <t>-1 (V-B)</t>
-        </is>
+      <c r="M7" s="5">
+        <f>IF(H7-J7=0,"Stable",IF(H7-J7&gt;0,"+"&amp;(H7-J7)&amp;" (V-B)",(H7-J7)&amp;" (V-B)"))</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -7572,47 +7805,54 @@
           <t>Qualcomm</t>
         </is>
       </c>
-      <c r="B8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>4</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>3.55</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="K8" s="16" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
+      <c r="B8" s="4">
+        <f>'4 Rankings'!B7</f>
+        <v/>
+      </c>
+      <c r="C8" s="4">
+        <f>'4 Rankings'!C7</f>
+        <v/>
+      </c>
+      <c r="D8" s="4">
+        <f>'4 Rankings'!F7</f>
+        <v/>
+      </c>
+      <c r="E8" s="4">
+        <f>'4 Rankings'!G7</f>
+        <v/>
+      </c>
+      <c r="F8" s="4">
+        <f>'4 Rankings'!H7</f>
+        <v/>
+      </c>
+      <c r="G8" s="4">
+        <f>(B8+C8+D8+E8+F8)/5</f>
+        <v/>
+      </c>
+      <c r="H8" s="4">
+        <f>RANK(G8,$G$4:$G$13,1)</f>
+        <v/>
+      </c>
+      <c r="I8" s="4">
+        <f>D8*0.30+F8*0.25+B8*0.15+C8*0.15+E8*0.15</f>
+        <v/>
+      </c>
+      <c r="J8" s="4">
+        <f>RANK(I8,$I$4:$I$13,1)</f>
+        <v/>
+      </c>
+      <c r="K8" s="16">
+        <f>IF(H8&lt;=3,"Q1",IF(H8&lt;=5,"Q2",IF(H8&lt;=8,"Q3","Q4")))</f>
+        <v/>
       </c>
       <c r="L8" s="13" t="inlineStr">
         <is>
           <t>Best CCC &amp; NWC%</t>
         </is>
       </c>
-      <c r="M8" s="4" t="inlineStr">
-        <is>
-          <t>+2 (V-B)</t>
-        </is>
+      <c r="M8" s="4">
+        <f>IF(H8-J8=0,"Stable",IF(H8-J8&gt;0,"+"&amp;(H8-J8)&amp;" (V-B)",(H8-J8)&amp;" (V-B)"))</f>
+        <v/>
       </c>
     </row>
     <row r="9">
@@ -7621,43 +7861,50 @@
           <t>NXP</t>
         </is>
       </c>
-      <c r="B9" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="C9" s="5" t="n">
-        <v>6</v>
-      </c>
-      <c r="D9" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="E9" s="5" t="n">
-        <v>7</v>
-      </c>
-      <c r="F9" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="G9" s="5" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="H9" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="I9" s="5" t="n">
-        <v>5.05</v>
-      </c>
-      <c r="J9" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="K9" s="16" t="inlineStr">
-        <is>
-          <t>Q2</t>
-        </is>
+      <c r="B9" s="5">
+        <f>'4 Rankings'!B8</f>
+        <v/>
+      </c>
+      <c r="C9" s="5">
+        <f>'4 Rankings'!C8</f>
+        <v/>
+      </c>
+      <c r="D9" s="5">
+        <f>'4 Rankings'!F8</f>
+        <v/>
+      </c>
+      <c r="E9" s="5">
+        <f>'4 Rankings'!G8</f>
+        <v/>
+      </c>
+      <c r="F9" s="5">
+        <f>'4 Rankings'!H8</f>
+        <v/>
+      </c>
+      <c r="G9" s="5">
+        <f>(B9+C9+D9+E9+F9)/5</f>
+        <v/>
+      </c>
+      <c r="H9" s="5">
+        <f>RANK(G9,$G$4:$G$13,1)</f>
+        <v/>
+      </c>
+      <c r="I9" s="5">
+        <f>D9*0.30+F9*0.25+B9*0.15+C9*0.15+E9*0.15</f>
+        <v/>
+      </c>
+      <c r="J9" s="5">
+        <f>RANK(I9,$I$4:$I$13,1)</f>
+        <v/>
+      </c>
+      <c r="K9" s="16">
+        <f>IF(H9&lt;=3,"Q1",IF(H9&lt;=5,"Q2",IF(H9&lt;=8,"Q3","Q4")))</f>
+        <v/>
       </c>
       <c r="L9" s="5" t="inlineStr"/>
-      <c r="M9" s="5" t="inlineStr">
-        <is>
-          <t>Stable</t>
-        </is>
+      <c r="M9" s="5">
+        <f>IF(H9-J9=0,"Stable",IF(H9-J9&gt;0,"+"&amp;(H9-J9)&amp;" (V-B)",(H9-J9)&amp;" (V-B)"))</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -7666,47 +7913,54 @@
           <t>TSMC</t>
         </is>
       </c>
-      <c r="B10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>6</v>
-      </c>
-      <c r="E10" s="4" t="n">
-        <v>1</v>
-      </c>
-      <c r="F10" s="4" t="n">
-        <v>5</v>
-      </c>
-      <c r="G10" s="4" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="H10" s="4" t="n">
-        <v>2</v>
-      </c>
-      <c r="I10" s="4" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="J10" s="4" t="n">
-        <v>3</v>
-      </c>
-      <c r="K10" s="14" t="inlineStr">
-        <is>
-          <t>Q1</t>
-        </is>
+      <c r="B10" s="4">
+        <f>'4 Rankings'!B9</f>
+        <v/>
+      </c>
+      <c r="C10" s="4">
+        <f>'4 Rankings'!C9</f>
+        <v/>
+      </c>
+      <c r="D10" s="4">
+        <f>'4 Rankings'!F9</f>
+        <v/>
+      </c>
+      <c r="E10" s="4">
+        <f>'4 Rankings'!G9</f>
+        <v/>
+      </c>
+      <c r="F10" s="4">
+        <f>'4 Rankings'!H9</f>
+        <v/>
+      </c>
+      <c r="G10" s="4">
+        <f>(B10+C10+D10+E10+F10)/5</f>
+        <v/>
+      </c>
+      <c r="H10" s="4">
+        <f>RANK(G10,$G$4:$G$13,1)</f>
+        <v/>
+      </c>
+      <c r="I10" s="4">
+        <f>D10*0.30+F10*0.25+B10*0.15+C10*0.15+E10*0.15</f>
+        <v/>
+      </c>
+      <c r="J10" s="4">
+        <f>RANK(I10,$I$4:$I$13,1)</f>
+        <v/>
+      </c>
+      <c r="K10" s="14">
+        <f>IF(H10&lt;=3,"Q1",IF(H10&lt;=5,"Q2",IF(H10&lt;=8,"Q3","Q4")))</f>
+        <v/>
       </c>
       <c r="L10" s="13" t="inlineStr">
         <is>
           <t>Best CRR</t>
         </is>
       </c>
-      <c r="M10" s="4" t="inlineStr">
-        <is>
-          <t>-1 (V-B)</t>
-        </is>
+      <c r="M10" s="4">
+        <f>IF(H10-J10=0,"Stable",IF(H10-J10&gt;0,"+"&amp;(H10-J10)&amp;" (V-B)",(H10-J10)&amp;" (V-B)"))</f>
+        <v/>
       </c>
     </row>
     <row r="11">
@@ -7715,43 +7969,50 @@
           <t>Micron</t>
         </is>
       </c>
-      <c r="B11" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="C11" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="D11" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="E11" s="5" t="n">
-        <v>4</v>
-      </c>
-      <c r="F11" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="G11" s="5" t="n">
-        <v>6.2</v>
-      </c>
-      <c r="H11" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="I11" s="5" t="n">
-        <v>6.75</v>
-      </c>
-      <c r="J11" s="5" t="n">
-        <v>8</v>
-      </c>
-      <c r="K11" s="15" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
+      <c r="B11" s="5">
+        <f>'4 Rankings'!B10</f>
+        <v/>
+      </c>
+      <c r="C11" s="5">
+        <f>'4 Rankings'!C10</f>
+        <v/>
+      </c>
+      <c r="D11" s="5">
+        <f>'4 Rankings'!F10</f>
+        <v/>
+      </c>
+      <c r="E11" s="5">
+        <f>'4 Rankings'!G10</f>
+        <v/>
+      </c>
+      <c r="F11" s="5">
+        <f>'4 Rankings'!H10</f>
+        <v/>
+      </c>
+      <c r="G11" s="5">
+        <f>(B11+C11+D11+E11+F11)/5</f>
+        <v/>
+      </c>
+      <c r="H11" s="5">
+        <f>RANK(G11,$G$4:$G$13,1)</f>
+        <v/>
+      </c>
+      <c r="I11" s="5">
+        <f>D11*0.30+F11*0.25+B11*0.15+C11*0.15+E11*0.15</f>
+        <v/>
+      </c>
+      <c r="J11" s="5">
+        <f>RANK(I11,$I$4:$I$13,1)</f>
+        <v/>
+      </c>
+      <c r="K11" s="15">
+        <f>IF(H11&lt;=3,"Q1",IF(H11&lt;=5,"Q2",IF(H11&lt;=8,"Q3","Q4")))</f>
+        <v/>
       </c>
       <c r="L11" s="5" t="inlineStr"/>
-      <c r="M11" s="5" t="inlineStr">
-        <is>
-          <t>Stable</t>
-        </is>
+      <c r="M11" s="5">
+        <f>IF(H11-J11=0,"Stable",IF(H11-J11&gt;0,"+"&amp;(H11-J11)&amp;" (V-B)",(H11-J11)&amp;" (V-B)"))</f>
+        <v/>
       </c>
     </row>
     <row r="12">
@@ -7760,43 +8021,50 @@
           <t>STM</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="C12" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="D12" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="E12" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="F12" s="4" t="n">
-        <v>7</v>
-      </c>
-      <c r="G12" s="4" t="n">
-        <v>8</v>
-      </c>
-      <c r="H12" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="I12" s="4" t="n">
-        <v>7.75</v>
-      </c>
-      <c r="J12" s="4" t="n">
-        <v>9</v>
-      </c>
-      <c r="K12" s="8" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
+      <c r="B12" s="4">
+        <f>'4 Rankings'!B11</f>
+        <v/>
+      </c>
+      <c r="C12" s="4">
+        <f>'4 Rankings'!C11</f>
+        <v/>
+      </c>
+      <c r="D12" s="4">
+        <f>'4 Rankings'!F11</f>
+        <v/>
+      </c>
+      <c r="E12" s="4">
+        <f>'4 Rankings'!G11</f>
+        <v/>
+      </c>
+      <c r="F12" s="4">
+        <f>'4 Rankings'!H11</f>
+        <v/>
+      </c>
+      <c r="G12" s="4">
+        <f>(B12+C12+D12+E12+F12)/5</f>
+        <v/>
+      </c>
+      <c r="H12" s="4">
+        <f>RANK(G12,$G$4:$G$13,1)</f>
+        <v/>
+      </c>
+      <c r="I12" s="4">
+        <f>D12*0.30+F12*0.25+B12*0.15+C12*0.15+E12*0.15</f>
+        <v/>
+      </c>
+      <c r="J12" s="4">
+        <f>RANK(I12,$I$4:$I$13,1)</f>
+        <v/>
+      </c>
+      <c r="K12" s="8">
+        <f>IF(H12&lt;=3,"Q1",IF(H12&lt;=5,"Q2",IF(H12&lt;=8,"Q3","Q4")))</f>
+        <v/>
       </c>
       <c r="L12" s="4" t="inlineStr"/>
-      <c r="M12" s="4" t="inlineStr">
-        <is>
-          <t>Stable</t>
-        </is>
+      <c r="M12" s="4">
+        <f>IF(H12-J12=0,"Stable",IF(H12-J12&gt;0,"+"&amp;(H12-J12)&amp;" (V-B)",(H12-J12)&amp;" (V-B)"))</f>
+        <v/>
       </c>
     </row>
     <row r="13">
@@ -7805,43 +8073,50 @@
           <t>Infineon</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="C13" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="D13" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="E13" s="5" t="n">
-        <v>5</v>
-      </c>
-      <c r="F13" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="G13" s="5" t="n">
-        <v>9</v>
-      </c>
-      <c r="H13" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="I13" s="5" t="n">
-        <v>9.25</v>
-      </c>
-      <c r="J13" s="5" t="n">
-        <v>10</v>
-      </c>
-      <c r="K13" s="8" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
+      <c r="B13" s="5">
+        <f>'4 Rankings'!B12</f>
+        <v/>
+      </c>
+      <c r="C13" s="5">
+        <f>'4 Rankings'!C12</f>
+        <v/>
+      </c>
+      <c r="D13" s="5">
+        <f>'4 Rankings'!F12</f>
+        <v/>
+      </c>
+      <c r="E13" s="5">
+        <f>'4 Rankings'!G12</f>
+        <v/>
+      </c>
+      <c r="F13" s="5">
+        <f>'4 Rankings'!H12</f>
+        <v/>
+      </c>
+      <c r="G13" s="5">
+        <f>(B13+C13+D13+E13+F13)/5</f>
+        <v/>
+      </c>
+      <c r="H13" s="5">
+        <f>RANK(G13,$G$4:$G$13,1)</f>
+        <v/>
+      </c>
+      <c r="I13" s="5">
+        <f>D13*0.30+F13*0.25+B13*0.15+C13*0.15+E13*0.15</f>
+        <v/>
+      </c>
+      <c r="J13" s="5">
+        <f>RANK(I13,$I$4:$I$13,1)</f>
+        <v/>
+      </c>
+      <c r="K13" s="8">
+        <f>IF(H13&lt;=3,"Q1",IF(H13&lt;=5,"Q2",IF(H13&lt;=8,"Q3","Q4")))</f>
+        <v/>
       </c>
       <c r="L13" s="5" t="inlineStr"/>
-      <c r="M13" s="5" t="inlineStr">
-        <is>
-          <t>Stable</t>
-        </is>
+      <c r="M13" s="5">
+        <f>IF(H13-J13=0,"Stable",IF(H13-J13&gt;0,"+"&amp;(H13-J13)&amp;" (V-B)",(H13-J13)&amp;" (V-B)"))</f>
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -7881,10 +8156,9 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Best-in-Class: DSO = Intel 35.50d | DIO = Qualcomm 54.28d | DPO = Qualcomm 88.44d</t>
-        </is>
+      <c r="A2" s="2">
+        <f>"Best-in-Class: DSO = "&amp;INDEX('3 Metrics'!$A$3:$A$12,MATCH(MIN('3 Metrics'!$H$3:$H$12),'3 Metrics'!$H$3:$H$12,0))&amp;" "&amp;TEXT(MIN('3 Metrics'!$H$3:$H$12),"0.00")&amp;"d | DIO = "&amp;INDEX('3 Metrics'!$A$3:$A$12,MATCH(MIN('3 Metrics'!$J$3:$J$12),'3 Metrics'!$J$3:$J$12,0))&amp;" "&amp;TEXT(MIN('3 Metrics'!$J$3:$J$12),"0.00")&amp;"d | DPO = "&amp;INDEX('3 Metrics'!$A$3:$A$12,MATCH(MAX('3 Metrics'!$K$3:$K$12),'3 Metrics'!$K$3:$K$12,0))&amp;" "&amp;TEXT(MAX('3 Metrics'!$K$3:$K$12),"0.00")&amp;"d"</f>
+        <v/>
       </c>
     </row>
     <row r="3">
@@ -7940,31 +8214,37 @@
           <t>TXN</t>
         </is>
       </c>
-      <c r="B4" s="16" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="C4" s="4" t="n">
-        <v>310</v>
-      </c>
-      <c r="D4" s="4" t="n">
-        <v>7.24</v>
-      </c>
-      <c r="E4" s="4" t="n">
-        <v>2867</v>
-      </c>
-      <c r="F4" s="4" t="n">
-        <v>164.42</v>
-      </c>
-      <c r="G4" s="4" t="n">
-        <v>1152</v>
-      </c>
-      <c r="H4" s="4" t="n">
-        <v>66.06999999999999</v>
-      </c>
-      <c r="I4" s="17" t="n">
-        <v>4329</v>
+      <c r="B4" s="16">
+        <f>'5 Scoring Model'!K7</f>
+        <v/>
+      </c>
+      <c r="C4" s="4">
+        <f>D4*('1 Raw Data'!B20/365)</f>
+        <v/>
+      </c>
+      <c r="D4" s="4">
+        <f>'3 Metrics'!H6-MIN('3 Metrics'!$H$3:$H$12)</f>
+        <v/>
+      </c>
+      <c r="E4" s="4">
+        <f>F4*('2 Average Balances'!E6/365)</f>
+        <v/>
+      </c>
+      <c r="F4" s="4">
+        <f>'3 Metrics'!J6-MIN('3 Metrics'!$J$3:$J$12)</f>
+        <v/>
+      </c>
+      <c r="G4" s="4">
+        <f>H4*('2 Average Balances'!E6/365)</f>
+        <v/>
+      </c>
+      <c r="H4" s="4">
+        <f>MAX('3 Metrics'!$K$3:$K$12)-'3 Metrics'!K6</f>
+        <v/>
+      </c>
+      <c r="I4" s="17">
+        <f>C4+E4+G4</f>
+        <v/>
       </c>
     </row>
     <row r="5">
@@ -7973,31 +8253,37 @@
           <t>AMD</t>
         </is>
       </c>
-      <c r="B5" s="16" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="C5" s="5" t="n">
-        <v>1773</v>
-      </c>
-      <c r="D5" s="5" t="n">
-        <v>25.09</v>
-      </c>
-      <c r="E5" s="5" t="n">
-        <v>207</v>
-      </c>
-      <c r="F5" s="5" t="n">
-        <v>6.31</v>
-      </c>
-      <c r="G5" s="5" t="n">
-        <v>1449</v>
-      </c>
-      <c r="H5" s="5" t="n">
-        <v>44.15</v>
-      </c>
-      <c r="I5" s="17" t="n">
-        <v>3429</v>
+      <c r="B5" s="16">
+        <f>'5 Scoring Model'!K5</f>
+        <v/>
+      </c>
+      <c r="C5" s="5">
+        <f>D5*('1 Raw Data'!B18/365)</f>
+        <v/>
+      </c>
+      <c r="D5" s="5">
+        <f>'3 Metrics'!H4-MIN('3 Metrics'!$H$3:$H$12)</f>
+        <v/>
+      </c>
+      <c r="E5" s="5">
+        <f>F5*('2 Average Balances'!E4/365)</f>
+        <v/>
+      </c>
+      <c r="F5" s="5">
+        <f>'3 Metrics'!J4-MIN('3 Metrics'!$J$3:$J$12)</f>
+        <v/>
+      </c>
+      <c r="G5" s="5">
+        <f>H5*('2 Average Balances'!E4/365)</f>
+        <v/>
+      </c>
+      <c r="H5" s="5">
+        <f>MAX('3 Metrics'!$K$3:$K$12)-'3 Metrics'!K4</f>
+        <v/>
+      </c>
+      <c r="I5" s="17">
+        <f>C5+E5+G5</f>
+        <v/>
       </c>
     </row>
     <row r="6">
@@ -8006,31 +8292,37 @@
           <t>Micron</t>
         </is>
       </c>
-      <c r="B6" s="16" t="inlineStr">
-        <is>
-          <t>Q3</t>
-        </is>
-      </c>
-      <c r="C6" s="4" t="n">
-        <v>587</v>
-      </c>
-      <c r="D6" s="4" t="n">
-        <v>8.539999999999999</v>
-      </c>
-      <c r="E6" s="4" t="n">
-        <v>5615</v>
-      </c>
-      <c r="F6" s="4" t="n">
-        <v>111.15</v>
-      </c>
-      <c r="G6" s="4" t="n">
-        <v>2512</v>
-      </c>
-      <c r="H6" s="4" t="n">
-        <v>49.71</v>
-      </c>
-      <c r="I6" s="17" t="n">
-        <v>8714</v>
+      <c r="B6" s="16">
+        <f>'5 Scoring Model'!K11</f>
+        <v/>
+      </c>
+      <c r="C6" s="4">
+        <f>D6*('1 Raw Data'!B24/365)</f>
+        <v/>
+      </c>
+      <c r="D6" s="4">
+        <f>'3 Metrics'!H10-MIN('3 Metrics'!$H$3:$H$12)</f>
+        <v/>
+      </c>
+      <c r="E6" s="4">
+        <f>F6*('2 Average Balances'!E10/365)</f>
+        <v/>
+      </c>
+      <c r="F6" s="4">
+        <f>'3 Metrics'!J10-MIN('3 Metrics'!$J$3:$J$12)</f>
+        <v/>
+      </c>
+      <c r="G6" s="4">
+        <f>H6*('2 Average Balances'!E10/365)</f>
+        <v/>
+      </c>
+      <c r="H6" s="4">
+        <f>MAX('3 Metrics'!$K$3:$K$12)-'3 Metrics'!K10</f>
+        <v/>
+      </c>
+      <c r="I6" s="17">
+        <f>C6+E6+G6</f>
+        <v/>
       </c>
     </row>
     <row r="7">
@@ -8039,31 +8331,37 @@
           <t>STM</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="C7" s="5" t="n">
-        <v>1016</v>
-      </c>
-      <c r="D7" s="5" t="n">
-        <v>27.93</v>
-      </c>
-      <c r="E7" s="5" t="n">
-        <v>1601</v>
-      </c>
-      <c r="F7" s="5" t="n">
-        <v>66.81999999999999</v>
-      </c>
-      <c r="G7" s="5" t="n">
-        <v>708</v>
-      </c>
-      <c r="H7" s="5" t="n">
-        <v>29.55</v>
-      </c>
-      <c r="I7" s="17" t="n">
-        <v>3325</v>
+      <c r="B7" s="8">
+        <f>'5 Scoring Model'!K12</f>
+        <v/>
+      </c>
+      <c r="C7" s="5">
+        <f>D7*('1 Raw Data'!B25/365)</f>
+        <v/>
+      </c>
+      <c r="D7" s="5">
+        <f>'3 Metrics'!H11-MIN('3 Metrics'!$H$3:$H$12)</f>
+        <v/>
+      </c>
+      <c r="E7" s="5">
+        <f>F7*('2 Average Balances'!E11/365)</f>
+        <v/>
+      </c>
+      <c r="F7" s="5">
+        <f>'3 Metrics'!J11-MIN('3 Metrics'!$J$3:$J$12)</f>
+        <v/>
+      </c>
+      <c r="G7" s="5">
+        <f>H7*('2 Average Balances'!E11/365)</f>
+        <v/>
+      </c>
+      <c r="H7" s="5">
+        <f>MAX('3 Metrics'!$K$3:$K$12)-'3 Metrics'!K11</f>
+        <v/>
+      </c>
+      <c r="I7" s="17">
+        <f>C7+E7+G7</f>
+        <v/>
       </c>
     </row>
     <row r="8">
@@ -8072,31 +8370,37 @@
           <t>Infineon</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
-        <is>
-          <t>Q4</t>
-        </is>
-      </c>
-      <c r="C8" s="4" t="n">
-        <v>815</v>
-      </c>
-      <c r="D8" s="4" t="n">
-        <v>35.47</v>
-      </c>
-      <c r="E8" s="4" t="n">
-        <v>2557</v>
-      </c>
-      <c r="F8" s="4" t="n">
-        <v>189.46</v>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>192</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>14.26</v>
-      </c>
-      <c r="I8" s="17" t="n">
-        <v>3564</v>
+      <c r="B8" s="8">
+        <f>'5 Scoring Model'!K13</f>
+        <v/>
+      </c>
+      <c r="C8" s="4">
+        <f>D8*('1 Raw Data'!B26/365)</f>
+        <v/>
+      </c>
+      <c r="D8" s="4">
+        <f>'3 Metrics'!H12-MIN('3 Metrics'!$H$3:$H$12)</f>
+        <v/>
+      </c>
+      <c r="E8" s="4">
+        <f>F8*('2 Average Balances'!E12/365)</f>
+        <v/>
+      </c>
+      <c r="F8" s="4">
+        <f>'3 Metrics'!J12-MIN('3 Metrics'!$J$3:$J$12)</f>
+        <v/>
+      </c>
+      <c r="G8" s="4">
+        <f>H8*('2 Average Balances'!E12/365)</f>
+        <v/>
+      </c>
+      <c r="H8" s="4">
+        <f>MAX('3 Metrics'!$K$3:$K$12)-'3 Metrics'!K12</f>
+        <v/>
+      </c>
+      <c r="I8" s="17">
+        <f>C8+E8+G8</f>
+        <v/>
       </c>
     </row>
     <row r="10">
@@ -9067,25 +9371,21 @@
           <t>DSO</t>
         </is>
       </c>
-      <c r="B3" s="13" t="inlineStr">
-        <is>
-          <t>Intel</t>
-        </is>
-      </c>
-      <c r="C3" s="4" t="inlineStr">
-        <is>
-          <t>35.50 days</t>
-        </is>
-      </c>
-      <c r="D3" s="12" t="inlineStr">
-        <is>
-          <t>Infineon</t>
-        </is>
-      </c>
-      <c r="E3" s="25" t="inlineStr">
-        <is>
-          <t>70.97 days</t>
-        </is>
+      <c r="B3" s="13">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MIN('3 Metrics'!$H$3:$H$12),'3 Metrics'!$H$3:$H$12,0))</f>
+        <v/>
+      </c>
+      <c r="C3" s="4">
+        <f>TEXT(MIN('3 Metrics'!$H$3:$H$12),"0.00")&amp;" days"</f>
+        <v/>
+      </c>
+      <c r="D3" s="12">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MAX('3 Metrics'!$H$3:$H$12),'3 Metrics'!$H$3:$H$12,0))</f>
+        <v/>
+      </c>
+      <c r="E3" s="25">
+        <f>TEXT(MAX('3 Metrics'!$H$3:$H$12),"0.00")&amp;" days"</f>
+        <v/>
       </c>
       <c r="F3" s="25" t="inlineStr">
         <is>
@@ -9099,25 +9399,21 @@
           <t>AR Turns</t>
         </is>
       </c>
-      <c r="B4" s="13" t="inlineStr">
-        <is>
-          <t>Intel</t>
-        </is>
-      </c>
-      <c r="C4" s="5" t="inlineStr">
-        <is>
-          <t>10.28×</t>
-        </is>
-      </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>Infineon</t>
-        </is>
-      </c>
-      <c r="E4" s="26" t="inlineStr">
-        <is>
-          <t>5.14×</t>
-        </is>
+      <c r="B4" s="13">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MAX('3 Metrics'!$I$3:$I$12),'3 Metrics'!$I$3:$I$12,0))</f>
+        <v/>
+      </c>
+      <c r="C4" s="5">
+        <f>TEXT(MAX('3 Metrics'!$I$3:$I$12),"0.00")&amp;"×"</f>
+        <v/>
+      </c>
+      <c r="D4" s="12">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MIN('3 Metrics'!$I$3:$I$12),'3 Metrics'!$I$3:$I$12,0))</f>
+        <v/>
+      </c>
+      <c r="E4" s="26">
+        <f>TEXT(MIN('3 Metrics'!$I$3:$I$12),"0.00")&amp;"×"</f>
+        <v/>
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
@@ -9131,25 +9427,21 @@
           <t>DIO</t>
         </is>
       </c>
-      <c r="B5" s="13" t="inlineStr">
-        <is>
-          <t>Qualcomm</t>
-        </is>
-      </c>
-      <c r="C5" s="4" t="inlineStr">
-        <is>
-          <t>54.28 days</t>
-        </is>
-      </c>
-      <c r="D5" s="12" t="inlineStr">
-        <is>
-          <t>Infineon</t>
-        </is>
-      </c>
-      <c r="E5" s="25" t="inlineStr">
-        <is>
-          <t>243.74 days</t>
-        </is>
+      <c r="B5" s="13">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MIN('3 Metrics'!$J$3:$J$12),'3 Metrics'!$J$3:$J$12,0))</f>
+        <v/>
+      </c>
+      <c r="C5" s="4">
+        <f>TEXT(MIN('3 Metrics'!$J$3:$J$12),"0.00")&amp;" days"</f>
+        <v/>
+      </c>
+      <c r="D5" s="12">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MAX('3 Metrics'!$J$3:$J$12),'3 Metrics'!$J$3:$J$12,0))</f>
+        <v/>
+      </c>
+      <c r="E5" s="25">
+        <f>TEXT(MAX('3 Metrics'!$J$3:$J$12),"0.00")&amp;" days"</f>
+        <v/>
       </c>
       <c r="F5" s="25" t="inlineStr">
         <is>
@@ -9163,25 +9455,21 @@
           <t>DPO</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
-        <is>
-          <t>Qualcomm</t>
-        </is>
-      </c>
-      <c r="C6" s="5" t="inlineStr">
-        <is>
-          <t>88.44 days</t>
-        </is>
-      </c>
-      <c r="D6" s="12" t="inlineStr">
-        <is>
-          <t>TXN</t>
-        </is>
-      </c>
-      <c r="E6" s="26" t="inlineStr">
-        <is>
-          <t>22.37 days</t>
-        </is>
+      <c r="B6" s="13">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MAX('3 Metrics'!$K$3:$K$12),'3 Metrics'!$K$3:$K$12,0))</f>
+        <v/>
+      </c>
+      <c r="C6" s="5">
+        <f>TEXT(MAX('3 Metrics'!$K$3:$K$12),"0.00")&amp;" days"</f>
+        <v/>
+      </c>
+      <c r="D6" s="12">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MIN('3 Metrics'!$K$3:$K$12),'3 Metrics'!$K$3:$K$12,0))</f>
+        <v/>
+      </c>
+      <c r="E6" s="26">
+        <f>TEXT(MIN('3 Metrics'!$K$3:$K$12),"0.00")&amp;" days"</f>
+        <v/>
       </c>
       <c r="F6" s="26" t="inlineStr">
         <is>
@@ -9195,25 +9483,21 @@
           <t>CCC</t>
         </is>
       </c>
-      <c r="B7" s="13" t="inlineStr">
-        <is>
-          <t>Qualcomm</t>
-        </is>
-      </c>
-      <c r="C7" s="4" t="inlineStr">
-        <is>
-          <t>22.11 days</t>
-        </is>
-      </c>
-      <c r="D7" s="12" t="inlineStr">
-        <is>
-          <t>Infineon</t>
-        </is>
-      </c>
-      <c r="E7" s="25" t="inlineStr">
-        <is>
-          <t>240.53 days</t>
-        </is>
+      <c r="B7" s="13">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MIN('3 Metrics'!$L$3:$L$12),'3 Metrics'!$L$3:$L$12,0))</f>
+        <v/>
+      </c>
+      <c r="C7" s="4">
+        <f>TEXT(MIN('3 Metrics'!$L$3:$L$12),"0.00")&amp;" days"</f>
+        <v/>
+      </c>
+      <c r="D7" s="12">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MAX('3 Metrics'!$L$3:$L$12),'3 Metrics'!$L$3:$L$12,0))</f>
+        <v/>
+      </c>
+      <c r="E7" s="25">
+        <f>TEXT(MAX('3 Metrics'!$L$3:$L$12),"0.00")&amp;" days"</f>
+        <v/>
       </c>
       <c r="F7" s="25" t="inlineStr">
         <is>
@@ -9227,25 +9511,21 @@
           <t>CRR</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
-        <is>
-          <t>TSMC</t>
-        </is>
-      </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>62.19%</t>
-        </is>
-      </c>
-      <c r="D8" s="12" t="inlineStr">
-        <is>
-          <t>AMD</t>
-        </is>
-      </c>
-      <c r="E8" s="26" t="inlineStr">
-        <is>
-          <t>10.46%</t>
-        </is>
+      <c r="B8" s="13">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MAX('3 Metrics'!$M$3:$M$12),'3 Metrics'!$M$3:$M$12,0))</f>
+        <v/>
+      </c>
+      <c r="C8" s="5">
+        <f>TEXT(MAX('3 Metrics'!$M$3:$M$12),"0.00")&amp;"%"</f>
+        <v/>
+      </c>
+      <c r="D8" s="12">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MIN('3 Metrics'!$M$3:$M$12),'3 Metrics'!$M$3:$M$12,0))</f>
+        <v/>
+      </c>
+      <c r="E8" s="26">
+        <f>TEXT(MIN('3 Metrics'!$M$3:$M$12),"0.00")&amp;"%"</f>
+        <v/>
       </c>
       <c r="F8" s="26" t="inlineStr">
         <is>
@@ -9259,25 +9539,21 @@
           <t>Operating NWC (absolute)</t>
         </is>
       </c>
-      <c r="B9" s="13" t="inlineStr">
-        <is>
-          <t>NXP</t>
-        </is>
-      </c>
-      <c r="C9" s="4" t="inlineStr">
-        <is>
-          <t>$2,450M</t>
-        </is>
-      </c>
-      <c r="D9" s="12" t="inlineStr">
-        <is>
-          <t>TSMC</t>
-        </is>
-      </c>
-      <c r="E9" s="25" t="inlineStr">
-        <is>
-          <t>$17,853M</t>
-        </is>
+      <c r="B9" s="13">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MIN('3 Metrics'!$D$3:$D$12),'3 Metrics'!$D$3:$D$12,0))</f>
+        <v/>
+      </c>
+      <c r="C9" s="4">
+        <f>"$"&amp;TEXT(MIN('3 Metrics'!$D$3:$D$12),"#,##0")&amp;"M"</f>
+        <v/>
+      </c>
+      <c r="D9" s="12">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MAX('3 Metrics'!$D$3:$D$12),'3 Metrics'!$D$3:$D$12,0))</f>
+        <v/>
+      </c>
+      <c r="E9" s="25">
+        <f>"$"&amp;TEXT(MAX('3 Metrics'!$D$3:$D$12),"#,##0")&amp;"M"</f>
+        <v/>
       </c>
       <c r="F9" s="25" t="inlineStr">
         <is>
@@ -9291,25 +9567,21 @@
           <t>NWC%</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
-        <is>
-          <t>Qualcomm</t>
-        </is>
-      </c>
-      <c r="C10" s="5" t="inlineStr">
-        <is>
-          <t>11.47%</t>
-        </is>
-      </c>
-      <c r="D10" s="12" t="inlineStr">
-        <is>
-          <t>Infineon</t>
-        </is>
-      </c>
-      <c r="E10" s="26" t="inlineStr">
-        <is>
-          <t>46.71%</t>
-        </is>
+      <c r="B10" s="13">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MIN('3 Metrics'!$E$3:$E$12),'3 Metrics'!$E$3:$E$12,0))</f>
+        <v/>
+      </c>
+      <c r="C10" s="5">
+        <f>TEXT(MIN('3 Metrics'!$E$3:$E$12),"0.00")&amp;"%"</f>
+        <v/>
+      </c>
+      <c r="D10" s="12">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MAX('3 Metrics'!$E$3:$E$12),'3 Metrics'!$E$3:$E$12,0))</f>
+        <v/>
+      </c>
+      <c r="E10" s="26">
+        <f>TEXT(MAX('3 Metrics'!$E$3:$E$12),"0.00")&amp;"%"</f>
+        <v/>
       </c>
       <c r="F10" s="26" t="inlineStr">
         <is>
@@ -9323,25 +9595,21 @@
           <t>WC Intensity</t>
         </is>
       </c>
-      <c r="B11" s="13" t="inlineStr">
-        <is>
-          <t>Intel</t>
-        </is>
-      </c>
-      <c r="C11" s="4" t="inlineStr">
-        <is>
-          <t>0.13</t>
-        </is>
-      </c>
-      <c r="D11" s="12" t="inlineStr">
-        <is>
-          <t>TSMC</t>
-        </is>
-      </c>
-      <c r="E11" s="25" t="inlineStr">
-        <is>
-          <t>0.49</t>
-        </is>
+      <c r="B11" s="13">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MIN('3 Metrics'!$F$3:$F$12),'3 Metrics'!$F$3:$F$12,0))</f>
+        <v/>
+      </c>
+      <c r="C11" s="4">
+        <f>TEXT(MIN('3 Metrics'!$F$3:$F$12),"0.00")&amp;""</f>
+        <v/>
+      </c>
+      <c r="D11" s="12">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MAX('3 Metrics'!$F$3:$F$12),'3 Metrics'!$F$3:$F$12,0))</f>
+        <v/>
+      </c>
+      <c r="E11" s="25">
+        <f>TEXT(MAX('3 Metrics'!$F$3:$F$12),"0.00")&amp;""</f>
+        <v/>
       </c>
       <c r="F11" s="25" t="inlineStr">
         <is>
@@ -9355,25 +9623,21 @@
           <t>Current Ratio</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
-        <is>
-          <t>NVIDIA (highest)</t>
-        </is>
-      </c>
-      <c r="C12" s="5" t="inlineStr">
-        <is>
-          <t>2.79</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Intel (lowest)</t>
-        </is>
-      </c>
-      <c r="E12" s="26" t="inlineStr">
-        <is>
-          <t>1.33</t>
-        </is>
+      <c r="B12" s="13">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MAX('3 Metrics'!$G$3:$G$12),'3 Metrics'!$G$3:$G$12,0))</f>
+        <v/>
+      </c>
+      <c r="C12" s="5">
+        <f>TEXT(MAX('3 Metrics'!$G$3:$G$12),"0.00")&amp;""</f>
+        <v/>
+      </c>
+      <c r="D12" s="12">
+        <f>INDEX('3 Metrics'!$A$3:$A$12,MATCH(MIN('3 Metrics'!$G$3:$G$12),'3 Metrics'!$G$3:$G$12,0))</f>
+        <v/>
+      </c>
+      <c r="E12" s="26">
+        <f>TEXT(MIN('3 Metrics'!$G$3:$G$12),"0.00")&amp;""</f>
+        <v/>
       </c>
       <c r="F12" s="26" t="inlineStr">
         <is>
@@ -9387,25 +9651,21 @@
           <t>Overall Best Practice (V-A &amp; V-B)</t>
         </is>
       </c>
-      <c r="B13" s="13" t="inlineStr">
-        <is>
-          <t>NVIDIA</t>
-        </is>
-      </c>
-      <c r="C13" s="4" t="inlineStr">
-        <is>
-          <t>Rank #1 both versions</t>
-        </is>
-      </c>
-      <c r="D13" s="12" t="inlineStr">
-        <is>
-          <t>Infineon</t>
-        </is>
-      </c>
-      <c r="E13" s="25" t="inlineStr">
-        <is>
-          <t>Rank #10 both versions</t>
-        </is>
+      <c r="B13" s="13">
+        <f>INDEX('5 Scoring Model'!$A$4:$A$13,MATCH(1,'5 Scoring Model'!$H$4:$H$13,0))</f>
+        <v/>
+      </c>
+      <c r="C13" s="4">
+        <f>"Rank #1 V-A &amp; Rank #"&amp;INDEX('5 Scoring Model'!$J$4:$J$13,MATCH(1,'5 Scoring Model'!$H$4:$H$13,0))&amp;" V-B"</f>
+        <v/>
+      </c>
+      <c r="D13" s="12">
+        <f>INDEX('5 Scoring Model'!$A$4:$A$13,MATCH(MAX('5 Scoring Model'!$H$4:$H$13),'5 Scoring Model'!$H$4:$H$13,0))</f>
+        <v/>
+      </c>
+      <c r="E13" s="25">
+        <f>"Rank #"&amp;MAX('5 Scoring Model'!$H$4:$H$13)&amp;" both versions"</f>
+        <v/>
       </c>
       <c r="F13" s="25" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: add 67 verified clickable URLs across 7 sections in Sheet 12; fix Intel IR URL; hyperlink all Sheet 10 filing references
Agent-Logs-Url: https://github.com/pramod51/medplus/sessions/9761af31-7d0a-4acd-88aa-9c2c4ec017bf

Co-authored-by: ydvashwani <47135442+ydvashwani@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/semiconductor_benchmarking.xlsx
+++ b/semiconductor_benchmarking.xlsx
@@ -28,7 +28,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="18">
+  <fonts count="20">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -123,8 +123,15 @@
       <sz val="10"/>
       <u val="single"/>
     </font>
+    <font>
+      <color rgb="000563C1"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
-  <fills count="19">
+  <fills count="20">
     <fill>
       <patternFill/>
     </fill>
@@ -216,6 +223,11 @@
         <fgColor rgb="00404040"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="7">
     <border>
@@ -293,7 +305,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="46">
+  <cellXfs count="55">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -426,6 +438,27 @@
     <xf numFmtId="0" fontId="15" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="10" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="19" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="19" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -2430,9 +2463,9 @@
         </is>
       </c>
       <c r="E3" s="4" t="inlineStr"/>
-      <c r="F3" s="42" t="inlineStr">
-        <is>
-          <t>SEC EDGAR — NVIDIA 10-K filings</t>
+      <c r="F3" s="46" t="inlineStr">
+        <is>
+          <t>EDGAR 10-K — NVIDIA (CIK 1045810)</t>
         </is>
       </c>
     </row>
@@ -2456,9 +2489,9 @@
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr"/>
-      <c r="F4" s="42" t="inlineStr">
-        <is>
-          <t>SEC EDGAR — AMD 10-K filings</t>
+      <c r="F4" s="46" t="inlineStr">
+        <is>
+          <t>EDGAR 10-K — AMD (CIK 2488)</t>
         </is>
       </c>
     </row>
@@ -2486,9 +2519,9 @@
           <t>COGS includes ~$5.2B impairment</t>
         </is>
       </c>
-      <c r="F5" s="42" t="inlineStr">
-        <is>
-          <t>SEC EDGAR — Intel 10-K filings</t>
+      <c r="F5" s="46" t="inlineStr">
+        <is>
+          <t>EDGAR 10-K — Intel (CIK 50863)</t>
         </is>
       </c>
     </row>
@@ -2512,9 +2545,9 @@
         </is>
       </c>
       <c r="E6" s="5" t="inlineStr"/>
-      <c r="F6" s="42" t="inlineStr">
-        <is>
-          <t>SEC EDGAR — Texas Instruments 10-K filings</t>
+      <c r="F6" s="46" t="inlineStr">
+        <is>
+          <t>EDGAR 10-K — Texas Instruments (CIK 97476)</t>
         </is>
       </c>
     </row>
@@ -2542,9 +2575,9 @@
           <t>FY = Oct–Sep</t>
         </is>
       </c>
-      <c r="F7" s="42" t="inlineStr">
-        <is>
-          <t>SEC EDGAR — Qualcomm 10-K filings</t>
+      <c r="F7" s="46" t="inlineStr">
+        <is>
+          <t>EDGAR 10-K — Qualcomm (CIK 804328)</t>
         </is>
       </c>
     </row>
@@ -2572,9 +2605,9 @@
           <t>US GAAP, USD</t>
         </is>
       </c>
-      <c r="F8" s="42" t="inlineStr">
-        <is>
-          <t>SEC EDGAR — NXP Semiconductors 20-F filings</t>
+      <c r="F8" s="46" t="inlineStr">
+        <is>
+          <t>EDGAR 20-F — NXP Semiconductors (CIK 1413447)</t>
         </is>
       </c>
     </row>
@@ -2602,9 +2635,9 @@
           <t>IFRS, TWD→USD</t>
         </is>
       </c>
-      <c r="F9" s="42" t="inlineStr">
-        <is>
-          <t>SEC EDGAR — TSMC 20-F filings</t>
+      <c r="F9" s="46" t="inlineStr">
+        <is>
+          <t>EDGAR 20-F — TSMC (CIK 1046179)</t>
         </is>
       </c>
     </row>
@@ -2632,9 +2665,9 @@
           <t>FY = Sep–Aug</t>
         </is>
       </c>
-      <c r="F10" s="42" t="inlineStr">
-        <is>
-          <t>SEC EDGAR — Micron Technology 10-K filings</t>
+      <c r="F10" s="46" t="inlineStr">
+        <is>
+          <t>EDGAR 10-K — Micron Technology (CIK 723125)</t>
         </is>
       </c>
     </row>
@@ -2662,9 +2695,9 @@
           <t>IFRS, reported USD</t>
         </is>
       </c>
-      <c r="F11" s="42" t="inlineStr">
-        <is>
-          <t>SEC EDGAR — STMicroelectronics 20-F filings</t>
+      <c r="F11" s="46" t="inlineStr">
+        <is>
+          <t>EDGAR 20-F — STMicroelectronics (CIK 912093)</t>
         </is>
       </c>
     </row>
@@ -2692,9 +2725,9 @@
           <t>FY = Oct–Sep</t>
         </is>
       </c>
-      <c r="F12" s="42" t="inlineStr">
-        <is>
-          <t>Infineon Annual Report 2024 (IR page)</t>
+      <c r="F12" s="46" t="inlineStr">
+        <is>
+          <t>Infineon Annual Report (IR page)</t>
         </is>
       </c>
     </row>
@@ -4419,20 +4452,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E51"/>
+  <dimension ref="A1:E80"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="28" customWidth="1" min="2" max="2"/>
-    <col width="52" customWidth="1" min="3" max="3"/>
-    <col width="90" customWidth="1" min="4" max="4"/>
-    <col width="28" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="38" customWidth="1" min="2" max="2"/>
+    <col width="70" customWidth="1" min="3" max="3"/>
+    <col width="80" customWidth="1" min="4" max="4"/>
+    <col width="35" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
-      <c r="A1" s="43" t="inlineStr">
-        <is>
-          <t>STEP 12 — COMPLETE URL REFERENCE LIST  |  All sources used in this benchmarking report</t>
+      <c r="A1" s="47" t="inlineStr">
+        <is>
+          <t>STEP 12 — COMPLETE URL REFERENCE LIST  |  All sources used in this benchmarking report  |  64 total reference URLs across 7 sections  |  All hyperlinks are clickable (Ctrl+Click in Excel)</t>
         </is>
       </c>
     </row>
@@ -4447,7 +4480,7 @@
           <t>Category</t>
         </is>
       </c>
-      <c r="C2" s="30" t="inlineStr">
+      <c r="C2" s="48" t="inlineStr">
         <is>
           <t>Description</t>
         </is>
@@ -4481,14 +4514,14 @@
           <t>SEC 10-K (NVIDIA)</t>
         </is>
       </c>
-      <c r="C4" s="32" t="inlineStr">
+      <c r="C4" s="49" t="inlineStr">
         <is>
           <t>NVIDIA Corporation — Form 10-K FY2025 (fiscal year ended Jan 26, 2025). Source of Revenue, COGS, AR, Inventory, AP, OCF for NVDA.</t>
         </is>
       </c>
-      <c r="D4" s="44" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001045810&amp;type=10-K&amp;dateb=&amp;owner=include&amp;count=5</t>
+      <c r="D4" s="50" t="inlineStr">
+        <is>
+          <t>EDGAR — NVIDIA 10-K filings (CIK 1045810)</t>
         </is>
       </c>
       <c r="E4" s="32" t="inlineStr">
@@ -4508,14 +4541,14 @@
           <t>SEC 10-K (AMD)</t>
         </is>
       </c>
-      <c r="C5" s="32" t="inlineStr">
+      <c r="C5" s="49" t="inlineStr">
         <is>
           <t>Advanced Micro Devices — Form 10-K FY2024 (fiscal year ended Dec 28, 2024). Source of Revenue, COGS, AR, Inventory, AP, OCF for AMD.</t>
         </is>
       </c>
-      <c r="D5" s="44" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0000002488&amp;type=10-K&amp;dateb=&amp;owner=include&amp;count=5</t>
+      <c r="D5" s="50" t="inlineStr">
+        <is>
+          <t>EDGAR — AMD 10-K filings (CIK 2488)</t>
         </is>
       </c>
       <c r="E5" s="32" t="inlineStr">
@@ -4535,14 +4568,14 @@
           <t>SEC 10-K (Intel)</t>
         </is>
       </c>
-      <c r="C6" s="32" t="inlineStr">
+      <c r="C6" s="49" t="inlineStr">
         <is>
           <t>Intel Corporation — Form 10-K FY2024 (fiscal year ended Dec 28, 2024). Note: COGS includes ~$5.2B asset impairment charge (not adjusted in this report).</t>
         </is>
       </c>
-      <c r="D6" s="44" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0000050863&amp;type=10-K&amp;dateb=&amp;owner=include&amp;count=5</t>
+      <c r="D6" s="50" t="inlineStr">
+        <is>
+          <t>EDGAR — Intel 10-K filings (CIK 50863)</t>
         </is>
       </c>
       <c r="E6" s="32" t="inlineStr">
@@ -4562,14 +4595,14 @@
           <t>SEC 10-K (Texas Instruments)</t>
         </is>
       </c>
-      <c r="C7" s="32" t="inlineStr">
+      <c r="C7" s="49" t="inlineStr">
         <is>
           <t>Texas Instruments Incorporated — Form 10-K FY2024 (fiscal year ended Dec 31, 2024). DIO elevated due to management-guided strategic inventory build (20–25 weeks target).</t>
         </is>
       </c>
-      <c r="D7" s="44" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0000097476&amp;type=10-K&amp;dateb=&amp;owner=include&amp;count=5</t>
+      <c r="D7" s="50" t="inlineStr">
+        <is>
+          <t>EDGAR — Texas Instruments 10-K filings (CIK 97476)</t>
         </is>
       </c>
       <c r="E7" s="32" t="inlineStr">
@@ -4589,14 +4622,14 @@
           <t>SEC 10-K (Qualcomm)</t>
         </is>
       </c>
-      <c r="C8" s="32" t="inlineStr">
+      <c r="C8" s="49" t="inlineStr">
         <is>
           <t>Qualcomm Incorporated — Form 10-K FY2024 (fiscal year ended Sep 29, 2024; FY = Oct–Sep). Best-in-class CCC (22.1d) and DIO (54.3d) in this peer group.</t>
         </is>
       </c>
-      <c r="D8" s="44" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0000804328&amp;type=10-K&amp;dateb=&amp;owner=include&amp;count=5</t>
+      <c r="D8" s="50" t="inlineStr">
+        <is>
+          <t>EDGAR — Qualcomm 10-K filings (CIK 804328)</t>
         </is>
       </c>
       <c r="E8" s="32" t="inlineStr">
@@ -4616,14 +4649,14 @@
           <t>SEC 20-F (NXP Semiconductors)</t>
         </is>
       </c>
-      <c r="C9" s="32" t="inlineStr">
+      <c r="C9" s="49" t="inlineStr">
         <is>
           <t>NXP Semiconductors N.V. — Form 20-F FY2024 (fiscal year ended Dec 31, 2024). Reports under US GAAP in USD. Best IDM in peer group (CCC ≈ 100d).</t>
         </is>
       </c>
-      <c r="D9" s="44" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001413447&amp;type=20-F&amp;dateb=&amp;owner=include&amp;count=5</t>
+      <c r="D9" s="50" t="inlineStr">
+        <is>
+          <t>EDGAR — NXP Semiconductors 20-F filings (CIK 1413447)</t>
         </is>
       </c>
       <c r="E9" s="32" t="inlineStr">
@@ -4643,14 +4676,14 @@
           <t>SEC 20-F (TSMC)</t>
         </is>
       </c>
-      <c r="C10" s="32" t="inlineStr">
+      <c r="C10" s="49" t="inlineStr">
         <is>
           <t>Taiwan Semiconductor Manufacturing Company Ltd — Form 20-F FY2024 (fiscal year ended Dec 31, 2024). Reported in New Taiwan Dollars (TWD); converted to USD at 32.0 TWD/USD (FY2024) and 31.1 TWD/USD (FY2023).</t>
         </is>
       </c>
-      <c r="D10" s="44" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001046179&amp;type=20-F&amp;dateb=&amp;owner=include&amp;count=5</t>
+      <c r="D10" s="50" t="inlineStr">
+        <is>
+          <t>EDGAR — TSMC 20-F filings (CIK 1046179)</t>
         </is>
       </c>
       <c r="E10" s="32" t="inlineStr">
@@ -4670,14 +4703,14 @@
           <t>SEC 10-K (Micron Technology)</t>
         </is>
       </c>
-      <c r="C11" s="32" t="inlineStr">
+      <c r="C11" s="49" t="inlineStr">
         <is>
           <t>Micron Technology Inc — Form 10-K FY2024 (fiscal year ended Aug 29, 2024; FY = Sep–Aug). FY2023 had negative gross profit (memory price collapse); DIO is cyclically distorted.</t>
         </is>
       </c>
-      <c r="D11" s="44" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0000723125&amp;type=10-K&amp;dateb=&amp;owner=include&amp;count=5</t>
+      <c r="D11" s="50" t="inlineStr">
+        <is>
+          <t>EDGAR — Micron Technology 10-K filings (CIK 723125)</t>
         </is>
       </c>
       <c r="E11" s="32" t="inlineStr">
@@ -4697,14 +4730,14 @@
           <t>SEC 20-F (STMicroelectronics)</t>
         </is>
       </c>
-      <c r="C12" s="32" t="inlineStr">
+      <c r="C12" s="49" t="inlineStr">
         <is>
           <t>STMicroelectronics N.V. — Form 20-F FY2024 (fiscal year ended Dec 31, 2024). Reports under IFRS in USD.</t>
         </is>
       </c>
-      <c r="D12" s="44" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0000912093&amp;type=20-F&amp;dateb=&amp;owner=include&amp;count=5</t>
+      <c r="D12" s="50" t="inlineStr">
+        <is>
+          <t>EDGAR — STMicroelectronics 20-F filings (CIK 912093)</t>
         </is>
       </c>
       <c r="E12" s="32" t="inlineStr">
@@ -4724,14 +4757,14 @@
           <t>Annual Report (Infineon)</t>
         </is>
       </c>
-      <c r="C13" s="32" t="inlineStr">
+      <c r="C13" s="49" t="inlineStr">
         <is>
           <t>Infineon Technologies AG — Annual Report FY2024 (fiscal year ended Sep 30, 2024; FY = Oct–Sep). Reports under IFRS in EUR; converted to USD at 1.085 USD/EUR (FY2024) and 1.082 (FY2023).</t>
         </is>
       </c>
-      <c r="D13" s="44" t="inlineStr">
-        <is>
-          <t>https://www.infineon.com/cms/en/about-infineon/investor/reports-and-presentations/annual-report/</t>
+      <c r="D13" s="50" t="inlineStr">
+        <is>
+          <t>Infineon Annual Report 2024 (Investor Relations)</t>
         </is>
       </c>
       <c r="E13" s="32" t="inlineStr">
@@ -4758,14 +4791,14 @@
           <t>SEC EDGAR Full-Text Search</t>
         </is>
       </c>
-      <c r="C15" s="32" t="inlineStr">
+      <c r="C15" s="49" t="inlineStr">
         <is>
           <t>EDGAR EFTS allows searching all filing text. Use to locate specific line-items (e.g., "accounts receivable", "inventories") within any 10-K or 20-F.</t>
         </is>
       </c>
-      <c r="D15" s="44" t="inlineStr">
-        <is>
-          <t>https://efts.sec.gov/LATEST/search-index?q=%22accounts+receivable%22&amp;dateRange=custom&amp;startdt=2024-01-01&amp;enddt=2025-03-31&amp;forms=10-K</t>
+      <c r="D15" s="50" t="inlineStr">
+        <is>
+          <t>EDGAR Full-Text Search (EFTS)</t>
         </is>
       </c>
       <c r="E15" s="32" t="inlineStr">
@@ -4785,14 +4818,14 @@
           <t>SEC EDGAR Company Search</t>
         </is>
       </c>
-      <c r="C16" s="32" t="inlineStr">
+      <c r="C16" s="49" t="inlineStr">
         <is>
           <t>Search any public company by name or CIK number to find all SEC filings.</t>
         </is>
       </c>
-      <c r="D16" s="44" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?company=&amp;CIK=&amp;type=10-K&amp;dateb=&amp;owner=include&amp;count=40&amp;search_text=&amp;action=getcompany</t>
+      <c r="D16" s="50" t="inlineStr">
+        <is>
+          <t>EDGAR Company Search Portal</t>
         </is>
       </c>
       <c r="E16" s="32" t="inlineStr">
@@ -4812,14 +4845,14 @@
           <t>SEC EDGAR Full-Text Filing Search (EFTS)</t>
         </is>
       </c>
-      <c r="C17" s="32" t="inlineStr">
+      <c r="C17" s="49" t="inlineStr">
         <is>
           <t>Primary interface for searching filings by keyword, form type, and date range.</t>
         </is>
       </c>
-      <c r="D17" s="44" t="inlineStr">
-        <is>
-          <t>https://efts.sec.gov/LATEST/search-index?q=&amp;forms=10-K,20-F&amp;dateRange=custom&amp;startdt=2024-07-01&amp;enddt=2025-04-30</t>
+      <c r="D17" s="50" t="inlineStr">
+        <is>
+          <t>EDGAR EFTS — 10-K / 20-F Filing Search (2024–2025)</t>
         </is>
       </c>
       <c r="E17" s="32" t="inlineStr">
@@ -4846,14 +4879,14 @@
           <t>NVIDIA Investor Relations</t>
         </is>
       </c>
-      <c r="C19" s="32" t="inlineStr">
+      <c r="C19" s="49" t="inlineStr">
         <is>
           <t>NVIDIA IR page — access to all annual reports, 10-K filings, earnings releases, and financial data tables.</t>
         </is>
       </c>
-      <c r="D19" s="44" t="inlineStr">
-        <is>
-          <t>https://investor.nvidia.com/financial-information/annual-reports/</t>
+      <c r="D19" s="50" t="inlineStr">
+        <is>
+          <t>NVIDIA Investor Relations — Annual Reports</t>
         </is>
       </c>
       <c r="E19" s="32" t="inlineStr">
@@ -4873,14 +4906,14 @@
           <t>AMD Investor Relations</t>
         </is>
       </c>
-      <c r="C20" s="32" t="inlineStr">
+      <c r="C20" s="49" t="inlineStr">
         <is>
           <t>AMD IR page — annual reports, 10-K, quarterly results.</t>
         </is>
       </c>
-      <c r="D20" s="44" t="inlineStr">
-        <is>
-          <t>https://ir.amd.com/financial-information/annual-reports</t>
+      <c r="D20" s="50" t="inlineStr">
+        <is>
+          <t>AMD Investor Relations — Annual Reports</t>
         </is>
       </c>
       <c r="E20" s="32" t="inlineStr">
@@ -4900,14 +4933,14 @@
           <t>Intel Investor Relations</t>
         </is>
       </c>
-      <c r="C21" s="32" t="inlineStr">
+      <c r="C21" s="49" t="inlineStr">
         <is>
           <t>Intel IR page — annual reports, 10-K, earnings releases.</t>
         </is>
       </c>
-      <c r="D21" s="44" t="inlineStr">
-        <is>
-          <t>https://www.intc.com/financial-information/annual-reports</t>
+      <c r="D21" s="50" t="inlineStr">
+        <is>
+          <t>Intel Investor Relations — Annual Reports</t>
         </is>
       </c>
       <c r="E21" s="32" t="inlineStr">
@@ -4927,14 +4960,14 @@
           <t>Texas Instruments Investor Relations</t>
         </is>
       </c>
-      <c r="C22" s="32" t="inlineStr">
+      <c r="C22" s="49" t="inlineStr">
         <is>
           <t>TXN IR page — annual report, 10-K, earnings releases, capital allocation policy.</t>
         </is>
       </c>
-      <c r="D22" s="44" t="inlineStr">
-        <is>
-          <t>https://ir.ti.com/financial-information/annual-reports</t>
+      <c r="D22" s="50" t="inlineStr">
+        <is>
+          <t>Texas Instruments Investor Relations — Annual Reports</t>
         </is>
       </c>
       <c r="E22" s="32" t="inlineStr">
@@ -4954,14 +4987,14 @@
           <t>Qualcomm Investor Relations</t>
         </is>
       </c>
-      <c r="C23" s="32" t="inlineStr">
+      <c r="C23" s="49" t="inlineStr">
         <is>
           <t>QCOM IR page — annual report, 10-K, quarterly earnings, supply-chain disclosures.</t>
         </is>
       </c>
-      <c r="D23" s="44" t="inlineStr">
-        <is>
-          <t>https://investor.qualcomm.com/financial-information/annual-reports</t>
+      <c r="D23" s="50" t="inlineStr">
+        <is>
+          <t>Qualcomm Investor Relations — Annual Reports</t>
         </is>
       </c>
       <c r="E23" s="32" t="inlineStr">
@@ -4981,14 +5014,14 @@
           <t>NXP Semiconductors Investor Relations</t>
         </is>
       </c>
-      <c r="C24" s="32" t="inlineStr">
+      <c r="C24" s="49" t="inlineStr">
         <is>
           <t>NXPI IR page — annual report, 20-F, earnings releases.</t>
         </is>
       </c>
-      <c r="D24" s="44" t="inlineStr">
-        <is>
-          <t>https://investors.nxp.com/financial-information/annual-reports</t>
+      <c r="D24" s="50" t="inlineStr">
+        <is>
+          <t>NXP Semiconductors Investor Relations — Annual Reports</t>
         </is>
       </c>
       <c r="E24" s="32" t="inlineStr">
@@ -5008,14 +5041,14 @@
           <t>TSMC Investor Relations</t>
         </is>
       </c>
-      <c r="C25" s="32" t="inlineStr">
+      <c r="C25" s="49" t="inlineStr">
         <is>
           <t>TSM IR page — annual report, 20-F, earnings, capacity disclosures.</t>
         </is>
       </c>
-      <c r="D25" s="44" t="inlineStr">
-        <is>
-          <t>https://investor.tsmc.com/english/annual-reports</t>
+      <c r="D25" s="50" t="inlineStr">
+        <is>
+          <t>TSMC Investor Relations — Annual Reports</t>
         </is>
       </c>
       <c r="E25" s="32" t="inlineStr">
@@ -5035,14 +5068,14 @@
           <t>Micron Technology Investor Relations</t>
         </is>
       </c>
-      <c r="C26" s="32" t="inlineStr">
+      <c r="C26" s="49" t="inlineStr">
         <is>
           <t>MU IR page — annual report, 10-K, earnings releases.</t>
         </is>
       </c>
-      <c r="D26" s="44" t="inlineStr">
-        <is>
-          <t>https://investors.micron.com/financial-information/annual-reports</t>
+      <c r="D26" s="50" t="inlineStr">
+        <is>
+          <t>Micron Technology Investor Relations — Annual Reports</t>
         </is>
       </c>
       <c r="E26" s="32" t="inlineStr">
@@ -5062,14 +5095,14 @@
           <t>STMicroelectronics Investor Relations</t>
         </is>
       </c>
-      <c r="C27" s="32" t="inlineStr">
+      <c r="C27" s="49" t="inlineStr">
         <is>
           <t>STM IR page — annual report, 20-F, earnings releases.</t>
         </is>
       </c>
-      <c r="D27" s="44" t="inlineStr">
-        <is>
-          <t>https://investors.st.com/financial-results-and-reports/annual-reports</t>
+      <c r="D27" s="50" t="inlineStr">
+        <is>
+          <t>STMicroelectronics Investor Relations — Annual Reports</t>
         </is>
       </c>
       <c r="E27" s="32" t="inlineStr">
@@ -5089,14 +5122,14 @@
           <t>Infineon Technologies Investor Relations</t>
         </is>
       </c>
-      <c r="C28" s="32" t="inlineStr">
+      <c r="C28" s="49" t="inlineStr">
         <is>
           <t>IFX IR page — annual report, earnings releases, sustainability report.</t>
         </is>
       </c>
-      <c r="D28" s="44" t="inlineStr">
-        <is>
-          <t>https://www.infineon.com/cms/en/about-infineon/investor/reports-and-presentations/annual-report/</t>
+      <c r="D28" s="50" t="inlineStr">
+        <is>
+          <t>Infineon Technologies Investor Relations — Annual Report</t>
         </is>
       </c>
       <c r="E28" s="32" t="inlineStr">
@@ -5123,14 +5156,14 @@
           <t>Federal Reserve H.10 Release — Foreign Exchange Rates</t>
         </is>
       </c>
-      <c r="C30" s="32" t="inlineStr">
+      <c r="C30" s="49" t="inlineStr">
         <is>
           <t>US Federal Reserve official annual average exchange rate data. Used for TWD/USD annual average verification (FY2024: 32.0, FY2023: 31.1 TWD/USD).</t>
         </is>
       </c>
-      <c r="D30" s="44" t="inlineStr">
-        <is>
-          <t>https://www.federalreserve.gov/releases/h10/summary/</t>
+      <c r="D30" s="50" t="inlineStr">
+        <is>
+          <t>Federal Reserve H.10 Release — Summary of Daily Exchange Rates</t>
         </is>
       </c>
       <c r="E30" s="32" t="inlineStr">
@@ -5150,14 +5183,14 @@
           <t>Federal Reserve H.10 — Historical Data (Annual)</t>
         </is>
       </c>
-      <c r="C31" s="32" t="inlineStr">
+      <c r="C31" s="49" t="inlineStr">
         <is>
           <t>Historical annual average exchange rates for major currencies against USD, published by the Federal Reserve Board.</t>
         </is>
       </c>
-      <c r="D31" s="44" t="inlineStr">
-        <is>
-          <t>https://www.federalreserve.gov/releases/h10/Hist/</t>
+      <c r="D31" s="50" t="inlineStr">
+        <is>
+          <t>Federal Reserve H.10 — Historical Annual Average Rates</t>
         </is>
       </c>
       <c r="E31" s="32" t="inlineStr">
@@ -5177,14 +5210,14 @@
           <t>European Central Bank — EUR/USD Reference Rates</t>
         </is>
       </c>
-      <c r="C32" s="32" t="inlineStr">
+      <c r="C32" s="49" t="inlineStr">
         <is>
           <t>ECB official EUR/USD reference rates. Used for Infineon EUR→USD conversion (FY2024: 1.085 USD/EUR; FY2023: 1.082 USD/EUR average).</t>
         </is>
       </c>
-      <c r="D32" s="44" t="inlineStr">
-        <is>
-          <t>https://data.ecb.europa.eu/data/datasets/EXR/EXR.D.USD.EUR.SP00.A</t>
+      <c r="D32" s="50" t="inlineStr">
+        <is>
+          <t>European Central Bank — EUR/USD Daily Reference Rates</t>
         </is>
       </c>
       <c r="E32" s="32" t="inlineStr">
@@ -5204,14 +5237,14 @@
           <t>TSMC Annual Report — Stated FX Rate</t>
         </is>
       </c>
-      <c r="C33" s="32" t="inlineStr">
+      <c r="C33" s="49" t="inlineStr">
         <is>
           <t>TSMC Form 20-F contains the company's own stated average TWD/USD translation rate (the authoritative source; verify against this for the [A] approximation used here).</t>
         </is>
       </c>
-      <c r="D33" s="44" t="inlineStr">
-        <is>
-          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0001046179&amp;type=20-F&amp;dateb=&amp;owner=include&amp;count=5</t>
+      <c r="D33" s="50" t="inlineStr">
+        <is>
+          <t>EDGAR — TSMC 20-F (stated FX rate in notes to financial statements)</t>
         </is>
       </c>
       <c r="E33" s="32" t="inlineStr">
@@ -5231,14 +5264,14 @@
           <t>Infineon Annual Report — Stated FX Rate</t>
         </is>
       </c>
-      <c r="C34" s="32" t="inlineStr">
+      <c r="C34" s="49" t="inlineStr">
         <is>
           <t>Infineon Annual Report 2024 contains the company's own stated average EUR/USD rate (verify [A] approximation against this).</t>
         </is>
       </c>
-      <c r="D34" s="44" t="inlineStr">
-        <is>
-          <t>https://www.infineon.com/cms/en/about-infineon/investor/reports-and-presentations/annual-report/</t>
+      <c r="D34" s="50" t="inlineStr">
+        <is>
+          <t>Infineon Annual Report 2024 (stated EUR/USD rate in financial statements)</t>
         </is>
       </c>
       <c r="E34" s="32" t="inlineStr">
@@ -5265,14 +5298,14 @@
           <t>CFA Institute — Working Capital Management</t>
         </is>
       </c>
-      <c r="C36" s="32" t="inlineStr">
+      <c r="C36" s="49" t="inlineStr">
         <is>
           <t>CFA Level 1 &amp; 2 curriculum defines DSO, DIO, DPO, CCC, and NWC ratios as used in this report. Formulas: DSO = Avg AR / (Revenue/365); DIO = Avg Inv / (COGS/365); DPO = Avg AP / (COGS/365); CCC = DSO + DIO − DPO.</t>
         </is>
       </c>
-      <c r="D36" s="44" t="inlineStr">
-        <is>
-          <t>https://www.cfainstitute.org/en/membership/professional-development/refresher-readings/working-capital-management</t>
+      <c r="D36" s="50" t="inlineStr">
+        <is>
+          <t>CFA Institute — Working Capital Management (Refresher Reading)</t>
         </is>
       </c>
       <c r="E36" s="32" t="inlineStr">
@@ -5292,14 +5325,14 @@
           <t>Investopedia — Cash Conversion Cycle</t>
         </is>
       </c>
-      <c r="C37" s="32" t="inlineStr">
+      <c r="C37" s="49" t="inlineStr">
         <is>
           <t>Clear definition and worked examples for CCC = DSO + DIO − DPO. Also covers interpretation: negative CCC examples (Amazon, Dell).</t>
         </is>
       </c>
-      <c r="D37" s="44" t="inlineStr">
-        <is>
-          <t>https://www.investopedia.com/terms/c/cashconversioncycle.asp</t>
+      <c r="D37" s="50" t="inlineStr">
+        <is>
+          <t>Investopedia — Cash Conversion Cycle (CCC)</t>
         </is>
       </c>
       <c r="E37" s="32" t="inlineStr">
@@ -5319,14 +5352,14 @@
           <t>Investopedia — Days Sales Outstanding (DSO)</t>
         </is>
       </c>
-      <c r="C38" s="32" t="inlineStr">
+      <c r="C38" s="49" t="inlineStr">
         <is>
           <t>DSO formula: DSO = (Accounts Receivable / Revenue) × Number of Days. Discussion of two-period average vs. single-period method.</t>
         </is>
       </c>
-      <c r="D38" s="44" t="inlineStr">
-        <is>
-          <t>https://www.investopedia.com/terms/d/dso.asp</t>
+      <c r="D38" s="50" t="inlineStr">
+        <is>
+          <t>Investopedia — Days Sales Outstanding (DSO)</t>
         </is>
       </c>
       <c r="E38" s="32" t="inlineStr">
@@ -5346,14 +5379,14 @@
           <t>Investopedia — Days Inventory Outstanding (DIO)</t>
         </is>
       </c>
-      <c r="C39" s="32" t="inlineStr">
+      <c r="C39" s="49" t="inlineStr">
         <is>
           <t>DIO = (Average Inventory / COGS) × 365. Discussion of impact of seasonality and strategic builds.</t>
         </is>
       </c>
-      <c r="D39" s="44" t="inlineStr">
-        <is>
-          <t>https://www.investopedia.com/terms/d/days-sales-inventory-dsi.asp</t>
+      <c r="D39" s="50" t="inlineStr">
+        <is>
+          <t>Investopedia — Days Inventory Outstanding / Days Sales of Inventory (DIO/DSI)</t>
         </is>
       </c>
       <c r="E39" s="32" t="inlineStr">
@@ -5373,14 +5406,14 @@
           <t>Investopedia — Days Payable Outstanding (DPO)</t>
         </is>
       </c>
-      <c r="C40" s="32" t="inlineStr">
+      <c r="C40" s="49" t="inlineStr">
         <is>
           <t>DPO = (Accounts Payable / COGS) × 365. Higher DPO = longer supplier payment terms = more free cash.</t>
         </is>
       </c>
-      <c r="D40" s="44" t="inlineStr">
-        <is>
-          <t>https://www.investopedia.com/terms/d/days-payable-outstanding.asp</t>
+      <c r="D40" s="50" t="inlineStr">
+        <is>
+          <t>Investopedia — Days Payable Outstanding (DPO)</t>
         </is>
       </c>
       <c r="E40" s="32" t="inlineStr">
@@ -5400,14 +5433,14 @@
           <t>Investopedia — Net Working Capital (NWC)</t>
         </is>
       </c>
-      <c r="C41" s="32" t="inlineStr">
+      <c r="C41" s="49" t="inlineStr">
         <is>
           <t>NWC = Current Assets − Current Liabilities. Operating NWC = AR + Inventory − AP. NWC% = Operating NWC / Revenue × 100.</t>
         </is>
       </c>
-      <c r="D41" s="44" t="inlineStr">
-        <is>
-          <t>https://www.investopedia.com/terms/n/workingcapital.asp</t>
+      <c r="D41" s="50" t="inlineStr">
+        <is>
+          <t>Investopedia — Net Working Capital (NWC)</t>
         </is>
       </c>
       <c r="E41" s="32" t="inlineStr">
@@ -5427,14 +5460,14 @@
           <t>Investopedia — Current Ratio</t>
         </is>
       </c>
-      <c r="C42" s="32" t="inlineStr">
+      <c r="C42" s="49" t="inlineStr">
         <is>
           <t>Current Ratio = Current Assets / Current Liabilities. Measures ability to pay short-term obligations.</t>
         </is>
       </c>
-      <c r="D42" s="44" t="inlineStr">
-        <is>
-          <t>https://www.investopedia.com/terms/c/currentratio.asp</t>
+      <c r="D42" s="50" t="inlineStr">
+        <is>
+          <t>Investopedia — Current Ratio</t>
         </is>
       </c>
       <c r="E42" s="32" t="inlineStr">
@@ -5454,14 +5487,14 @@
           <t>Investopedia — Operating Cash Flow Ratio</t>
         </is>
       </c>
-      <c r="C43" s="32" t="inlineStr">
+      <c r="C43" s="49" t="inlineStr">
         <is>
           <t>CRR (Cash Return Ratio) = OCF / Revenue × 100. Also known as operating cash flow margin.</t>
         </is>
       </c>
-      <c r="D43" s="44" t="inlineStr">
-        <is>
-          <t>https://www.investopedia.com/terms/o/operating-cash-flow-margin.asp</t>
+      <c r="D43" s="50" t="inlineStr">
+        <is>
+          <t>Investopedia — Operating Cash Flow Margin (CRR)</t>
         </is>
       </c>
       <c r="E43" s="32" t="inlineStr">
@@ -5481,14 +5514,14 @@
           <t>FASB ASC 210 — Balance Sheet (US GAAP)</t>
         </is>
       </c>
-      <c r="C44" s="32" t="inlineStr">
+      <c r="C44" s="49" t="inlineStr">
         <is>
           <t>U.S. GAAP guidance on classification of current assets and liabilities. Governs presentation of AR, Inventory, AP for 10-K companies.</t>
         </is>
       </c>
-      <c r="D44" s="44" t="inlineStr">
-        <is>
-          <t>https://asc.fasb.org/210</t>
+      <c r="D44" s="50" t="inlineStr">
+        <is>
+          <t>FASB Accounting Standards Codification — ASC 210 (Balance Sheet)</t>
         </is>
       </c>
       <c r="E44" s="32" t="inlineStr">
@@ -5508,14 +5541,14 @@
           <t>IFRS IAS 1 — Presentation of Financial Statements</t>
         </is>
       </c>
-      <c r="C45" s="32" t="inlineStr">
+      <c r="C45" s="49" t="inlineStr">
         <is>
           <t>IFRS standard governing balance sheet classification (current / non-current). Applies to TSMC, NXP, STM, Infineon (IFRS reporters in this peer group).</t>
         </is>
       </c>
-      <c r="D45" s="44" t="inlineStr">
-        <is>
-          <t>https://www.ifrs.org/issued-standards/list-of-standards/ias-1-presentation-of-financial-statements/</t>
+      <c r="D45" s="50" t="inlineStr">
+        <is>
+          <t>IFRS Foundation — IAS 1 Presentation of Financial Statements</t>
         </is>
       </c>
       <c r="E45" s="32" t="inlineStr">
@@ -5535,14 +5568,14 @@
           <t>IFRS IAS 2 — Inventories</t>
         </is>
       </c>
-      <c r="C46" s="32" t="inlineStr">
+      <c r="C46" s="49" t="inlineStr">
         <is>
           <t>IFRS standard for inventory measurement and disclosure. Defines cost formulas (FIFO, weighted average) used by IFRS reporters in this group.</t>
         </is>
       </c>
-      <c r="D46" s="44" t="inlineStr">
-        <is>
-          <t>https://www.ifrs.org/issued-standards/list-of-standards/ias-2-inventories/</t>
+      <c r="D46" s="50" t="inlineStr">
+        <is>
+          <t>IFRS Foundation — IAS 2 Inventories</t>
         </is>
       </c>
       <c r="E46" s="32" t="inlineStr">
@@ -5562,14 +5595,14 @@
           <t>Semiconductor Industry Association (SIA) — Annual State of the Industry</t>
         </is>
       </c>
-      <c r="C47" s="32" t="inlineStr">
+      <c r="C47" s="49" t="inlineStr">
         <is>
           <t>Industry context: global semiconductor market data, fab capacity trends, and demand cycles referenced in the business model commentary (Sheet 8).</t>
         </is>
       </c>
-      <c r="D47" s="44" t="inlineStr">
-        <is>
-          <t>https://www.semiconductors.org/industry-statistics/</t>
+      <c r="D47" s="50" t="inlineStr">
+        <is>
+          <t>Semiconductor Industry Association (SIA) — Industry Statistics</t>
         </is>
       </c>
       <c r="E47" s="32" t="inlineStr">
@@ -5589,14 +5622,14 @@
           <t>McKinsey — Working Capital Management in Semiconductors</t>
         </is>
       </c>
-      <c r="C48" s="32" t="inlineStr">
+      <c r="C48" s="49" t="inlineStr">
         <is>
           <t>Industry practice benchmarks for NWC optimisation in the semiconductor sector. Basis for recommended strategies in Sheet 7 (NWC Strategy).</t>
         </is>
       </c>
-      <c r="D48" s="44" t="inlineStr">
-        <is>
-          <t>https://www.mckinsey.com/capabilities/operations/our-insights/the-power-of-working-capital</t>
+      <c r="D48" s="50" t="inlineStr">
+        <is>
+          <t>McKinsey &amp; Company — The Power of Working Capital</t>
         </is>
       </c>
       <c r="E48" s="32" t="inlineStr">
@@ -5616,14 +5649,14 @@
           <t>Taulia — Supply Chain Finance / Reverse Factoring</t>
         </is>
       </c>
-      <c r="C49" s="32" t="inlineStr">
+      <c r="C49" s="49" t="inlineStr">
         <is>
           <t>Background on reverse factoring (supplier finance) programmes referenced in NWC strategy recommendations for extending DPO (Sheet 7).</t>
         </is>
       </c>
-      <c r="D49" s="44" t="inlineStr">
-        <is>
-          <t>https://taulia.com/solutions/supply-chain-finance/</t>
+      <c r="D49" s="50" t="inlineStr">
+        <is>
+          <t>Taulia — Supply Chain Finance / Reverse Factoring</t>
         </is>
       </c>
       <c r="E49" s="32" t="inlineStr">
@@ -5632,10 +5665,710 @@
         </is>
       </c>
     </row>
+    <row r="50"/>
     <row r="51" ht="42" customHeight="1">
       <c r="A51" s="45" t="inlineStr">
         <is>
           <t>NOTE: All SEC EDGAR URLs link to the company's filing index page where the specific 10-K or 20-F can be located. For direct document links, navigate to the filing index and select the primary document (usually the .htm or .pdf file). FX rate approximations marked [A] should be verified against the company's own stated rates in their annual report notes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="52"/>
+    <row r="53">
+      <c r="A53" s="51" t="inlineStr">
+        <is>
+          <t>F — DIRECT EDGAR EFTS PER-COMPANY FILING SEARCH  (Full-text search for each company's latest 10-K / 20-F)</t>
+        </is>
+      </c>
+      <c r="B53" s="52" t="n"/>
+      <c r="C53" s="52" t="n"/>
+      <c r="D53" s="52" t="n"/>
+      <c r="E53" s="52" t="n"/>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>F1</t>
+        </is>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>EDGAR EFTS — NVIDIA 10-K</t>
+        </is>
+      </c>
+      <c r="C54" s="53" t="inlineStr">
+        <is>
+          <t>Full-text EDGAR search for NVIDIA Corporation 10-K filings. Returns most recent annual report.</t>
+        </is>
+      </c>
+      <c r="D54" s="54" t="inlineStr">
+        <is>
+          <t>https://efts.sec.gov/LATEST/search-index?q=%22NVIDIA+Corporation%22&amp;entity=NVIDIA&amp;forms=10-K&amp;dateRange=custom&amp;startdt=2025-01-01&amp;enddt=2025-06-30</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>FY2025 10-K filed ~Feb 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>F2</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>EDGAR EFTS — AMD 10-K</t>
+        </is>
+      </c>
+      <c r="C55" s="53" t="inlineStr">
+        <is>
+          <t>Full-text EDGAR search for Advanced Micro Devices 10-K filings.</t>
+        </is>
+      </c>
+      <c r="D55" s="54" t="inlineStr">
+        <is>
+          <t>https://efts.sec.gov/LATEST/search-index?q=%22Advanced+Micro+Devices%22&amp;entity=AMD&amp;forms=10-K&amp;dateRange=custom&amp;startdt=2025-01-01&amp;enddt=2025-06-30</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>FY2024 10-K filed ~Feb 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>F3</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>EDGAR EFTS — Intel 10-K</t>
+        </is>
+      </c>
+      <c r="C56" s="53" t="inlineStr">
+        <is>
+          <t>Full-text EDGAR search for Intel Corporation 10-K filings.</t>
+        </is>
+      </c>
+      <c r="D56" s="54" t="inlineStr">
+        <is>
+          <t>https://efts.sec.gov/LATEST/search-index?q=%22Intel+Corporation%22&amp;entity=Intel&amp;forms=10-K&amp;dateRange=custom&amp;startdt=2025-01-01&amp;enddt=2025-06-30</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>FY2024 10-K filed ~Jan 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>F4</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>EDGAR EFTS — TXN 10-K</t>
+        </is>
+      </c>
+      <c r="C57" s="53" t="inlineStr">
+        <is>
+          <t>Full-text EDGAR search for Texas Instruments 10-K filings.</t>
+        </is>
+      </c>
+      <c r="D57" s="54" t="inlineStr">
+        <is>
+          <t>https://efts.sec.gov/LATEST/search-index?q=%22Texas+Instruments%22&amp;entity=Texas+Instruments&amp;forms=10-K&amp;dateRange=custom&amp;startdt=2025-01-01&amp;enddt=2025-06-30</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>FY2024 10-K filed ~Feb 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>F5</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>EDGAR EFTS — Qualcomm 10-K</t>
+        </is>
+      </c>
+      <c r="C58" s="53" t="inlineStr">
+        <is>
+          <t>Full-text EDGAR search for Qualcomm 10-K filings.</t>
+        </is>
+      </c>
+      <c r="D58" s="54" t="inlineStr">
+        <is>
+          <t>https://efts.sec.gov/LATEST/search-index?q=%22Qualcomm+Incorporated%22&amp;entity=Qualcomm&amp;forms=10-K&amp;dateRange=custom&amp;startdt=2024-10-01&amp;enddt=2025-03-31</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>FY2024 10-K (Oct–Sep FY) filed ~Nov 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>F6</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>EDGAR EFTS — NXP 20-F</t>
+        </is>
+      </c>
+      <c r="C59" s="53" t="inlineStr">
+        <is>
+          <t>Full-text EDGAR search for NXP Semiconductors 20-F filings.</t>
+        </is>
+      </c>
+      <c r="D59" s="54" t="inlineStr">
+        <is>
+          <t>https://efts.sec.gov/LATEST/search-index?q=%22NXP+Semiconductors%22&amp;entity=NXP&amp;forms=20-F&amp;dateRange=custom&amp;startdt=2025-01-01&amp;enddt=2025-06-30</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>FY2024 20-F filed ~Mar 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>F7</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>EDGAR EFTS — TSMC 20-F</t>
+        </is>
+      </c>
+      <c r="C60" s="53" t="inlineStr">
+        <is>
+          <t>Full-text EDGAR search for Taiwan Semiconductor Manufacturing 20-F filings.</t>
+        </is>
+      </c>
+      <c r="D60" s="54" t="inlineStr">
+        <is>
+          <t>https://efts.sec.gov/LATEST/search-index?q=%22Taiwan+Semiconductor%22&amp;entity=TSMC&amp;forms=20-F&amp;dateRange=custom&amp;startdt=2025-01-01&amp;enddt=2025-06-30</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>FY2024 20-F filed ~Apr 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>F8</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>EDGAR EFTS — Micron 10-K</t>
+        </is>
+      </c>
+      <c r="C61" s="53" t="inlineStr">
+        <is>
+          <t>Full-text EDGAR search for Micron Technology 10-K filings.</t>
+        </is>
+      </c>
+      <c r="D61" s="54" t="inlineStr">
+        <is>
+          <t>https://efts.sec.gov/LATEST/search-index?q=%22Micron+Technology%22&amp;entity=Micron&amp;forms=10-K&amp;dateRange=custom&amp;startdt=2024-09-01&amp;enddt=2025-02-28</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>FY2024 10-K (Sep–Aug FY) filed ~Oct 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>F9</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>EDGAR EFTS — STM 20-F</t>
+        </is>
+      </c>
+      <c r="C62" s="53" t="inlineStr">
+        <is>
+          <t>Full-text EDGAR search for STMicroelectronics 20-F filings.</t>
+        </is>
+      </c>
+      <c r="D62" s="54" t="inlineStr">
+        <is>
+          <t>https://efts.sec.gov/LATEST/search-index?q=%22STMicroelectronics%22&amp;entity=STMicroelectronics&amp;forms=20-F&amp;dateRange=custom&amp;startdt=2025-01-01&amp;enddt=2025-06-30</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>FY2024 20-F filed ~Mar 2025</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>F10</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>EDGAR EFTS — Infineon 20-F</t>
+        </is>
+      </c>
+      <c r="C63" s="53" t="inlineStr">
+        <is>
+          <t>Infineon files a 20-F (annual report on Form 20-F) with the SEC. FY = Oct–Sep.</t>
+        </is>
+      </c>
+      <c r="D63" s="54" t="inlineStr">
+        <is>
+          <t>https://efts.sec.gov/LATEST/search-index?q=%22Infineon+Technologies%22&amp;entity=Infineon&amp;forms=20-F&amp;dateRange=custom&amp;startdt=2024-10-01&amp;enddt=2025-04-30</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>FY2024 20-F filed ~Nov 2024</t>
+        </is>
+      </c>
+    </row>
+    <row r="64"/>
+    <row r="65">
+      <c r="A65" s="51" t="inlineStr">
+        <is>
+          <t>G — ADDITIONAL INDUSTRY &amp; CONTEXT REFERENCES  (Semiconductor sector, accounting standards, strategy)</t>
+        </is>
+      </c>
+      <c r="B65" s="52" t="n"/>
+      <c r="C65" s="52" t="n"/>
+      <c r="D65" s="52" t="n"/>
+      <c r="E65" s="52" t="n"/>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>G1</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>SEMI — Industry Statistics &amp; Reports</t>
+        </is>
+      </c>
+      <c r="C66" s="53" t="inlineStr">
+        <is>
+          <t>SEMI is the global industry association for the electronics design and manufacturing supply chain. Industry capacity and fab data referenced in Sheet 8 business model commentary.</t>
+        </is>
+      </c>
+      <c r="D66" s="54" t="inlineStr">
+        <is>
+          <t>https://www.semi.org/en/market-research-statistics</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>Fab capacity &amp; market data</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>G2</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>IC Insights — Semiconductor Market Research</t>
+        </is>
+      </c>
+      <c r="C67" s="53" t="inlineStr">
+        <is>
+          <t>IC Insights provides semiconductor industry market research including capacity, shipments, and company rankings used in context of Sheet 8 business model analysis.</t>
+        </is>
+      </c>
+      <c r="D67" s="54" t="inlineStr">
+        <is>
+          <t>https://www.icinsights.com/</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>Market share &amp; capacity data</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>G3</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Gartner — Top 25 Supply Chains (Semiconductor)</t>
+        </is>
+      </c>
+      <c r="C68" s="53" t="inlineStr">
+        <is>
+          <t>Gartner's annual Top 25 Supply Chains ranking includes semiconductor leaders like TSMC, NVIDIA, and Qualcomm referenced in NWC strategy commentary (Sheet 7).</t>
+        </is>
+      </c>
+      <c r="D68" s="54" t="inlineStr">
+        <is>
+          <t>https://www.gartner.com/en/supply-chain/research/top-25-supply-chains</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>Supply chain benchmarking</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>G4</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>TXN Strategic Inventory Build — Management Commentary (Q3 2023 Earnings)</t>
+        </is>
+      </c>
+      <c r="C69" s="53" t="inlineStr">
+        <is>
+          <t>Texas Instruments management guidance on deliberate inventory build-up (20–25 weeks target) referenced in Sheet 7 NWC strategy and Sheet 8 business model.</t>
+        </is>
+      </c>
+      <c r="D69" s="54" t="inlineStr">
+        <is>
+          <t>https://ir.ti.com/news-releases/news-release-details/texas-instruments-reports-third-quarter-2023-financial-results</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>TXN inventory strategy context</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>G5</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>Intel Q4 2024 Earnings — Impairment Charge Commentary</t>
+        </is>
+      </c>
+      <c r="C70" s="53" t="inlineStr">
+        <is>
+          <t>Intel's Q4/FY2024 earnings release provides context for the ~$5.2B COGS impairment that distorts Intel's gross margin and DIO metrics in this report.</t>
+        </is>
+      </c>
+      <c r="D70" s="54" t="inlineStr">
+        <is>
+          <t>https://www.intc.com/news-releases/news-release-details/intel-reports-fourth-quarter-and-full-year-2024-financial-results</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>Intel COGS impairment context</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>G6</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>Qualcomm FY2024 Annual Report — Supply Chain Commentary</t>
+        </is>
+      </c>
+      <c r="C71" s="53" t="inlineStr">
+        <is>
+          <t>Qualcomm's FY2024 10-K provides detail on fabless model, TSMC supply chain, and extended payment terms driving best-in-class DPO (88.44d) and CCC (22.11d).</t>
+        </is>
+      </c>
+      <c r="D71" s="54" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0000804328&amp;type=10-K&amp;dateb=&amp;owner=include&amp;count=5</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>Qualcomm fabless DPO context</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>G7</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Micron FY2024 Annual Report — Memory Cycle Recovery Commentary</t>
+        </is>
+      </c>
+      <c r="C72" s="53" t="inlineStr">
+        <is>
+          <t>Micron's 10-K provides context for the FY2023 memory trough (negative gross profit) and FY2024 recovery affecting two-period average DIO calculations.</t>
+        </is>
+      </c>
+      <c r="D72" s="54" t="inlineStr">
+        <is>
+          <t>https://www.sec.gov/cgi-bin/browse-edgar?action=getcompany&amp;CIK=0000723125&amp;type=10-K&amp;dateb=&amp;owner=include&amp;count=5</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>Micron memory cycle context</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>G8</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>TSMC Integrated Report 2024 (Chinese/English)</t>
+        </is>
+      </c>
+      <c r="C73" s="53" t="inlineStr">
+        <is>
+          <t>TSMC's Integrated Report (20-F supplement) provides OCF, capex, and operating data in NT$ used to estimate USD OCF for CRR calculation (Sheet 3, col M).</t>
+        </is>
+      </c>
+      <c r="D73" s="54" t="inlineStr">
+        <is>
+          <t>https://investor.tsmc.com/english/annual-reports</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>TSMC OCF estimation source</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>G9</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>Infineon Annual Report 2024 — Auto Semiconductor Market Commentary</t>
+        </is>
+      </c>
+      <c r="C74" s="53" t="inlineStr">
+        <is>
+          <t>Infineon's FY2024 annual report documents the automotive semiconductor demand collapse context driving DIO of 243.74d, the worst in this peer group.</t>
+        </is>
+      </c>
+      <c r="D74" s="54" t="inlineStr">
+        <is>
+          <t>https://www.infineon.com/cms/en/about-infineon/investor/reports-and-presentations/annual-report/</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>Infineon auto crisis context</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>G10</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Investopedia — Accounts Receivable Turnover Ratio</t>
+        </is>
+      </c>
+      <c r="C75" s="53" t="inlineStr">
+        <is>
+          <t>AR Turnover formula: AR Turns = Net Revenue / Average Accounts Receivable. This is the inverse of DSO × 365. Used in Sheet 3 col I and Sheet 4 rankings.</t>
+        </is>
+      </c>
+      <c r="D75" s="54" t="inlineStr">
+        <is>
+          <t>https://www.investopedia.com/terms/a/assetturnover.asp</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>AR Turns definition</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>G11</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>Investopedia — Working Capital Turnover Ratio</t>
+        </is>
+      </c>
+      <c r="C76" s="53" t="inlineStr">
+        <is>
+          <t>WC Intensity = WC / Revenue. Measures how efficiently a company uses its working capital to generate revenue. Used in Sheet 3 col F and scoring model.</t>
+        </is>
+      </c>
+      <c r="D76" s="54" t="inlineStr">
+        <is>
+          <t>https://www.investopedia.com/terms/w/workingcapitalturnover.asp</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>WC Intensity / turnover</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>G12</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>CFA Institute — Financial Statement Analysis (Inventory &amp; Receivables)</t>
+        </is>
+      </c>
+      <c r="C77" s="53" t="inlineStr">
+        <is>
+          <t>CFA curriculum chapter covering ratio analysis of current assets including DIO, DSO, and inventory quality metrics used across Sheets 3–6 of this report.</t>
+        </is>
+      </c>
+      <c r="D77" s="54" t="inlineStr">
+        <is>
+          <t>https://www.cfainstitute.org/en/membership/professional-development/refresher-readings/inventories</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>Inventory ratio methodology</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>G13</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>IFRS Foundation — IFRS 15 Revenue from Contracts with Customers</t>
+        </is>
+      </c>
+      <c r="C78" s="53" t="inlineStr">
+        <is>
+          <t>Governs revenue recognition for TSMC, NXP, STM, and Infineon (IFRS reporters). Relevant for interpreting AR timing and DSO comparability across GAAP/IFRS companies.</t>
+        </is>
+      </c>
+      <c r="D78" s="54" t="inlineStr">
+        <is>
+          <t>https://www.ifrs.org/issued-standards/list-of-standards/ifrs-15-revenue-from-contracts-with-customers/</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>IFRS revenue recognition — DSO comparability</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>G14</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>ASC 606 — Revenue from Contracts with Customers (US GAAP)</t>
+        </is>
+      </c>
+      <c r="C79" s="53" t="inlineStr">
+        <is>
+          <t>US GAAP equivalent of IFRS 15. Governs revenue recognition for NVIDIA, AMD, Intel, TXN, Qualcomm, and Micron. Affects AR timing and DSO calculation.</t>
+        </is>
+      </c>
+      <c r="D79" s="54" t="inlineStr">
+        <is>
+          <t>https://asc.fasb.org/606</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>US GAAP revenue recognition — DSO comparability</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>G15</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>Federal Reserve Statistical Release H.10 — Taiwan Dollar vs USD (Annual avg)</t>
+        </is>
+      </c>
+      <c r="C80" s="53" t="inlineStr">
+        <is>
+          <t>Annual average TWD/USD exchange rate series. Used to verify TSMC FX assumption (32.0 TWD/USD for 2024, 31.1 for 2023) for USD conversion of financial data.</t>
+        </is>
+      </c>
+      <c r="D80" s="54" t="inlineStr">
+        <is>
+          <t>https://www.federalreserve.gov/releases/h10/20250120/</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>TWD/USD annual average Jan 2025 release</t>
         </is>
       </c>
     </row>
@@ -5692,6 +6425,31 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D47" r:id="rId40"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D48" r:id="rId41"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D49" r:id="rId42"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D54" r:id="rId43"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D55" r:id="rId44"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D56" r:id="rId45"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D57" r:id="rId46"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D58" r:id="rId47"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D59" r:id="rId48"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D60" r:id="rId49"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D61" r:id="rId50"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D62" r:id="rId51"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D63" r:id="rId52"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D66" r:id="rId53"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D67" r:id="rId54"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D68" r:id="rId55"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D69" r:id="rId56"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D70" r:id="rId57"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D71" r:id="rId58"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D72" r:id="rId59"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D73" r:id="rId60"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D74" r:id="rId61"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D75" r:id="rId62"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D76" r:id="rId63"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D77" r:id="rId64"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D78" r:id="rId65"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D79" r:id="rId66"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="D80" r:id="rId67"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>